<commit_message>
docs: kompletni rewrite README a BAZAR_WATCHER.md
- README: top-level prehled obou modulu, struktura, workflow s plain SMTP env
- BAZAR_WATCHER.md: architektura+datovy tok, CLI flagy, scrapery, parsery, recepty pro zmeny
- workflow: SMTP credentials primo v env: bloku (privatni repo, no secrets)
- .env.example: aktualizovany pro lokalni use-case
- cleanup: smazan README.OLD.md a run_final.txt
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vsechny inzeraty" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dnes pridane" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martin – M mid-B a níže" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kamarádka – XS-S EN A" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -526,11 +528,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-3-22-85-105kg-no-sivs-no-flying-on-the-sand-n-6761/</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>450</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2013</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>450.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -582,8 +588,10 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2022</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -630,11 +638,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-7-80-105kg-concertinas-new-tc-fresh-tc-valid-6747/</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2025</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2750.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -682,8 +694,10 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2018</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -734,11 +748,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-trees-no-water-wit-6727/</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2022</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1250.0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -789,11 +807,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-no-flying-on-the-sand-no-t-6715/</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2020</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1400.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -845,8 +867,10 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>2018</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -898,8 +922,10 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>2017</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -951,8 +977,10 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>2016</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1004,8 +1032,10 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="n">
-        <v>2020</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1053,8 +1083,10 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>2018</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1106,8 +1138,10 @@
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
-        <v>2014</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1155,8 +1189,10 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>2024</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1207,11 +1243,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G15" t="n">
-        <v>2023</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1259,8 +1299,10 @@
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="n">
-        <v>2021</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1312,8 +1354,10 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
-        <v>2018</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1365,8 +1409,10 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>2009</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1414,8 +1460,10 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="n">
-        <v>2017</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1466,11 +1514,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-eden-3-trend-3-24-70-90kg-concertinas-no-flying-on-t-6580/</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>320</v>
-      </c>
-      <c r="G20" t="n">
-        <v>2010</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>320.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2010.0</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1522,8 +1574,10 @@
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
-        <v>2016</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1575,8 +1629,10 @@
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="n">
-        <v>2023</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1623,11 +1679,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>599</v>
-      </c>
-      <c r="G23" t="n">
-        <v>2015</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1674,11 +1734,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-95-115kg-concertinas-lightened-no-si-6556/</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G24" t="n">
-        <v>2022</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1729,11 +1793,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-100-130kg-no-sivs-no-flying-on-the-sand--6535/</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G25" t="n">
-        <v>2019</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1785,8 +1853,10 @@
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="n">
-        <v>2022</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1838,8 +1908,10 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="n">
-        <v>2024</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1890,11 +1962,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-6521/</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>1150</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2020</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1150.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1946,8 +2022,10 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="n">
-        <v>2025</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1999,8 +2077,10 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="n">
-        <v>2019</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -2051,11 +2131,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kangri-s-65-85kg-concertinas-lightened-no-sivs-no-fly-6508/</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>1425</v>
-      </c>
-      <c r="G31" t="n">
-        <v>2020</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1425.0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -2107,8 +2191,10 @@
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="n">
-        <v>2017</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -2160,8 +2246,10 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>2017</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2209,8 +2297,10 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="n">
-        <v>2025</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2262,8 +2352,10 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="n">
-        <v>2013</v>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2315,8 +2407,10 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="n">
-        <v>2013</v>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2368,8 +2462,10 @@
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="n">
-        <v>2023</v>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2420,11 +2516,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-no-sivs-tc-fresh-tc-valid-with-bag-6411/</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G38" t="n">
-        <v>2023</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2200.0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2475,11 +2575,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-110-130kg-concertinas-no-sivs-no-flying--6408/</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2019</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2531,8 +2635,10 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="n">
-        <v>2017</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2583,11 +2689,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-sky-apollo-3-95-119kg-no-water-concertinas-with-list-6385/</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G41" t="n">
-        <v>2024</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2635,8 +2745,10 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="n">
-        <v>2007</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2007.0</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2687,11 +2799,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95kg-concertinas-no-sivs-no-flying-6749/</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>2300</v>
-      </c>
-      <c r="G43" t="n">
-        <v>2024</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2300.0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2743,8 +2859,10 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="n">
-        <v>2019</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2796,8 +2914,10 @@
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
-      <c r="G45" t="n">
-        <v>2009</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2845,8 +2965,10 @@
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="n">
-        <v>2020</v>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2897,11 +3019,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2020</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2952,11 +3078,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-22-50-85kg-no-sivs-no-flying-on-the-sand-6667/</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G48" t="n">
-        <v>2025</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>1800.0</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3007,11 +3137,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/swing-mito-s-70-95kg-concertinas-no-sivs-no-tc-no-trees--6664/</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G49" t="n">
-        <v>2021</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2200.0</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3063,8 +3197,10 @@
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="n">
-        <v>2015</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3115,11 +3251,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G51" t="n">
-        <v>2026</v>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3170,11 +3310,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-l-95kg-115-concertinas-no-sivs-no-tc-no-f-6610/</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G52" t="n">
-        <v>2022</v>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -3225,11 +3369,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-8-dls-26-70-110kg-concertinas-no-sivs-no-f-6534/</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G53" t="n">
-        <v>2025</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -3280,11 +3428,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G54" t="n">
-        <v>2020</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3336,8 +3488,10 @@
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="n">
-        <v>2021</v>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -3389,8 +3543,10 @@
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
-      <c r="G56" t="n">
-        <v>2016</v>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -3441,11 +3597,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/phi-symphonia-26-26-105-130kg-no-sivs-no-trees-no-water--6492/</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>500</v>
-      </c>
-      <c r="G57" t="n">
-        <v>2018</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -3496,8 +3656,10 @@
           <t>https://paragliding-bazar.cz/cs/offering/apco-gradient-nevada-2-26-80-102kg-concertinas-6467/</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>2000</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
@@ -3550,8 +3712,10 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="n">
-        <v>2023</v>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -3602,11 +3766,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-95-115kg-concertinas-no-sivs-no-flying-on-6445/</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G60" t="n">
-        <v>2020</v>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -3658,8 +3826,10 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="n">
-        <v>2020</v>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -3711,8 +3881,10 @@
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="n">
-        <v>2004</v>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2004.0</t>
+        </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3760,8 +3932,10 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="n">
-        <v>2013</v>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -3812,11 +3986,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-flying-on-the-sand-no-t-6390/</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G64" t="n">
-        <v>2025</v>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -3918,11 +4096,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-28-80-118kg-no-water-with-bag-6354/</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G66" t="n">
-        <v>2021</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -3974,8 +4156,10 @@
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="n">
-        <v>2022</v>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -4027,8 +4211,10 @@
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="n">
-        <v>2019</v>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -4080,8 +4266,10 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="n">
-        <v>2026</v>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
@@ -4121,8 +4309,10 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="n">
-        <v>2024</v>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -4205,8 +4395,10 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="n">
-        <v>2023</v>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -5818,8 +6010,10 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" t="n">
-        <v>2026</v>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
@@ -5871,8 +6065,10 @@
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
-      <c r="G114" t="n">
-        <v>2026</v>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
@@ -5924,8 +6120,10 @@
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
-      <c r="G115" t="n">
-        <v>2026</v>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
@@ -6206,8 +6404,10 @@
           <t>https://www.flugschule-alpstein.ch/occasionen/</t>
         </is>
       </c>
-      <c r="F122" t="n">
-        <v>3333</v>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>3333.0</t>
+        </is>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
@@ -6259,8 +6459,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m377e1eb6cccd2f2c</t>
         </is>
       </c>
-      <c r="F123" t="n">
-        <v>820</v>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>820.0</t>
+        </is>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
@@ -6300,8 +6502,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mcc7c8f0a633a63a2</t>
         </is>
       </c>
-      <c r="F124" t="n">
-        <v>980</v>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
@@ -6345,8 +6549,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mc8d74414d3dc920f</t>
         </is>
       </c>
-      <c r="F125" t="n">
-        <v>980</v>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
@@ -6390,8 +6596,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mf054d2f1cbaf2545</t>
         </is>
       </c>
-      <c r="F126" t="n">
-        <v>1690</v>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>1690.0</t>
+        </is>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -6435,8 +6643,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mc887178d2dcf8019</t>
         </is>
       </c>
-      <c r="F127" t="n">
-        <v>3650</v>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>3650.0</t>
+        </is>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
@@ -6480,8 +6690,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mc101661395c53166</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>560</v>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>560.0</t>
+        </is>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
@@ -6521,8 +6733,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m7e2b567d0e32224a</t>
         </is>
       </c>
-      <c r="F129" t="n">
-        <v>1490</v>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>1490.0</t>
+        </is>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
@@ -6562,8 +6776,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mced2378820175461</t>
         </is>
       </c>
-      <c r="F130" t="n">
-        <v>3490</v>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>3490.0</t>
+        </is>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
@@ -6607,8 +6823,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m1673bde027bc8bdc</t>
         </is>
       </c>
-      <c r="F131" t="n">
-        <v>3450</v>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>3450.0</t>
+        </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
@@ -6652,8 +6870,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m9d1212e26ac4cee3</t>
         </is>
       </c>
-      <c r="F132" t="n">
-        <v>1940</v>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>1940.0</t>
+        </is>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
@@ -6697,8 +6917,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m08e6dcb39b086e55</t>
         </is>
       </c>
-      <c r="F133" t="n">
-        <v>2099</v>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>2099.0</t>
+        </is>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
@@ -6742,8 +6964,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m75b78a590a74ced2</t>
         </is>
       </c>
-      <c r="F134" t="n">
-        <v>1890</v>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>1890.0</t>
+        </is>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
@@ -6783,8 +7007,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m119044a6b1ca9781</t>
         </is>
       </c>
-      <c r="F135" t="n">
-        <v>1250</v>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>1250.0</t>
+        </is>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr"/>
@@ -6824,8 +7050,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m58c75d27403c654c</t>
         </is>
       </c>
-      <c r="F136" t="n">
-        <v>1290</v>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>1290.0</t>
+        </is>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
@@ -6865,8 +7093,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m8025c05329adeb81</t>
         </is>
       </c>
-      <c r="F137" t="n">
-        <v>490</v>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>490.0</t>
+        </is>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
@@ -6911,8 +7141,10 @@
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
-      <c r="G138" t="n">
-        <v>2020</v>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -6960,8 +7192,10 @@
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
-      <c r="G139" t="n">
-        <v>2023</v>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -7009,8 +7243,10 @@
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
-      <c r="G140" t="n">
-        <v>2025</v>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
@@ -7058,8 +7294,10 @@
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
-      <c r="G141" t="n">
-        <v>2025</v>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
@@ -7107,8 +7345,10 @@
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
-      <c r="G142" t="n">
-        <v>2024</v>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
@@ -7156,8 +7396,10 @@
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
-      <c r="G143" t="n">
-        <v>2024</v>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
@@ -7205,8 +7447,10 @@
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
-      <c r="G144" t="n">
-        <v>2024</v>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
@@ -7253,8 +7497,10 @@
           <t>https://paraglidingshop.ch/Mentor-5-light-S-80kg-100kg/SW10333</t>
         </is>
       </c>
-      <c r="F145" t="n">
-        <v>951</v>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>951.0</t>
+        </is>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
@@ -7298,11 +7544,15 @@
           <t>https://paraglidingshop.ch/Skywalk-Tonic-EN-B-56-80kg-EN-C81-105-kg/SW10339</t>
         </is>
       </c>
-      <c r="F146" t="n">
-        <v>951</v>
-      </c>
-      <c r="G146" t="n">
-        <v>2014</v>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>951.0</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -7354,8 +7604,10 @@
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
-      <c r="G147" t="n">
-        <v>2021</v>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
@@ -7504,8 +7756,10 @@
           <t>https://www.flugschule-alpstein.ch/occasionen/</t>
         </is>
       </c>
-      <c r="F150" t="n">
-        <v>2333</v>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>2333.0</t>
+        </is>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
@@ -7553,8 +7807,10 @@
           <t>https://www.flugschule-alpstein.ch/occasionen/</t>
         </is>
       </c>
-      <c r="F151" t="n">
-        <v>3190</v>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>3190.0</t>
+        </is>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr"/>
@@ -7684,11 +7940,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F154" t="n">
-        <v>980</v>
-      </c>
-      <c r="G154" t="n">
-        <v>2016</v>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
@@ -7739,11 +7999,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F155" t="n">
-        <v>980</v>
-      </c>
-      <c r="G155" t="n">
-        <v>2020</v>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
@@ -7794,11 +8058,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F156" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G156" t="n">
-        <v>2020</v>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>1250.0</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
@@ -7849,11 +8117,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F157" t="n">
-        <v>1690</v>
-      </c>
-      <c r="G157" t="n">
-        <v>2021</v>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>1690.0</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
@@ -7900,11 +8172,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F158" t="n">
-        <v>1490</v>
-      </c>
-      <c r="G158" t="n">
-        <v>2024</v>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>1490.0</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr">
@@ -7955,8 +8231,10 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F159" t="n">
-        <v>3450</v>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>3450.0</t>
+        </is>
       </c>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr"/>
@@ -8008,11 +8286,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F160" t="n">
-        <v>3490</v>
-      </c>
-      <c r="G160" t="n">
-        <v>2025</v>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>3490.0</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr">
@@ -8063,11 +8345,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F161" t="n">
-        <v>3650</v>
-      </c>
-      <c r="G161" t="n">
-        <v>2024</v>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>3650.0</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
@@ -8118,11 +8404,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F162" t="n">
-        <v>1940</v>
-      </c>
-      <c r="G162" t="n">
-        <v>2024</v>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>1940.0</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
@@ -8173,8 +8463,10 @@
           <t>https://paraglidingshop.ch/Advance-Iota-DLS-25-Royal-Occasion-EN-B-80-100kg/SW10406</t>
         </is>
       </c>
-      <c r="F163" t="n">
-        <v>2667</v>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>2667.0</t>
+        </is>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
@@ -8226,8 +8518,10 @@
           <t>https://paraglidingshop.ch/Advance-Pi-3-27-weiss-Ex-Demo/SW10521</t>
         </is>
       </c>
-      <c r="F164" t="n">
-        <v>1895</v>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>1895.0</t>
+        </is>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr"/>
@@ -8271,8 +8565,10 @@
           <t>https://paraglidingshop.ch/Ozone-Swift-6-ML-Ex-Demo/SW10522</t>
         </is>
       </c>
-      <c r="F165" t="n">
-        <v>2667</v>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>2667.0</t>
+        </is>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
@@ -8320,8 +8616,10 @@
           <t>https://paraglidingshop.ch/Phi-Maestro-23/SW10330</t>
         </is>
       </c>
-      <c r="F166" t="n">
-        <v>952</v>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>952.0</t>
+        </is>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr"/>
@@ -8461,11 +8759,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-3-22-85-105kg-no-sivs-no-flying-on-the-sand-n-6761/</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>450</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2013</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>450.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -8517,8 +8819,10 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2022</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -8565,11 +8869,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-7-80-105kg-concertinas-new-tc-fresh-tc-valid-6747/</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2025</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2750.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -8617,8 +8925,10 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2018</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -8669,11 +8979,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-trees-no-water-wit-6727/</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2022</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1250.0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -8724,11 +9038,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-no-flying-on-the-sand-no-t-6715/</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2020</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1400.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -8780,8 +9098,10 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>2018</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -8833,8 +9153,10 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>2017</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -8886,8 +9208,10 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>2016</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -8939,8 +9263,10 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="n">
-        <v>2020</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -8988,8 +9314,10 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>2018</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -9041,8 +9369,10 @@
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
-        <v>2014</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -9090,8 +9420,10 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>2024</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -9142,11 +9474,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G15" t="n">
-        <v>2023</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -9194,8 +9530,10 @@
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="n">
-        <v>2021</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -9247,8 +9585,10 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
-        <v>2018</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -9300,8 +9640,10 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>2009</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -9349,8 +9691,10 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="n">
-        <v>2017</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -9401,11 +9745,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-eden-3-trend-3-24-70-90kg-concertinas-no-flying-on-t-6580/</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>320</v>
-      </c>
-      <c r="G20" t="n">
-        <v>2010</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>320.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2010.0</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -9457,8 +9805,10 @@
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
-        <v>2016</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -9510,8 +9860,10 @@
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="n">
-        <v>2023</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -9558,11 +9910,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>599</v>
-      </c>
-      <c r="G23" t="n">
-        <v>2015</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -9609,11 +9965,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-95-115kg-concertinas-lightened-no-si-6556/</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G24" t="n">
-        <v>2022</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -9664,11 +10024,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-100-130kg-no-sivs-no-flying-on-the-sand--6535/</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G25" t="n">
-        <v>2019</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -9720,8 +10084,10 @@
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="n">
-        <v>2022</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -9773,8 +10139,10 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="n">
-        <v>2024</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -9825,11 +10193,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-6521/</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>1150</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2020</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1150.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -9881,8 +10253,10 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="n">
-        <v>2025</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -9934,8 +10308,10 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="n">
-        <v>2019</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -9986,11 +10362,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kangri-s-65-85kg-concertinas-lightened-no-sivs-no-fly-6508/</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>1425</v>
-      </c>
-      <c r="G31" t="n">
-        <v>2020</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1425.0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -10042,8 +10422,10 @@
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="n">
-        <v>2017</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -10095,8 +10477,10 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>2017</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -10144,8 +10528,10 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="n">
-        <v>2025</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -10197,8 +10583,10 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="n">
-        <v>2013</v>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -10250,8 +10638,10 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="n">
-        <v>2013</v>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -10303,8 +10693,10 @@
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="n">
-        <v>2023</v>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -10355,11 +10747,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-no-sivs-tc-fresh-tc-valid-with-bag-6411/</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G38" t="n">
-        <v>2023</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2200.0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -10410,11 +10806,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-110-130kg-concertinas-no-sivs-no-flying--6408/</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2019</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -10466,8 +10866,10 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="n">
-        <v>2017</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -10518,11 +10920,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-sky-apollo-3-95-119kg-no-water-concertinas-with-list-6385/</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G41" t="n">
-        <v>2024</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -10570,8 +10976,10 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="n">
-        <v>2007</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2007.0</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -10622,11 +11030,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95kg-concertinas-no-sivs-no-flying-6749/</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>2300</v>
-      </c>
-      <c r="G43" t="n">
-        <v>2024</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2300.0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -10678,8 +11090,10 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="n">
-        <v>2019</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -10731,8 +11145,10 @@
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
-      <c r="G45" t="n">
-        <v>2009</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -10780,8 +11196,10 @@
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="n">
-        <v>2020</v>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -10832,11 +11250,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2020</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -10887,11 +11309,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-22-50-85kg-no-sivs-no-flying-on-the-sand-6667/</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G48" t="n">
-        <v>2025</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>1800.0</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -10942,11 +11368,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/swing-mito-s-70-95kg-concertinas-no-sivs-no-tc-no-trees--6664/</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G49" t="n">
-        <v>2021</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2200.0</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -10998,8 +11428,10 @@
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="n">
-        <v>2015</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -11050,11 +11482,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G51" t="n">
-        <v>2026</v>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -11105,11 +11541,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-l-95kg-115-concertinas-no-sivs-no-tc-no-f-6610/</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G52" t="n">
-        <v>2022</v>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -11160,11 +11600,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-8-dls-26-70-110kg-concertinas-no-sivs-no-f-6534/</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G53" t="n">
-        <v>2025</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -11215,11 +11659,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G54" t="n">
-        <v>2020</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -11271,8 +11719,10 @@
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="n">
-        <v>2021</v>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -11324,8 +11774,10 @@
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
-      <c r="G56" t="n">
-        <v>2016</v>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -11376,11 +11828,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/phi-symphonia-26-26-105-130kg-no-sivs-no-trees-no-water--6492/</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>500</v>
-      </c>
-      <c r="G57" t="n">
-        <v>2018</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -11431,8 +11887,10 @@
           <t>https://paragliding-bazar.cz/cs/offering/apco-gradient-nevada-2-26-80-102kg-concertinas-6467/</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>2000</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
@@ -11485,8 +11943,10 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="n">
-        <v>2023</v>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -11537,11 +11997,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-95-115kg-concertinas-no-sivs-no-flying-on-6445/</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G60" t="n">
-        <v>2020</v>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -11593,8 +12057,10 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="n">
-        <v>2020</v>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -11646,8 +12112,10 @@
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="n">
-        <v>2004</v>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2004.0</t>
+        </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -11695,8 +12163,10 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="n">
-        <v>2013</v>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -11747,11 +12217,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-flying-on-the-sand-no-t-6390/</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G64" t="n">
-        <v>2025</v>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2000.0</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -11853,11 +12327,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-28-80-118kg-no-water-with-bag-6354/</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G66" t="n">
-        <v>2021</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -11909,8 +12387,10 @@
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="n">
-        <v>2022</v>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -11962,8 +12442,10 @@
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="n">
-        <v>2019</v>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -12015,8 +12497,10 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="n">
-        <v>2026</v>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
@@ -12056,8 +12540,10 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="n">
-        <v>2024</v>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -12140,8 +12626,10 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="n">
-        <v>2023</v>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -13753,8 +14241,10 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" t="n">
-        <v>2026</v>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
@@ -13806,8 +14296,10 @@
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
-      <c r="G114" t="n">
-        <v>2026</v>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
@@ -14092,8 +14584,10 @@
           <t>https://www.flugschule-alpstein.ch/occasionen/</t>
         </is>
       </c>
-      <c r="F121" t="n">
-        <v>3333</v>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>3333.0</t>
+        </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
@@ -14145,8 +14639,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m377e1eb6cccd2f2c</t>
         </is>
       </c>
-      <c r="F122" t="n">
-        <v>820</v>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>820.0</t>
+        </is>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
@@ -14186,8 +14682,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mcc7c8f0a633a63a2</t>
         </is>
       </c>
-      <c r="F123" t="n">
-        <v>980</v>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
@@ -14231,8 +14729,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mc8d74414d3dc920f</t>
         </is>
       </c>
-      <c r="F124" t="n">
-        <v>980</v>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
@@ -14276,8 +14776,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mf054d2f1cbaf2545</t>
         </is>
       </c>
-      <c r="F125" t="n">
-        <v>1690</v>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>1690.0</t>
+        </is>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
@@ -14321,8 +14823,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mc887178d2dcf8019</t>
         </is>
       </c>
-      <c r="F126" t="n">
-        <v>3650</v>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>3650.0</t>
+        </is>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -14366,8 +14870,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mc101661395c53166</t>
         </is>
       </c>
-      <c r="F127" t="n">
-        <v>560</v>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>560.0</t>
+        </is>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
@@ -14407,8 +14913,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m7e2b567d0e32224a</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>1490</v>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>1490.0</t>
+        </is>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
@@ -14448,8 +14956,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/mced2378820175461</t>
         </is>
       </c>
-      <c r="F129" t="n">
-        <v>3490</v>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>3490.0</t>
+        </is>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
@@ -14493,8 +15003,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m1673bde027bc8bdc</t>
         </is>
       </c>
-      <c r="F130" t="n">
-        <v>3450</v>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>3450.0</t>
+        </is>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
@@ -14538,8 +15050,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m9d1212e26ac4cee3</t>
         </is>
       </c>
-      <c r="F131" t="n">
-        <v>1940</v>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>1940.0</t>
+        </is>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
@@ -14583,8 +15097,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m08e6dcb39b086e55</t>
         </is>
       </c>
-      <c r="F132" t="n">
-        <v>2099</v>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2099.0</t>
+        </is>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
@@ -14628,8 +15144,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m75b78a590a74ced2</t>
         </is>
       </c>
-      <c r="F133" t="n">
-        <v>1890</v>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>1890.0</t>
+        </is>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
@@ -14669,8 +15187,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m119044a6b1ca9781</t>
         </is>
       </c>
-      <c r="F134" t="n">
-        <v>1250</v>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>1250.0</t>
+        </is>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
@@ -14710,8 +15230,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m58c75d27403c654c</t>
         </is>
       </c>
-      <c r="F135" t="n">
-        <v>1290</v>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>1290.0</t>
+        </is>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr"/>
@@ -14751,8 +15273,10 @@
           <t>https://www.paragliding-store.at//app/module/webproduct/goto/m/m8025c05329adeb81</t>
         </is>
       </c>
-      <c r="F136" t="n">
-        <v>490</v>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>490.0</t>
+        </is>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
@@ -14797,8 +15321,10 @@
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
-      <c r="G137" t="n">
-        <v>2020</v>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
@@ -14846,8 +15372,10 @@
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
-      <c r="G138" t="n">
-        <v>2023</v>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
@@ -14895,8 +15423,10 @@
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
-      <c r="G139" t="n">
-        <v>2025</v>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
@@ -14944,8 +15474,10 @@
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
-      <c r="G140" t="n">
-        <v>2025</v>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
@@ -14993,8 +15525,10 @@
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
-      <c r="G141" t="n">
-        <v>2024</v>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
@@ -15042,8 +15576,10 @@
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
-      <c r="G142" t="n">
-        <v>2024</v>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
@@ -15091,8 +15627,10 @@
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
-      <c r="G143" t="n">
-        <v>2024</v>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
@@ -15139,8 +15677,10 @@
           <t>https://paraglidingshop.ch/Mentor-5-light-S-80kg-100kg/SW10333</t>
         </is>
       </c>
-      <c r="F144" t="n">
-        <v>951</v>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>951.0</t>
+        </is>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr"/>
@@ -15184,11 +15724,15 @@
           <t>https://paraglidingshop.ch/Skywalk-Tonic-EN-B-56-80kg-EN-C81-105-kg/SW10339</t>
         </is>
       </c>
-      <c r="F145" t="n">
-        <v>951</v>
-      </c>
-      <c r="G145" t="n">
-        <v>2014</v>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>951.0</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
@@ -15240,8 +15784,10 @@
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
-      <c r="G146" t="n">
-        <v>2021</v>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -15390,8 +15936,10 @@
           <t>https://www.flugschule-alpstein.ch/occasionen/</t>
         </is>
       </c>
-      <c r="F149" t="n">
-        <v>2333</v>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>2333.0</t>
+        </is>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
@@ -15439,8 +15987,10 @@
           <t>https://www.flugschule-alpstein.ch/occasionen/</t>
         </is>
       </c>
-      <c r="F150" t="n">
-        <v>3190</v>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>3190.0</t>
+        </is>
       </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
@@ -15570,11 +16120,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F153" t="n">
-        <v>980</v>
-      </c>
-      <c r="G153" t="n">
-        <v>2016</v>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr">
@@ -15625,11 +16179,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F154" t="n">
-        <v>980</v>
-      </c>
-      <c r="G154" t="n">
-        <v>2020</v>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
@@ -15680,11 +16238,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F155" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G155" t="n">
-        <v>2020</v>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>1250.0</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
@@ -15735,11 +16297,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F156" t="n">
-        <v>1690</v>
-      </c>
-      <c r="G156" t="n">
-        <v>2021</v>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>1690.0</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
@@ -15786,11 +16352,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F157" t="n">
-        <v>1490</v>
-      </c>
-      <c r="G157" t="n">
-        <v>2024</v>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>1490.0</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
@@ -15841,8 +16411,10 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F158" t="n">
-        <v>3450</v>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>3450.0</t>
+        </is>
       </c>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr"/>
@@ -15894,11 +16466,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F159" t="n">
-        <v>3490</v>
-      </c>
-      <c r="G159" t="n">
-        <v>2025</v>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>3490.0</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr">
@@ -15949,11 +16525,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F160" t="n">
-        <v>3650</v>
-      </c>
-      <c r="G160" t="n">
-        <v>2024</v>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>3650.0</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr">
@@ -16004,11 +16584,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F161" t="n">
-        <v>1940</v>
-      </c>
-      <c r="G161" t="n">
-        <v>2024</v>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>1940.0</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
@@ -16059,8 +16643,10 @@
           <t>https://paraglidingshop.ch/Advance-Iota-DLS-25-Royal-Occasion-EN-B-80-100kg/SW10406</t>
         </is>
       </c>
-      <c r="F162" t="n">
-        <v>2667</v>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>2667.0</t>
+        </is>
       </c>
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
@@ -16112,8 +16698,10 @@
           <t>https://paraglidingshop.ch/Advance-Pi-3-27-weiss-Ex-Demo/SW10521</t>
         </is>
       </c>
-      <c r="F163" t="n">
-        <v>1895</v>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>1895.0</t>
+        </is>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr"/>
@@ -16157,8 +16745,10 @@
           <t>https://paraglidingshop.ch/Ozone-Swift-6-ML-Ex-Demo/SW10522</t>
         </is>
       </c>
-      <c r="F164" t="n">
-        <v>2667</v>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>2667.0</t>
+        </is>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
@@ -16206,8 +16796,10 @@
           <t>https://paraglidingshop.ch/Phi-Maestro-23/SW10330</t>
         </is>
       </c>
-      <c r="F165" t="n">
-        <v>952</v>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>952.0</t>
+        </is>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr"/>
@@ -16324,4 +16916,928 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Nevětveno Nekoupáno S batohem Křídlo EN B Sky Country DISCOVERY 5 M 80-10</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-trees-no-water-wit-6727/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá TK platná Křídlo EN B GIN Explorer 2 M 85-105kg Lis</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-t-6524/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-6441/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 177,07 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-flying-on-the-sand-no-t-6390/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ozone Swift 6 ML Ex-Demo</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Ozone-Swift-6-ML-Ex-Demo/SW10522</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2667</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ENB</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Supair Birdy (EN A)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>3333</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>80kg–105kg</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Airdesign Vivo (EN B)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>85kg–105kg</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Phi Maestro</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>75kg-95kg</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Doudek Soul</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 807,04 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Al</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Airdesign Rise 4 (EN B)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>72kg–92kg</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-04-27
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -16924,20 +16924,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17006,524 +17006,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Nevětveno Nekoupáno S batohem Křídlo EN B Sky Country DISCOVERY 5 M 80-10</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-trees-no-water-wit-6727/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá TK platná Křídlo EN B GIN Explorer 2 M 85-105kg Lis</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-t-6524/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-6441/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 177,07 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho M 80-103kg Nové Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-flying-on-the-sand-no-t-6390/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Ozone Swift 6 ML Ex-Demo</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Ozone-Swift-6-ML-Ex-Demo/SW10522</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2667</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ENB</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Supair Birdy (EN A)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>3333</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>80kg–105kg</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Airdesign Vivo (EN B)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>85kg–105kg</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Phi Maestro</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>3190</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>75kg-95kg</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Doudek Soul</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -17538,20 +17020,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17623,220 +17105,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 807,04 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Al</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Airdesign Rise 4 (EN B)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>72kg–92kg</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(sources): add airsport_cz (PrestaShop) + abc_paragliding_cz (HTML tabulka)
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M149"/>
+  <dimension ref="A1:M161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8234,6 +8234,654 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Gradient - Bright 5 (2014, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>1680.0</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Gradient - Bright 5 (2014, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>1450.0</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 4 (2013, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 2 (2009, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Gradiuent - Impuls 4 (2011, vel. 26)</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>960.0</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2011.0</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Gradient - Orbit 3 (2009, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>990.0</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>EN-B</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Gradiuent - Impuls 4 (2012, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>990.0</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2012.0</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 2 (2009, vel. 30)</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>960.0</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 2 (2010, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>780.0</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2010.0</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Gradient - Aspen 5 (2104, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>1680.0</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>EN-C</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Gadient - Stream 2 (2011, vel. 26)</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>1090.0</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2011.0</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>EN-C</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>BRIGHT5 30</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=325&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>840.0</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8245,7 +8893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M148"/>
+  <dimension ref="A1:M160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16002,6 +16650,654 @@
       <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Gradient - Bright 5 (2014, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>1680.0</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Gradient - Bright 5 (2014, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>1450.0</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 4 (2013, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 2 (2009, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Gradiuent - Impuls 4 (2011, vel. 26)</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>960.0</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2011.0</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Gradient - Orbit 3 (2009, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>990.0</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>EN-B</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Gradiuent - Impuls 4 (2012, vel. 28)</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>990.0</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2012.0</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 2 (2009, vel. 30)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>960.0</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2009.0</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Gradient - Impuls 2 (2010, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>780.0</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2010.0</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>EN-A</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Gradient - Aspen 5 (2104, vel. 24)</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>1680.0</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>EN-C</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>abc_paragliding_cz</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>ABC Paragliding CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Gadient - Stream 2 (2011, vel. 26)</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://www.abcparagliding.cz/bazar/13-prodam/</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>1090.0</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2011.0</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>EN-C</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>BRIGHT5 30</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=325&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>840.0</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
@@ -16114,20 +17410,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -16196,1218 +17492,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Nevětveno Nekoupáno S batohem Křídlo EN B Sky Country DISCOVERY 5 M 80-10</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-trees-no-water-wit-6727/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1250</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-6645/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Iota DLS 27 95-115kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupán Křídlo EN B</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-95-115kg-concertinas-lightened-no-si-6556/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá TK platná Křídlo EN B GIN Explorer 2 M 85-105kg Lis</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-t-6524/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-6441/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Illusion 28 Žádné SIV TK čerstvá TK platná S batohem Křídlo EN B MAC Illusion 28 Žádné SIV TK čerstvá TK</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-no-sivs-tc-fresh-tc-valid-with-bag-6411/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 145,91 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nevětveno Nekoupáno Drobné opravy TK platná S batohem Křídlo EN A MAC Luck</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-trees-no-water-small--6463/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho M 80-103kg Nové Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-flying-on-the-sand-no-t-6390/</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 28 80-118kg Nekoupáno S batohem Křídlo EN A Advance Alpha 7 28 80-118kg Nekoupáno S batohem</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-28-80-118kg-no-water-with-bag-6354/</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Advance Sigma 12 28</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>3650</v>
-      </c>
-      <c r="G12" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>105kg-128kg</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>sehr guter Zustand  --&gt; 12 Flüge mit 3h</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>parafly_at</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Parafly AT – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Skywalk RANGE X-ALPS3 Athlete Version M</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://shop.parafly.at/produkt/skywalk-range-x-alps3-athlete-version-m/</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>1690</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>flugsport_de</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Flugsport DE – Gebrauchtschirme</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Swing Nyra RS M</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>B-G</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>85-105</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>ADVANCE Epsilon DLS 28</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Epsilon-DLS-28</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>2950</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>ADVANCE Iota DLS 27</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-IotaDLS-27</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>ADVANCE Pi 3.27</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3.27</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>2350</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>ADVANCE Pi 3.27</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3.27/SW10845</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>2475</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>ADVANCE Success 5 M</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Success-5-M/SW10858</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>750</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Advance Pi 3 27 weiss, Ex-Demo</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Advance-Pi-3-27-weiss-Ex-Demo/SW10521</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>1895</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Ozone Swift 6 ML Ex-Demo</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Ozone-Swift-6-ML-Ex-Demo/SW10522</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>2667</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>ENB</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Supair Birdy (EN A)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>3333</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>80kg–105kg</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Airdesign Vivo (EN B)</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>85kg–105kg</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Phi Maestro</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>3190</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>75kg-95kg</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Doudek Soul</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -17422,20 +17506,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17507,1751 +17591,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Nové Křídlo EN B Advance Iota DLS 25 80-100kg Nové 80 000,00 CZK EN B Velikost:</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-new-6764/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Pluto 4 S 60-85kg Žádné SIV Nelétáno na písku Nekoupáno Drobné opravy S batohem Křídlo EN B AXIS Pluto</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-s-60-85kg-no-sivs-no-flying-on-the-sand-no--6602/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Epsilon 10 DLS 24 65-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Adva</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-10-dls-24-65-90kg-concertinas-no-sivs-no-6569/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B Advance</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-si-6416/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kom</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95kg-concertinas-no-sivs-no-flying-6749/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2300</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 22 50-85kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Alp</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-22-50-85kg-no-sivs-no-flying-on-the-sand-6667/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SWING Mito S 70-95kg Listovaný Žádné SIV TK není Nevětveno Nekoupáno Drobné opravy S batohem Křídlo EN A SWI</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/swing-mito-s-70-95kg-concertinas-no-sivs-no-tc-no-trees--6664/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 8 DLS 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Advanc</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-8-dls-26-70-110kg-concertinas-no-sivs-no-f-6534/</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Křídlo EN A APCO gradient Nevada 2 26 80-102kg Listovaný Křídlo EN A APCO gradient Nevada 2 26 80-102kg Listovaný 10 000</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/apco-gradient-nevada-2-26-80-102kg-concertinas-6467/</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Niviuk Artik 7 P 24</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>3450</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>85kg-105kg</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>sehr gut/neuwertig --&gt; 24 Flüge  --&gt; kei</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Niviuk Artik 7 P 22</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>3490</v>
-      </c>
-      <c r="G13" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>65kg-85kg</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>sehr gut/neuwertig --&gt; 27 Flüge  --&gt; kei</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>parafly_at</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Parafly AT – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>AirDesign Vivo in Größe S</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://shop.parafly.at/produkt/airdesign-vivo-in-groesse-s/</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>flugsport_de</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Flugsport DE – Gebrauchtschirme</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Swing Serac RS XS</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>B-G</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>55-80</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>flugsport_de</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Flugsport DE – Gebrauchtschirme</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Swing Nyra RS S</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>B-G</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>75-95</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>ADVANCE Epsilon DLS 24</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-EpsilonDLS-24</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>2650</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>ADVANCE Impress 4 S</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/Advance-Impress-4-S</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>1290</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>ADVANCE Iota DLS 25</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Iota-DLS-25</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>2550</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>ADVANCE Iota DLS 25</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Iota-DLS-25/SW10844</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>1975</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>ADVANCE Pi 3.23</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/Advance-Pi-3-23</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>2175</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>ADVANCE Pi 3.25</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3-25</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>ADVANCE Pi 3.25</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3.25/SW10847</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>2650</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>ADVANCE Sigma DLS 26</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-SigmaDLS-26</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>3675</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Livi XS</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-XS</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>2450</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Soar S</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-S</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>1650</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Airdesign Soar XS</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/Airdesign-Soar-XS</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>1075</v>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>swissgliders_ch</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Swissgliders CH – Fundgrube</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Verkaufe Niviuk Ikuma 2 24 ( 70 -90 kg</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>https://swissgliders.ch/de/2026/04/14/verkaufe-niviuk-ikuma-2-24-70-90-kg/</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>1429</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>70-90kg</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>swissgliders_ch</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Swissgliders CH – Fundgrube</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>AirDesign Soar XS – Farbe: sky</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>https://swissgliders.ch/de/2026/04/14/airdesign-soar-xs-farbe-sky/</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>952</v>
-      </c>
-      <c r="G29" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>60-78kg</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>swissgliders_ch</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Swissgliders CH – Fundgrube</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Nova Ion 5 Light XS</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>https://swissgliders.ch/de/2026/03/25/nova-ion-5-light-xs/</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>952</v>
-      </c>
-      <c r="G30" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Advance Iota DLS 25 Royal Occasion (EN-B 80-100kg)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Advance-Iota-DLS-25-Royal-Occasion-EN-B-80-100kg/SW10406</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>2667</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>EN-B</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>80-100kg</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Mentor 5 light /S (80kg-100kg)</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Mentor-5-light-S-80kg-100kg/SW10333</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>951</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Phi Maestro 23</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Phi-Maestro-23/SW10330</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>952</v>
-      </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Supair Birdy (EN A)</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>3333</v>
-      </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>65kg–85kg</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Airdesign Rise 4 (EN B)</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>72kg–92kg</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Gradient Bright 5</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>2333</v>
-      </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>63kg-80kg</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-04-28
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -10,8 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vsechny inzeraty" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dnes pridane" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martin – velikost M (mid-B a..." sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martin – velikost XS (mid-B ..." sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martin – velikost S-M (mid-B..." sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A, XS-S, do 1500 €" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17410,20 +17410,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17492,6 +17492,2694 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Nové Křídlo EN B Advance Iota DLS 25 80-100kg Nové 80 000,00 CZK EN B Velikost:</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-new-6764/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Nevětveno Nekoupáno S batohem Křídlo EN B Sky Country DISCOVERY 5 M 80-10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-trees-no-water-wit-6727/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-6645/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 4 S 60-85kg Žádné SIV Nelétáno na písku Nekoupáno Drobné opravy S batohem Křídlo EN B AXIS Pluto</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-s-60-85kg-no-sivs-no-flying-on-the-sand-no--6602/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon 10 DLS 24 65-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Adva</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-10-dls-24-65-90kg-concertinas-no-sivs-no-6569/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 27 95-115kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupán Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-95-115kg-concertinas-lightened-no-si-6556/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá TK platná Křídlo EN B GIN Explorer 2 M 85-105kg Lis</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-t-6524/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-6441/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B Advance</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-si-6416/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 Žádné SIV TK čerstvá TK platná S batohem Křídlo EN B MAC Illusion 28 Žádné SIV TK čerstvá TK</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-no-sivs-tc-fresh-tc-valid-with-bag-6411/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kom</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95kg-concertinas-no-sivs-no-flying-6749/</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SWING Mito S 70-95kg Listovaný Žádné SIV TK není Nevětveno Nekoupáno Drobné opravy S batohem Křídlo EN A SWI</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/swing-mito-s-70-95kg-concertinas-no-sivs-no-tc-no-trees--6664/</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 145,91 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 8 DLS 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Advanc</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-8-dls-26-70-110kg-concertinas-no-sivs-no-f-6534/</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Křídlo EN A APCO gradient Nevada 2 26 80-102kg Listovaný Křídlo EN A APCO gradient Nevada 2 26 80-102kg Listovaný 10 000</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/apco-gradient-nevada-2-26-80-102kg-concertinas-6467/</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nevětveno Nekoupáno Drobné opravy TK platná S batohem Křídlo EN A MAC Luck</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-trees-no-water-small--6463/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-flying-on-the-sand-no-t-6390/</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 28 80-118kg Nekoupáno S batohem Křídlo EN A Advance Alpha 7 28 80-118kg Nekoupáno S batohem</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-28-80-118kg-no-water-with-bag-6354/</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Niviuk Artik 7 P 24</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>85kg-105kg</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>sehr gut/neuwertig --&gt; 24 Flüge  --&gt; kei</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Advance Sigma 12 28</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>105kg-128kg</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand  --&gt; 12 Flüge mit 3h</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Skywalk RANGE X-ALPS3 Athlete Version M</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/skywalk-range-x-alps3-athlete-version-m/</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1690</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>AirDesign Vivo in Größe S</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/airdesign-vivo-in-groesse-s/</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>flugsport_de</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Flugsport DE – Gebrauchtschirme</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Swing Nyra RS S</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>B-G</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>75-95</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>flugsport_de</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Flugsport DE – Gebrauchtschirme</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Swing Nyra RS M</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>B-G</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>85-105</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ADVANCE Epsilon DLS 24</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-EpsilonDLS-24</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ADVANCE Epsilon DLS 28</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Epsilon-DLS-28</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ADVANCE Impress 4 S</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Advance-Impress-4-S</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1290</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ADVANCE Iota DLS 25</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Iota-DLS-25</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>2550</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ADVANCE Iota DLS 25</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Iota-DLS-25/SW10844</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1975</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ADVANCE Iota DLS 27</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-IotaDLS-27</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ADVANCE Pi 3.25</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3-25</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>ADVANCE Pi 3.25</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3.25/SW10847</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ADVANCE Pi 3.27</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3.27</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ADVANCE Pi 3.27</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Pi-3.27/SW10845</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>2475</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ADVANCE Sigma DLS 26</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-SigmaDLS-26</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>3675</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ADVANCE Success 5 M</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Success-5-M/SW10858</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>750</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Soar S</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-S</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>swissgliders_ch</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Swissgliders CH – Fundgrube</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Verkaufe Niviuk Ikuma 2 24 ( 70 -90 kg</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://swissgliders.ch/de/2026/04/14/verkaufe-niviuk-ikuma-2-24-70-90-kg/</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1429</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>70-90kg</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Advance Iota DLS 25 Royal Occasion (EN-B 80-100kg)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Advance-Iota-DLS-25-Royal-Occasion-EN-B-80-100kg/SW10406</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>2667</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EN-B</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>80-100kg</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Advance Pi 3 27 weiss, Ex-Demo</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Advance-Pi-3-27-weiss-Ex-Demo/SW10521</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1895</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Mentor 5 light /S (80kg-100kg)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Mentor-5-light-S-80kg-100kg/SW10333</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>951</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Ozone Swift 6 ML Ex-Demo</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Ozone-Swift-6-ML-Ex-Demo/SW10522</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>2667</v>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>ENB</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Supair Birdy (EN A)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>3333</v>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>65kg–85kg</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Supair Birdy (EN A)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>3333</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>80kg–105kg</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Airdesign Vivo (EN B)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>85kg–105kg</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Airdesign Rise 4 (EN B)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>72kg–92kg</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Gradient Bright 5</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>2333</v>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>63kg-80kg</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Phi Maestro</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>75kg-95kg</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>alpstein_ch</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Flugschule Alpstein CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Doudek Soul</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Gin Explorer 2 S Occasion</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/gin-explorer-2-s-occasion/</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1667</v>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Ozone Delta 5 Lime ML Occasion</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/ozone-delta-5-lime-ml-occasion/</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>2848</v>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Alta S Occasion Schirm</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/alta-s-occasion-schirm/</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>2752</v>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Calypso 2 M Occasion Schirm</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/calypso-2-m-occasion-schirm/</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>3038</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -17506,20 +20194,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17591,6 +20279,169 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 790,72 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Al</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: Klarka pridat low-B, opravit text bez limitu 1500 eur
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dnes pridane" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martin – velikost S-M (mid-B..." sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A, XS-S" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A, XS-S, do 1500 €" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20194,16 +20194,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -20297,19 +20297,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kom</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 790,72 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95kg-concertinas-no-sivs-no-flying-6749/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2300</v>
+        <v>1100</v>
       </c>
       <c r="G2" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -20318,13 +20318,13 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -20352,16 +20352,16 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 790,72 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Al</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6683/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="G3" t="n">
         <v>2020</v>
@@ -20373,13 +20373,13 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -20407,19 +20407,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 7 22 50-85kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Alp</t>
+          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-22-50-85kg-no-sivs-no-flying-on-the-sand-6667/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1800</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -20428,7 +20426,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -20439,330 +20437,6 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SWING Mito S 70-95kg Listovaný Žádné SIV TK není Nevětveno Nekoupáno Drobné opravy S batohem Křídlo EN A SWI</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/swing-mito-s-70-95kg-concertinas-no-sivs-no-tc-no-trees--6664/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 8 DLS 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Advanc</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-8-dls-26-70-110kg-concertinas-no-sivs-no-f-6534/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Advance Al</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-no-sivs-no-flying-on-the-san-6529/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-80kg-concertinas-no-sivs-no-flying-6506/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN A APCO gradient Nevada 2 26 80-102kg Listovaný Křídlo EN A APCO gradient Nevada 2 26 80-102kg Listovaný 10 000</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/apco-gradient-nevada-2-26-80-102kg-concertinas-6467/</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>alpstein_ch</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Flugschule Alpstein CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Supair Birdy (EN A)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://www.flugschule-alpstein.ch/occasionen/</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>3333</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>65kg–85kg</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-06
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M179"/>
+  <dimension ref="A1:M196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -9786,8 +9786,10 @@
         </is>
       </c>
       <c r="F178" t="inlineStr"/>
-      <c r="G178" t="n">
-        <v>2025</v>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
@@ -9838,8 +9840,10 @@
           <t>https://shop.flugschule-hochries.de/Advance-Lightness-2L</t>
         </is>
       </c>
-      <c r="F179" t="n">
-        <v>385</v>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>385.0</t>
+        </is>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr"/>
@@ -9854,6 +9858,911 @@
       <c r="M179" t="inlineStr">
         <is>
           <t>2026-05-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient BiGolden 4 37 100-190kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstv Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bigolden-4-37-100-190kg-new-no-sivs-no-flying-o-6824/</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 29 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Advance</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-29-105-130kg-concertinas-no-sivs-no-fly-6816/</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platná Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platn</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-ultralite-3-21-55-90kg-lightened-tc-valid-6814/</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="n">
+        <v>2013</v>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base S 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná S batohe Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-s-60-80kg-concertinas-no-sivs-no-flying-on-the--6813/</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 S 70-90kg TK není Nekoupáno Drobné opravy S batohem Křídlo EN B Sky Country DISCOVER</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-s-70-90kg-no-tc-no-water-small-r-6812/</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G186" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 694,18 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G187" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 603,70 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>599</v>
+      </c>
+      <c r="G188" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr"/>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>720</v>
+      </c>
+      <c r="G189" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Golden 4 30 105-130kg TK platná S batohem S listovacím obalem Křídlo EN A Gradient Golden 4 30 105-</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-30-105-130kg-tc-valid-with-bag-with-li-6820/</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G192" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY AYA-XL 100-130kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná Křídlo EN A SKY AY</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-100-130kg-concertinas-no-sivs-no-flying-on-th-6818/</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Bright 26 75-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient Bright 26 75</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-26-75-95kg-no-sivs-no-flying-on-the-sand-6815/</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>290</v>
+      </c>
+      <c r="G194" t="n">
+        <v>2003</v>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G195" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 198,28 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G196" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr"/>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -9868,7 +10777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -10856,8 +11765,10 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>2025</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -10908,8 +11819,10 @@
           <t>https://shop.flugschule-hochries.de/Advance-Lightness-2L</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>385</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>385.0</t>
+        </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -10924,6 +11837,911 @@
       <c r="M19" t="inlineStr">
         <is>
           <t>2026-05-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient BiGolden 4 37 100-190kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstv Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bigolden-4-37-100-190kg-new-no-sivs-no-flying-o-6824/</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 29 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Advance</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-29-105-130kg-concertinas-no-sivs-no-fly-6816/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platná Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platn</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-ultralite-3-21-55-90kg-lightened-tc-valid-6814/</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>2013</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base S 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná S batohe Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-s-60-80kg-concertinas-no-sivs-no-flying-on-the--6813/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 S 70-90kg TK není Nekoupáno Drobné opravy S batohem Křídlo EN B Sky Country DISCOVER</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-s-70-90kg-no-tc-no-water-small-r-6812/</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 694,18 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 603,70 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>599</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>720</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Golden 4 30 105-130kg TK platná S batohem S listovacím obalem Křídlo EN A Gradient Golden 4 30 105-</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-30-105-130kg-tc-valid-with-bag-with-li-6820/</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY AYA-XL 100-130kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná Křídlo EN A SKY AY</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-100-130kg-concertinas-no-sivs-no-flying-on-th-6818/</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Bright 26 75-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient Bright 26 75</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-26-75-95kg-no-sivs-no-flying-on-the-sand-6815/</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>290</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2003</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 198,28 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -10938,20 +12756,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -11026,98 +12844,905 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>flugsport_de</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Flugsport DE – Gebrauchtschirme</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Advance Iota DLS 25</t>
+          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>B-R</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>80-100</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hochries_de</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Advance Lightness 2 L</t>
+          <t>Křídlo EN B Gradient BiGolden 4 37 100-190kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstv Křídlo EN B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/Advance-Lightness-2L</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>385</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bigolden-4-37-100-190kg-new-no-sivs-no-flying-o-6824/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>37</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 29 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Advance</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-29-105-130kg-concertinas-no-sivs-no-fly-6816/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platná Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platn</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-ultralite-3-21-55-90kg-lightened-tc-valid-6814/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2013</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base S 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná S batohe Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-s-60-80kg-concertinas-no-sivs-no-flying-on-the--6813/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 S 70-90kg TK není Nekoupáno Drobné opravy S batohem Křídlo EN B Sky Country DISCOVER</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-s-70-90kg-no-tc-no-water-small-r-6812/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 694,18 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 603,70 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>599</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>720</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Golden 4 30 105-130kg TK platná S batohem S listovacím obalem Křídlo EN A Gradient Golden 4 30 105-</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-30-105-130kg-tc-valid-with-bag-with-li-6820/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY AYA-XL 100-130kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná Křídlo EN A SKY AY</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-100-130kg-concertinas-no-sivs-no-flying-on-th-6818/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Bright 26 75-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient Bright 26 75</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-26-75-95kg-no-sivs-no-flying-on-the-sand-6815/</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>290</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2003</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 198,28 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -11132,20 +13757,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -11220,53 +13845,271 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>flugsport_de</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Flugsport DE – Gebrauchtschirme</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Advance Iota DLS 25</t>
+          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>B-R</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>80-100</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>720</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 198,28 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -11281,20 +14124,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -11363,6 +14206,226 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>720</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -11377,20 +14440,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="59" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -11465,45 +14528,269 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hochries_de</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Advance Lightness 2 L</t>
+          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/Advance-Lightness-2L</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>385</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 29 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Advance</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-29-105-130kg-concertinas-no-sivs-no-fly-6816/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-07
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M196"/>
+  <dimension ref="A1:M202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -9888,8 +9888,10 @@
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
-      <c r="G180" t="n">
-        <v>2024</v>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
@@ -9941,8 +9943,10 @@
         </is>
       </c>
       <c r="F181" t="inlineStr"/>
-      <c r="G181" t="n">
-        <v>2019</v>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
@@ -9994,8 +9998,10 @@
         </is>
       </c>
       <c r="F182" t="inlineStr"/>
-      <c r="G182" t="n">
-        <v>2023</v>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
@@ -10047,8 +10053,10 @@
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
-      <c r="G183" t="n">
-        <v>2013</v>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
@@ -10100,8 +10108,10 @@
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
-      <c r="G184" t="n">
-        <v>2018</v>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
@@ -10153,8 +10163,10 @@
         </is>
       </c>
       <c r="F185" t="inlineStr"/>
-      <c r="G185" t="n">
-        <v>2016</v>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
@@ -10205,11 +10217,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F186" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G186" t="n">
-        <v>2020</v>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
@@ -10260,11 +10276,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F187" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G187" t="n">
-        <v>2023</v>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
@@ -10311,11 +10331,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F188" t="n">
-        <v>599</v>
-      </c>
-      <c r="G188" t="n">
-        <v>2015</v>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
@@ -10362,11 +10386,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
         </is>
       </c>
-      <c r="F189" t="n">
-        <v>720</v>
-      </c>
-      <c r="G189" t="n">
-        <v>2021</v>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>720.0</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
@@ -10418,8 +10446,10 @@
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
-      <c r="G190" t="n">
-        <v>2025</v>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
@@ -10471,8 +10501,10 @@
         </is>
       </c>
       <c r="F191" t="inlineStr"/>
-      <c r="G191" t="n">
-        <v>2011</v>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
@@ -10523,11 +10555,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
         </is>
       </c>
-      <c r="F192" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G192" t="n">
-        <v>2024</v>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
@@ -10579,8 +10615,10 @@
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
-      <c r="G193" t="n">
-        <v>2021</v>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
@@ -10627,11 +10665,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-26-75-95kg-no-sivs-no-flying-on-the-sand-6815/</t>
         </is>
       </c>
-      <c r="F194" t="n">
-        <v>290</v>
-      </c>
-      <c r="G194" t="n">
-        <v>2003</v>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>290.0</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
@@ -10682,11 +10724,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
         </is>
       </c>
-      <c r="F195" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G195" t="n">
-        <v>2020</v>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
@@ -10737,11 +10783,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F196" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G196" t="n">
-        <v>2026</v>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
@@ -10763,6 +10813,326 @@
       <c r="M196" t="inlineStr">
         <is>
           <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G197" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr"/>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 641,72 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G198" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr"/>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 579,53 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>599</v>
+      </c>
+      <c r="G199" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr"/>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr"/>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G201" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr"/>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 113,55 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G202" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -10777,7 +11147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11867,8 +12237,10 @@
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="n">
-        <v>2024</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -11920,8 +12292,10 @@
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
-        <v>2019</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -11973,8 +12347,10 @@
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="n">
-        <v>2023</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -12026,8 +12402,10 @@
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="n">
-        <v>2013</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -12079,8 +12457,10 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>2018</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -12132,8 +12512,10 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="n">
-        <v>2016</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -12184,11 +12566,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G26" t="n">
-        <v>2020</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -12239,11 +12625,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G27" t="n">
-        <v>2023</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -12290,11 +12680,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>599</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2015</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -12341,11 +12735,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>720</v>
-      </c>
-      <c r="G29" t="n">
-        <v>2021</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>720.0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -12397,8 +12795,10 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="n">
-        <v>2025</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -12450,8 +12850,10 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="n">
-        <v>2011</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -12502,11 +12904,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G32" t="n">
-        <v>2024</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -12558,8 +12964,10 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>2021</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -12606,11 +13014,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-26-75-95kg-no-sivs-no-flying-on-the-sand-6815/</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>290</v>
-      </c>
-      <c r="G34" t="n">
-        <v>2003</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>290.0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -12661,11 +13073,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G35" t="n">
-        <v>2020</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -12716,11 +13132,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G36" t="n">
-        <v>2026</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -12742,6 +13162,326 @@
       <c r="M36" t="inlineStr">
         <is>
           <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 641,72 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 579,53 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>599</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 113,55 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -12756,7 +13496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -12859,17 +13599,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
       <c r="G2" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -12884,13 +13626,13 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -12912,28 +13654,26 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient BiGolden 4 37 100-190kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstv Křídlo EN B</t>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 641,72 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-bigolden-4-37-100-190kg-new-no-sivs-no-flying-o-6824/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1300</v>
+      </c>
       <c r="G3" t="n">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
@@ -12943,7 +13683,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -12965,50 +13705,48 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Iota DLS 29 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Advance</t>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 579,53 CZK (599,00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-29-105-130kg-concertinas-no-sivs-no-fly-6816/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>599</v>
+      </c>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -13018,50 +13756,50 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platná Křídlo EN B Ozone ultralite 3 21 55-90kg Odlehčeno TK platn</t>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-ultralite-3-21-55-90kg-lightened-tc-valid-6814/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2013</v>
+        <v>2024</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -13071,26 +13809,28 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Base S 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná S batohe Křídlo EN B</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-s-60-80kg-concertinas-no-sivs-no-flying-on-the--6813/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1100</v>
+      </c>
       <c r="G6" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -13102,19 +13842,19 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -13124,625 +13864,40 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN B Sky Country DISCOVERY 5 S 70-90kg TK není Nekoupáno Drobné opravy S batohem Křídlo EN B Sky Country DISCOVER</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 113,55 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-s-70-90kg-no-tc-no-water-small-r-6812/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2100</v>
+      </c>
       <c r="G7" t="n">
-        <v>2016</v>
+        <v>2026</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 694,18 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 603,70 CZK (599,00</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>599</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>720</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Gradient Golden 4 30 105-130kg TK platná S batohem S listovacím obalem Křídlo EN A Gradient Golden 4 30 105-</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-30-105-130kg-tc-valid-with-bag-with-li-6820/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
-        <v>2011</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G14" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SKY AYA-XL 100-130kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná Křídlo EN A SKY AY</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-100-130kg-concertinas-no-sivs-no-flying-on-th-6818/</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Gradient Bright 26 75-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient Bright 26 75</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-26-75-95kg-no-sivs-no-flying-on-the-sand-6815/</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>290</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2003</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G17" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 198,28 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G18" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -13757,7 +13912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13845,12 +14000,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -13860,12 +14015,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -13874,12 +14029,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -13891,7 +14046,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -13913,19 +14068,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 113,55 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>720</v>
+        <v>2100</v>
       </c>
       <c r="G3" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -13934,182 +14089,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 198,28 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -14124,7 +14116,213 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14227,7 +14425,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -14260,7 +14458,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -14282,19 +14480,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-6826/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>720</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -14303,7 +14499,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -14315,7 +14511,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -14337,19 +14533,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Nova aonic S-80kg 100 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-80kg-100-concertinas-no-sivs-no-flying-on-t-6819/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1600</v>
+        <v>1100</v>
       </c>
       <c r="G4" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -14358,439 +14554,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B SKY Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B SKY K</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-2-m-74-94kg-no-sivs-no-flying-on-the-sand-no-t-6829/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Iota DLS 29 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Advance</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-29-105-130kg-concertinas-no-sivs-no-fly-6816/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 380,14 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho M 80-103kg Nové Žádné SIV Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A Drift carancho</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-new-no-sivs-no-trees-no-water--6825/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 818,15 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6774/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-08
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M202"/>
+  <dimension ref="A1:M207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -10842,11 +10842,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F197" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G197" t="n">
-        <v>2020</v>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
@@ -10897,11 +10901,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F198" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G198" t="n">
-        <v>2023</v>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
@@ -10948,11 +10956,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F199" t="n">
-        <v>599</v>
-      </c>
-      <c r="G199" t="n">
-        <v>2015</v>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
@@ -11000,8 +11012,10 @@
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
-      <c r="G200" t="n">
-        <v>2024</v>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
@@ -11052,11 +11066,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
         </is>
       </c>
-      <c r="F201" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G201" t="n">
-        <v>2020</v>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
@@ -11107,11 +11125,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F202" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G202" t="n">
-        <v>2026</v>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
@@ -11133,6 +11155,277 @@
       <c r="M202" t="inlineStr">
         <is>
           <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G203" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr"/>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 596,34 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G204" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G205" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr"/>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G206" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr"/>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Niviuk Ikuma 3 26</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G207" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H207" t="inlineStr"/>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>85kg-105kg</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr"/>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -11147,7 +11440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11160,7 +11453,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -13191,11 +13484,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G37" t="n">
-        <v>2020</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -13246,11 +13543,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G38" t="n">
-        <v>2023</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -13297,11 +13598,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>599</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2015</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -13349,8 +13654,10 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="n">
-        <v>2024</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -13401,11 +13708,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G41" t="n">
-        <v>2020</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -13456,11 +13767,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G42" t="n">
-        <v>2026</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -13482,6 +13797,277 @@
       <c r="M42" t="inlineStr">
         <is>
           <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 596,34 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G44" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Niviuk Ikuma 3 26</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>85kg-105kg</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -13496,7 +14082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13509,7 +14095,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -13599,7 +14185,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -13632,7 +14218,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -13654,7 +14240,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 641,72 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 596,34 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -13683,19 +14269,19 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -13705,36 +14291,40 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 579,53 CZK (599,00</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>599</v>
+        <v>1100</v>
       </c>
       <c r="G4" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -13756,17 +14346,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2100</v>
+      </c>
       <c r="G5" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -13775,129 +14367,74 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_store_at</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Store AT – Used</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Niviuk Ikuma 3 26</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1100</v>
+        <v>2390</v>
       </c>
       <c r="G6" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
+        <v>2024</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>85kg-105kg</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 113,55 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -13925,7 +14462,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -14015,17 +14552,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2100</v>
+      </c>
       <c r="G2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -14034,74 +14573,74 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_store_at</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Store AT – Used</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 113,55 CZK (2 100,00</t>
+          <t>Niviuk Ikuma 3 26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2100</v>
+        <v>2390</v>
       </c>
       <c r="G3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
+        <v>2024</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>85kg-105kg</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -14111,6 +14650,322 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Niviuk Ikuma 3 26</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>85kg-105kg</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14219,7 +15074,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -14252,7 +15107,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -14274,7 +15129,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -14307,266 +15162,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 339,78 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-concertinas-no-sivs-no-flying-on-6838/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 773,76 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-09
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M207"/>
+  <dimension ref="A1:M209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11184,11 +11184,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F203" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G203" t="n">
-        <v>2020</v>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
@@ -11239,11 +11243,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F204" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G204" t="n">
-        <v>2023</v>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
@@ -11290,11 +11298,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
         </is>
       </c>
-      <c r="F205" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G205" t="n">
-        <v>2020</v>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
@@ -11345,11 +11357,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F206" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G206" t="n">
-        <v>2026</v>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
@@ -11400,11 +11416,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F207" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G207" t="n">
-        <v>2024</v>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>2390.0</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
@@ -11426,6 +11446,110 @@
       <c r="M207" t="inlineStr">
         <is>
           <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr"/>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 558,62 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>599</v>
+      </c>
+      <c r="G209" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13826,11 +13950,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G43" t="n">
-        <v>2020</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -13881,11 +14009,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G44" t="n">
-        <v>2023</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -13932,11 +14064,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G45" t="n">
-        <v>2020</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -13987,11 +14123,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G46" t="n">
-        <v>2026</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -14042,11 +14182,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2024</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2390.0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
@@ -14068,6 +14212,110 @@
       <c r="M47" t="inlineStr">
         <is>
           <t>2026-05-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 558,62 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>599</v>
+      </c>
+      <c r="G49" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -14077,895 +14325,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 596,34 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Niviuk Ikuma 3 26</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>85kg-105kg</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Niviuk Ikuma 3 26</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>85kg-105kg</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 040,25 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Niviuk Ikuma 3 26</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2390</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>85kg-105kg</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>sehr gut --&gt; 60 Flüge  --&gt; keine Beschäd</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15074,19 +14433,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 304,88 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2025</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -15095,7 +14452,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -15107,19 +14464,19 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -15129,40 +14486,430 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 558,62 CZK (599,00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6833/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1100</v>
+        <v>599</v>
       </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-10
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M209"/>
+  <dimension ref="A1:M213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11476,8 +11476,10 @@
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
-      <c r="G208" t="n">
-        <v>2025</v>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
@@ -11528,11 +11530,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F209" t="n">
-        <v>599</v>
-      </c>
-      <c r="G209" t="n">
-        <v>2015</v>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
@@ -11550,6 +11556,220 @@
       <c r="M209" t="inlineStr">
         <is>
           <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SI</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-90-115kg-no-sivs-no-trees-no-water-tc-val-6856/</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr"/>
+      <c r="G210" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr"/>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-concertinas-no-sivs-no-flying-on-6852/</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr"/>
+      <c r="G211" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr"/>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr"/>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G212" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr"/>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr"/>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr"/>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr"/>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -11564,7 +11784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14242,8 +14462,10 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="n">
-        <v>2025</v>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -14294,11 +14516,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>599</v>
-      </c>
-      <c r="G49" t="n">
-        <v>2015</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -14316,6 +14542,220 @@
       <c r="M49" t="inlineStr">
         <is>
           <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SI</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-90-115kg-no-sivs-no-trees-no-water-tc-val-6856/</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-concertinas-no-sivs-no-flying-on-6852/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G52" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -14330,7 +14770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14343,7 +14783,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -14433,17 +14873,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+          <t>Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-90-115kg-no-sivs-no-trees-no-water-tc-val-6856/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -14452,19 +14892,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -14486,36 +14926,146 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 558,62 CZK (599,00</t>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>599</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-concertinas-no-sivs-no-flying-on-6852/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2015</v>
+        <v>2024</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -14618,12 +15168,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -14633,26 +15183,26 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -14664,7 +15214,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -14679,103 +15229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14863,6 +15317,210 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
@@ -14878,17 +15536,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 28 118-91kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+          <t>Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-118-91kg-no-sivs-no-flying-on-the-6848/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-90-115kg-no-sivs-no-trees-no-water-tc-val-6856/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -14897,19 +15555,180 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-concertinas-no-sivs-no-flying-on-6852/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-11
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M213"/>
+  <dimension ref="A1:M215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11586,8 +11586,10 @@
         </is>
       </c>
       <c r="F210" t="inlineStr"/>
-      <c r="G210" t="n">
-        <v>2021</v>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
@@ -11639,8 +11641,10 @@
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
-      <c r="G211" t="n">
-        <v>2024</v>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
@@ -11691,11 +11695,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
-      <c r="F212" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G212" t="n">
-        <v>2020</v>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
@@ -11747,8 +11755,10 @@
         </is>
       </c>
       <c r="F213" t="inlineStr"/>
-      <c r="G213" t="n">
-        <v>2022</v>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
@@ -11770,6 +11780,114 @@
       <c r="M213" t="inlineStr">
         <is>
           <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 6 L 95-115kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozone Rush 6 L</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-6-l-95-115kg-concertinas-no-flying-on-the-san-6866/</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr"/>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr"/>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 013</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>700</v>
+      </c>
+      <c r="G215" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -11784,7 +11902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14572,8 +14690,10 @@
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="n">
-        <v>2021</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -14625,8 +14745,10 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="n">
-        <v>2024</v>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -14677,11 +14799,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G52" t="n">
-        <v>2020</v>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -14733,8 +14859,10 @@
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="n">
-        <v>2022</v>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -14756,6 +14884,114 @@
       <c r="M53" t="inlineStr">
         <is>
           <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 6 L 95-115kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozone Rush 6 L</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-6-l-95-115kg-concertinas-no-flying-on-the-san-6866/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 013</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>700</v>
+      </c>
+      <c r="G55" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -14770,7 +15006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14873,12 +15109,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SI</t>
+          <t>Křídlo EN B Ozone Rush 6 L 95-115kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozone Rush 6 L</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-90-115kg-no-sivs-no-trees-no-water-tc-val-6856/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-6-l-95-115kg-concertinas-no-flying-on-the-san-6866/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -14898,13 +15134,13 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -14926,17 +15162,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 013</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-concertinas-no-sivs-no-flying-on-6852/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>700</v>
+      </c>
       <c r="G3" t="n">
-        <v>2024</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -14945,7 +15183,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -14957,115 +15195,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -15075,6 +15205,198 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15168,12 +15490,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -15183,365 +15505,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+          <t>Křídlo EN B Ozone Rush 6 L 95-115kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozone Rush 6 L</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4 L 90-115kg Žádné SI</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-l-90-115kg-no-sivs-no-trees-no-water-tc-val-6856/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-6-l-95-115kg-concertinas-no-flying-on-the-san-6866/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -15561,174 +15530,13 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-concertinas-no-sivs-no-flying-on-6852/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 735,37 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-110kg-concertinas-no-sivs-no-flyin-6854/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-12
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M215"/>
+  <dimension ref="A1:M223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11810,8 +11810,10 @@
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
-      <c r="G214" t="n">
-        <v>2021</v>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
@@ -11862,11 +11864,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F215" t="n">
-        <v>700</v>
-      </c>
-      <c r="G215" t="n">
-        <v>2018</v>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
@@ -11888,6 +11894,422 @@
       <c r="M215" t="inlineStr">
         <is>
           <t>2026-05-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 034</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>700</v>
+      </c>
+      <c r="G216" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr"/>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G217" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr"/>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr"/>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 635,56 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G218" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr"/>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr"/>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 576,69 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>599</v>
+      </c>
+      <c r="G219" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr"/>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr"/>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 TK čerstvá Křídlo EN A MAC Lucky 4 TK čerstvá 17 000,00 CZK EN A Vlastnosti: TK čerstvá Opotřebe</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-tc-fresh-6871/</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr"/>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr"/>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G221" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr"/>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 103,59 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G222" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr"/>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>flugsport_de</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Flugsport DE – Gebrauchtschirme</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Swing Mito-3 RS, alle Größen</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr"/>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="inlineStr"/>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>
@@ -11902,7 +12324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14914,8 +15336,10 @@
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="n">
-        <v>2021</v>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -14966,11 +15390,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>700</v>
-      </c>
-      <c r="G55" t="n">
-        <v>2018</v>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -14992,6 +15420,422 @@
       <c r="M55" t="inlineStr">
         <is>
           <t>2026-05-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 034</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>700</v>
+      </c>
+      <c r="G56" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G57" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 635,56 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 576,69 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>599</v>
+      </c>
+      <c r="G59" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 TK čerstvá Křídlo EN A MAC Lucky 4 TK čerstvá 17 000,00 CZK EN A Vlastnosti: TK čerstvá Opotřebe</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-tc-fresh-6871/</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 103,59 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>flugsport_de</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Flugsport DE – Gebrauchtschirme</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Swing Mito-3 RS, alle Größen</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>
@@ -15006,11 +15850,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -15109,17 +15953,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Ozone Rush 6 L 95-115kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozone Rush 6 L</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 034</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-6-l-95-115kg-concertinas-no-flying-on-the-san-6866/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>700</v>
+      </c>
       <c r="G2" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -15128,19 +15974,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>
@@ -15162,19 +16008,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 013</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -15189,13 +16035,319 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 635,56 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 576,69 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>599</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 TK čerstvá Křídlo EN A MAC Lucky 4 TK čerstvá 17 000,00 CZK EN A Vlastnosti: TK čerstvá Opotřebe</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-tc-fresh-6871/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 103,59 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>flugsport_de</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Flugsport DE – Gebrauchtschirme</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Swing Mito-3 RS, alle Größen</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>
@@ -15205,198 +16357,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15490,12 +16450,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -15505,26 +16465,28 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Ozone Rush 6 L 95-115kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozone Rush 6 L</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 103,59 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-6-l-95-115kg-concertinas-no-flying-on-the-san-6866/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2100</v>
+      </c>
       <c r="G2" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -15536,7 +16498,419 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-13
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -12,7 +12,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dnes pridane" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martin – velikost S-M (mid-B..." sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A - low-B, XS-S" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kamarád 1 – M-ML-L, mid-B (8..." sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M223"/>
+  <dimension ref="A1:M231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11923,11 +11922,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F216" t="n">
-        <v>700</v>
-      </c>
-      <c r="G216" t="n">
-        <v>2018</v>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
@@ -11978,11 +11981,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F217" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G217" t="n">
-        <v>2020</v>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
@@ -12033,11 +12040,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F218" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G218" t="n">
-        <v>2023</v>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
@@ -12084,11 +12095,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F219" t="n">
-        <v>599</v>
-      </c>
-      <c r="G219" t="n">
-        <v>2015</v>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H219" t="inlineStr">
         <is>
@@ -12136,8 +12151,10 @@
         </is>
       </c>
       <c r="F220" t="inlineStr"/>
-      <c r="G220" t="n">
-        <v>2016</v>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
@@ -12184,11 +12201,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
-      <c r="F221" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G221" t="n">
-        <v>2020</v>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
@@ -12239,11 +12260,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F222" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G222" t="n">
-        <v>2026</v>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
@@ -12295,8 +12320,10 @@
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
-      <c r="G223" t="n">
-        <v>2026</v>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
@@ -12310,6 +12337,432 @@
       <c r="M223" t="inlineStr">
         <is>
           <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon 9 28 92-114kg Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B Advance Epsilon 9 28 92-1</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-9-28-92-114kg-no-trees-no-water-tc-fresh-6883/</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr"/>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 024</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>700</v>
+      </c>
+      <c r="G225" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr"/>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr"/>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 320,25 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G226" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr"/>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr"/>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 616,32 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G227" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr"/>
+      <c r="J227" t="inlineStr"/>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr"/>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 567,83 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>599</v>
+      </c>
+      <c r="G228" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr"/>
+      <c r="J228" t="inlineStr"/>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr"/>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 240,19 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>750</v>
+      </c>
+      <c r="G229" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr"/>
+      <c r="J229" t="inlineStr"/>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr"/>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 752,27 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G230" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr"/>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 072,52 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F231" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G231" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr"/>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -12324,7 +12777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -15449,11 +15902,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>700</v>
-      </c>
-      <c r="G56" t="n">
-        <v>2018</v>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -15504,11 +15961,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G57" t="n">
-        <v>2020</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -15559,11 +16020,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G58" t="n">
-        <v>2023</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -15610,11 +16075,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>599</v>
-      </c>
-      <c r="G59" t="n">
-        <v>2015</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -15662,8 +16131,10 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="n">
-        <v>2016</v>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -15710,11 +16181,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G61" t="n">
-        <v>2020</v>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -15765,11 +16240,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G62" t="n">
-        <v>2026</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -15821,8 +16300,10 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="n">
-        <v>2026</v>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -15836,6 +16317,432 @@
       <c r="M63" t="inlineStr">
         <is>
           <t>2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon 9 28 92-114kg Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B Advance Epsilon 9 28 92-1</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-9-28-92-114kg-no-trees-no-water-tc-fresh-6883/</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 024</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>700</v>
+      </c>
+      <c r="G65" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 320,25 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G66" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 616,32 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G67" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 567,83 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>599</v>
+      </c>
+      <c r="G68" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 240,19 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>750</v>
+      </c>
+      <c r="G69" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 752,27 CZK (1 100,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G70" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 072,52 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -15854,7 +16761,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -15953,19 +16860,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 034</t>
+          <t>Křídlo EN B Advance Epsilon 9 28 92-114kg Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B Advance Epsilon 9 28 92-1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-9-28-92-114kg-no-trees-no-water-tc-fresh-6883/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -15974,19 +16879,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16008,19 +16913,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 024</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -16035,13 +16940,13 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16063,26 +16968,30 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 635,56 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 320,25 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
@@ -16092,7 +17001,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16114,19 +17023,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 576,69 CZK (599,00</t>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 616,32 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>599</v>
+        <v>1300</v>
       </c>
       <c r="G5" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -16143,19 +17052,19 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -16165,34 +17074,36 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN A MAC Lucky 4 TK čerstvá Křídlo EN A MAC Lucky 4 TK čerstvá 17 000,00 CZK EN A Vlastnosti: TK čerstvá Opotřebe</t>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 567,83 CZK (599,00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-tc-fresh-6871/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>599</v>
+      </c>
       <c r="G6" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16214,40 +17125,36 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 240,19 CZK (750,00 EUR) E</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1100</v>
+        <v>750</v>
       </c>
       <c r="G7" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16269,19 +17176,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 103,59 CZK (2 100,00</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 752,27 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2100</v>
+        <v>1100</v>
       </c>
       <c r="G8" t="n">
-        <v>2026</v>
+        <v>2020</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -16290,64 +17197,74 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>flugsport_de</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Flugsport DE – Gebrauchtschirme</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Swing Mito-3 RS, alle Größen</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 072,52 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.flugsport.de/flugsportladen/gebrauchtschirme.html</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>2100</v>
+      </c>
       <c r="G9" t="n">
         <v>2026</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16465,7 +17382,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 103,59 CZK (2 100,00</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 072,52 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -16498,7 +17415,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16616,7 +17533,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 320,25 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -16649,7 +17566,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -16671,7 +17588,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 752,27 CZK (1 100,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -16704,213 +17621,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 335,04 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 768,55 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-14
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M231"/>
+  <dimension ref="A1:M233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -12367,8 +12367,10 @@
         </is>
       </c>
       <c r="F224" t="inlineStr"/>
-      <c r="G224" t="n">
-        <v>2019</v>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
@@ -12419,11 +12421,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F225" t="n">
-        <v>700</v>
-      </c>
-      <c r="G225" t="n">
-        <v>2018</v>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
@@ -12474,11 +12480,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F226" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G226" t="n">
-        <v>2020</v>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
@@ -12529,11 +12539,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F227" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G227" t="n">
-        <v>2023</v>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H227" t="inlineStr">
         <is>
@@ -12580,11 +12594,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F228" t="n">
-        <v>599</v>
-      </c>
-      <c r="G228" t="n">
-        <v>2015</v>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
@@ -12631,11 +12649,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F229" t="n">
-        <v>750</v>
-      </c>
-      <c r="G229" t="n">
-        <v>2023</v>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H229" t="inlineStr">
         <is>
@@ -12682,11 +12704,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
-      <c r="F230" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G230" t="n">
-        <v>2020</v>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H230" t="inlineStr">
         <is>
@@ -12737,11 +12763,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F231" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G231" t="n">
-        <v>2026</v>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H231" t="inlineStr">
         <is>
@@ -12763,6 +12793,108 @@
       <c r="M231" t="inlineStr">
         <is>
           <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 95-120kg Listovaný Žádné SIV Nelétáno na písku TK čerstvá TK platná (Součást komplet</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-95-120kg-concertinas-no-sivs-no--6894/</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr"/>
+      <c r="J232" t="inlineStr"/>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr"/>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Anakis 3 XL 99-125kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A SKY</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-anakis-3-xl-99-125kg-concertinas-no-sivs-no-flying-o-6889/</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr"/>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -12777,7 +12909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16347,8 +16479,10 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="n">
-        <v>2019</v>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -16399,11 +16533,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>700</v>
-      </c>
-      <c r="G65" t="n">
-        <v>2018</v>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -16454,11 +16592,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G66" t="n">
-        <v>2020</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -16509,11 +16651,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G67" t="n">
-        <v>2023</v>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -16560,11 +16706,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>599</v>
-      </c>
-      <c r="G68" t="n">
-        <v>2015</v>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -16611,11 +16761,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>750</v>
-      </c>
-      <c r="G69" t="n">
-        <v>2023</v>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -16662,11 +16816,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G70" t="n">
-        <v>2020</v>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -16717,11 +16875,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F71" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G71" t="n">
-        <v>2026</v>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -16743,6 +16905,108 @@
       <c r="M71" t="inlineStr">
         <is>
           <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 95-120kg Listovaný Žádné SIV Nelétáno na písku TK čerstvá TK platná (Součást komplet</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-95-120kg-concertinas-no-sivs-no--6894/</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Anakis 3 XL 99-125kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A SKY</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-anakis-3-xl-99-125kg-concertinas-no-sivs-no-flying-o-6889/</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -16752,679 +17016,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Epsilon 9 28 92-114kg Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B Advance Epsilon 9 28 92-1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-9-28-92-114kg-no-trees-no-water-tc-fresh-6883/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 024</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>700</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2018</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 320,25 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 616,32 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 567,83 CZK (599,00</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>599</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 240,19 CZK (750,00 EUR) E</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>750</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 752,27 CZK (1 100,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 072,52 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G9" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 072,52 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17533,40 +17124,34 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 320,25 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 95-120kg Listovaný Žádné SIV Nelétáno na písku TK čerstvá TK platná (Součást komplet</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-95-120kg-concertinas-no-sivs-no--6894/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -17588,19 +17173,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 752,27 CZK (1 100,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A SKY Anakis 3 XL 99-125kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A SKY</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6855/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1100</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-anakis-3-xl-99-125kg-concertinas-no-sivs-no-flying-o-6889/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -17609,19 +17192,211 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-15
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M233"/>
+  <dimension ref="A1:M236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -12823,8 +12823,10 @@
         </is>
       </c>
       <c r="F232" t="inlineStr"/>
-      <c r="G232" t="n">
-        <v>2017</v>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
@@ -12872,8 +12874,10 @@
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
-      <c r="G233" t="n">
-        <v>2015</v>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
@@ -12895,6 +12899,171 @@
       <c r="M233" t="inlineStr">
         <is>
           <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 010</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>700</v>
+      </c>
+      <c r="G234" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr"/>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 300,16 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G235" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr"/>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 727,95 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G236" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr"/>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -12909,7 +13078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16935,8 +17104,10 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="n">
-        <v>2017</v>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -16984,8 +17155,10 @@
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="n">
-        <v>2015</v>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -17007,6 +17180,171 @@
       <c r="M73" t="inlineStr">
         <is>
           <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 010</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>700</v>
+      </c>
+      <c r="G74" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 300,16 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G75" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 727,95 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G76" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -17021,7 +17359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17034,7 +17372,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17124,46 +17462,52 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Sky Country DISCOVERY 5 95-120kg Listovaný Žádné SIV Nelétáno na písku TK čerstvá TK platná (Součást komplet</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 010</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-95-120kg-concertinas-no-sivs-no--6894/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>700</v>
+      </c>
       <c r="G2" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -17173,26 +17517,28 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A SKY Anakis 3 XL 99-125kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A SKY</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 300,16 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-anakis-3-xl-99-125kg-concertinas-no-sivs-no-flying-o-6889/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1000</v>
+      </c>
       <c r="G3" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -17204,7 +17550,62 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 727,95 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -17315,20 +17716,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17400,6 +17801,116 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 300,16 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 727,95 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-16
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M236"/>
+  <dimension ref="A1:M239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -12928,11 +12928,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F234" t="n">
-        <v>700</v>
-      </c>
-      <c r="G234" t="n">
-        <v>2018</v>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
@@ -12983,11 +12987,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F235" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G235" t="n">
-        <v>2020</v>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
@@ -13038,11 +13046,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F236" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G236" t="n">
-        <v>2020</v>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
@@ -13064,6 +13076,159 @@
       <c r="M236" t="inlineStr">
         <is>
           <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SWING Mistral 3 24 65-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A SWING Mistr</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/swing-mistral-3-24-65-95kg-no-sivs-no-flying-on-the-sand-6907/</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>190</v>
+      </c>
+      <c r="G237" t="n">
+        <v>2005</v>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr"/>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr"/>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Ozone Jomo S 65-85kg Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Ozo</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-jomo-s-65-85kg-lightened-no-sivs-no-flying-on-the--6905/</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr"/>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>mamekridla_cz</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Máme Křídla CZ</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS pluto 2 m Pluto 2 M 80-105kg</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>https://mamekridla.cz/kridlo-en-b-axis-pluto-2-m-pluto-2-m-80-105kg/722</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr"/>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="inlineStr"/>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -13078,7 +13243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M76"/>
+  <dimension ref="A1:M79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17209,11 +17374,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>700</v>
-      </c>
-      <c r="G74" t="n">
-        <v>2018</v>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -17264,11 +17433,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G75" t="n">
-        <v>2020</v>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -17319,11 +17492,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G76" t="n">
-        <v>2020</v>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -17345,6 +17522,159 @@
       <c r="M76" t="inlineStr">
         <is>
           <t>2026-05-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SWING Mistral 3 24 65-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A SWING Mistr</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/swing-mistral-3-24-65-95kg-no-sivs-no-flying-on-the-sand-6907/</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>190</v>
+      </c>
+      <c r="G77" t="n">
+        <v>2005</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Ozone Jomo S 65-85kg Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Ozo</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-jomo-s-65-85kg-lightened-no-sivs-no-flying-on-the--6905/</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>mamekridla_cz</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Máme Křídla CZ</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS pluto 2 m Pluto 2 M 80-105kg</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://mamekridla.cz/kridlo-en-b-axis-pluto-2-m-pluto-2-m-80-105kg/722</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -17372,7 +17702,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17447,12 +17777,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -17462,52 +17792,52 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 010</t>
+          <t>Křídlo EN A SWING Mistral 3 24 65-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A SWING Mistr</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/swing-mistral-3-24-65-95kg-no-sivs-no-flying-on-the-sand-6907/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>700</v>
+        <v>190</v>
       </c>
       <c r="G2" t="n">
-        <v>2018</v>
+        <v>2005</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -17517,52 +17847,50 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 300,16 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN A Ozone Jomo S 65-85kg Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Ozo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1000</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-jomo-s-65-85kg-lightened-no-sivs-no-flying-on-the--6905/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>mamekridla_cz</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Máme Křídla CZ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -17572,40 +17900,30 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 727,95 CZK (1 099,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN B AXIS pluto 2 m Pluto 2 M 80-105kg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1099</v>
-      </c>
+          <t>https://mamekridla.cz/kridlo-en-b-axis-pluto-2-m-pluto-2-m-80-105kg/722</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -17615,6 +17933,147 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mamekridla_cz</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Máme Křídla CZ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS pluto 2 m Pluto 2 M 80-105kg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://mamekridla.cz/kridlo-en-b-axis-pluto-2-m-pluto-2-m-80-105kg/722</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17708,210 +18167,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 300,16 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 727,95 CZK (1 099,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-17
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M239"/>
+  <dimension ref="A1:M242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13105,11 +13105,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/swing-mistral-3-24-65-95kg-no-sivs-no-flying-on-the-sand-6907/</t>
         </is>
       </c>
-      <c r="F237" t="n">
-        <v>190</v>
-      </c>
-      <c r="G237" t="n">
-        <v>2005</v>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>190.0</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
@@ -13161,8 +13165,10 @@
         </is>
       </c>
       <c r="F238" t="inlineStr"/>
-      <c r="G238" t="n">
-        <v>2018</v>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H238" t="inlineStr">
         <is>
@@ -13214,8 +13220,10 @@
         </is>
       </c>
       <c r="F239" t="inlineStr"/>
-      <c r="G239" t="n">
-        <v>2026</v>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
@@ -13229,6 +13237,167 @@
       <c r="M239" t="inlineStr">
         <is>
           <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nelétáno na písku Nevětveno Drobné opravy TK čerstvá TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-no-flying-on-the-sand-n-6912/</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>987</v>
+      </c>
+      <c r="G240" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr"/>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 744,21 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G241" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr"/>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr"/>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 251,28 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F242" t="n">
+        <v>750</v>
+      </c>
+      <c r="G242" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr"/>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr"/>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -13243,7 +13412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17551,11 +17720,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/swing-mistral-3-24-65-95kg-no-sivs-no-flying-on-the-sand-6907/</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>190</v>
-      </c>
-      <c r="G77" t="n">
-        <v>2005</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>190.0</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -17607,8 +17780,10 @@
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
-      <c r="G78" t="n">
-        <v>2018</v>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -17660,8 +17835,10 @@
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
-      <c r="G79" t="n">
-        <v>2026</v>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -17675,6 +17852,167 @@
       <c r="M79" t="inlineStr">
         <is>
           <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nelétáno na písku Nevětveno Drobné opravy TK čerstvá TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-no-flying-on-the-sand-n-6912/</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>987</v>
+      </c>
+      <c r="G80" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 744,21 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G81" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 251,28 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>750</v>
+      </c>
+      <c r="G82" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -17702,7 +18040,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17777,12 +18115,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -17792,40 +18130,40 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A SWING Mistral 3 24 65-95kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A SWING Mistr</t>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nelétáno na písku Nevětveno Drobné opravy TK čerstvá TK platná Křídlo EN B BG</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/swing-mistral-3-24-65-95kg-no-sivs-no-flying-on-the-sand-6907/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-no-flying-on-the-sand-n-6912/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>190</v>
+        <v>987</v>
       </c>
       <c r="G2" t="n">
-        <v>2005</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Olétané (více než 300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -17847,17 +18185,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Ozone Jomo S 65-85kg Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Ozo</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 744,21 CZK (1 099,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-jomo-s-65-85kg-lightened-no-sivs-no-flying-on-the--6905/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1099</v>
+      </c>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -17866,7 +18206,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -17878,19 +18218,19 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mamekridla_cz</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Máme Křídla CZ</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -17900,30 +18240,36 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS pluto 2 m Pluto 2 M 80-105kg</t>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 251,28 CZK (750,00 EUR) E</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://mamekridla.cz/kridlo-en-b-axis-pluto-2-m-pluto-2-m-80-105kg/722</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>750</v>
+      </c>
       <c r="G4" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -17941,17 +18287,17 @@
   <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18026,12 +18372,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mamekridla_cz</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Máme Křídla CZ</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18041,30 +18387,36 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS pluto 2 m Pluto 2 M 80-105kg</t>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 251,28 CZK (750,00 EUR) E</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://mamekridla.cz/kridlo-en-b-axis-pluto-2-m-pluto-2-m-80-105kg/722</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>750</v>
+      </c>
       <c r="G2" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -18079,20 +18431,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18164,6 +18516,61 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 744,21 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-18
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M242"/>
+  <dimension ref="A1:M247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13266,11 +13266,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-no-flying-on-the-sand-n-6912/</t>
         </is>
       </c>
-      <c r="F240" t="n">
-        <v>987</v>
-      </c>
-      <c r="G240" t="n">
-        <v>2020</v>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>987.0</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
@@ -13321,11 +13325,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F241" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G241" t="n">
-        <v>2020</v>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
@@ -13376,11 +13384,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F242" t="n">
-        <v>750</v>
-      </c>
-      <c r="G242" t="n">
-        <v>2023</v>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
@@ -13398,6 +13410,269 @@
       <c r="M242" t="inlineStr">
         <is>
           <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr"/>
+      <c r="G243" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr"/>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr"/>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr"/>
+      <c r="G244" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr"/>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr"/>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 SM 60-85kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN B AXIS Pluto 3 S</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-sm-60-85kg-no-sivs-no-flying-on-the-sand-no-6916/</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G245" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr"/>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr"/>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Fides 1 80-110kg Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN A SKY Fides 1 80-110kg Žádné</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-fides-1-80-110kg-no-sivs-no-flying-on-the-sand-no-wa-6926/</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr"/>
+      <c r="G246" t="n">
+        <v>2004</v>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr"/>
+      <c r="J246" t="inlineStr"/>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr"/>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Golden 2 L 90-115kg TK není Nekoupáno Drobné opravy Křídlo EN A Gradient Golden 2 L 90-115kg TK nen</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-2-l-90-115kg-no-tc-no-water-small-repair-6923/</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr"/>
+      <c r="G247" t="n">
+        <v>2008</v>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr"/>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr"/>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -13412,7 +13687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17881,11 +18156,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-no-flying-on-the-sand-n-6912/</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>987</v>
-      </c>
-      <c r="G80" t="n">
-        <v>2020</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>987.0</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -17936,11 +18215,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G81" t="n">
-        <v>2020</v>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -17991,11 +18274,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>750</v>
-      </c>
-      <c r="G82" t="n">
-        <v>2023</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -18013,6 +18300,269 @@
       <c r="M82" t="inlineStr">
         <is>
           <t>2026-05-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 SM 60-85kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN B AXIS Pluto 3 S</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-sm-60-85kg-no-sivs-no-flying-on-the-sand-no-6916/</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G85" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Fides 1 80-110kg Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN A SKY Fides 1 80-110kg Žádné</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-fides-1-80-110kg-no-sivs-no-flying-on-the-sand-no-wa-6926/</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="n">
+        <v>2004</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Golden 2 L 90-115kg TK není Nekoupáno Drobné opravy Křídlo EN A Gradient Golden 2 L 90-115kg TK nen</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-2-l-90-115kg-no-tc-no-water-small-repair-6923/</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="n">
+        <v>2008</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -18027,7 +18577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18130,19 +18680,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nelétáno na písku Nevětveno Drobné opravy TK čerstvá TK platná Křídlo EN B BG</t>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-no-flying-on-the-sand-n-6912/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>987</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -18151,31 +18699,31 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Olétané (více než 300h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18185,52 +18733,50 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 744,21 CZK (1 099,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B AXI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1099</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -18240,36 +18786,142 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 251,28 CZK (750,00 EUR) E</t>
+          <t>Křídlo EN B AXIS Pluto 3 SM 60-85kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN B AXIS Pluto 3 S</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-sm-60-85kg-no-sivs-no-flying-on-the-sand-no-6916/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>750</v>
+        <v>1350</v>
       </c>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2017</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Fides 1 80-110kg Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN A SKY Fides 1 80-110kg Žádné</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-fides-1-80-110kg-no-sivs-no-flying-on-the-sand-no-wa-6926/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2004</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Golden 2 L 90-115kg TK není Nekoupáno Drobné opravy Křídlo EN A Gradient Golden 2 L 90-115kg TK nen</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-2-l-90-115kg-no-tc-no-water-small-repair-6923/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2008</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -18297,7 +18949,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18372,12 +19024,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18387,36 +19039,38 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 251,28 CZK (750,00 EUR) E</t>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>750</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -18519,12 +19173,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18534,28 +19188,26 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 744,21 CZK (1 099,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1099</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -18567,7 +19219,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-19
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M247"/>
+  <dimension ref="A1:M249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13440,8 +13440,10 @@
         </is>
       </c>
       <c r="F243" t="inlineStr"/>
-      <c r="G243" t="n">
-        <v>2023</v>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
@@ -13493,8 +13495,10 @@
         </is>
       </c>
       <c r="F244" t="inlineStr"/>
-      <c r="G244" t="n">
-        <v>2022</v>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
@@ -13545,11 +13549,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-sm-60-85kg-no-sivs-no-flying-on-the-sand-no-6916/</t>
         </is>
       </c>
-      <c r="F245" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G245" t="n">
-        <v>2017</v>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>1350.0</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
@@ -13601,8 +13609,10 @@
         </is>
       </c>
       <c r="F246" t="inlineStr"/>
-      <c r="G246" t="n">
-        <v>2004</v>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
@@ -13650,8 +13660,10 @@
         </is>
       </c>
       <c r="F247" t="inlineStr"/>
-      <c r="G247" t="n">
-        <v>2008</v>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
@@ -13673,6 +13685,110 @@
       <c r="M247" t="inlineStr">
         <is>
           <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
+        </is>
+      </c>
+      <c r="F248" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G248" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr"/>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr"/>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Ascent 3 90-135kg Drobné opravy TK platná (Součást kompletu) Křídlo EN A UP Ascent 3 90-135kg Drobné opra</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-ascent-3-90-135kg-small-repairs-tc-valid-6932/</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr"/>
+      <c r="J249" t="inlineStr"/>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr"/>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -13687,7 +13803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18330,8 +18446,10 @@
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" t="n">
-        <v>2023</v>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -18383,8 +18501,10 @@
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="n">
-        <v>2022</v>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -18435,11 +18555,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-sm-60-85kg-no-sivs-no-flying-on-the-sand-no-6916/</t>
         </is>
       </c>
-      <c r="F85" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G85" t="n">
-        <v>2017</v>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>1350.0</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -18491,8 +18615,10 @@
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="n">
-        <v>2004</v>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -18540,8 +18666,10 @@
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="n">
-        <v>2008</v>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -18563,6 +18691,110 @@
       <c r="M87" t="inlineStr">
         <is>
           <t>2026-05-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G88" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Ascent 3 90-135kg Drobné opravy TK platná (Součást kompletu) Křídlo EN A UP Ascent 3 90-135kg Drobné opra</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-ascent-3-90-135kg-small-repairs-tc-valid-6932/</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -18577,7 +18809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18590,7 +18822,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18680,17 +18912,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -18699,31 +18933,31 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18733,195 +18967,34 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN B AXI</t>
+          <t>Křídlo EN A UP Ascent 3 90-135kg Drobné opravy TK platná (Součást kompletu) Křídlo EN A UP Ascent 3 90-135kg Drobné opra</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-ascent-3-90-135kg-small-repairs-tc-valid-6932/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Pluto 3 SM 60-85kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN B AXIS Pluto 3 S</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-sm-60-85kg-no-sivs-no-flying-on-the-sand-no-6916/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2017</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>SM</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SKY Fides 1 80-110kg Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN A SKY Fides 1 80-110kg Žádné</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-fides-1-80-110kg-no-sivs-no-flying-on-the-sand-no-wa-6926/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2004</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Gradient Golden 2 L 90-115kg TK není Nekoupáno Drobné opravy Křídlo EN A Gradient Golden 2 L 90-115kg TK nen</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-2-l-90-115kg-no-tc-no-water-small-repair-6923/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
-        <v>2008</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Olétané (více než 300h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -19039,17 +19112,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -19058,19 +19133,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -19188,17 +19263,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Iota DLS 25 80-100kg Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN B Advance Iota DLS</t>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-25-80-100kg-concertinas-lightened-no-tr-6927/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -19207,19 +19284,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-20
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M249"/>
+  <dimension ref="A1:M256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13714,11 +13714,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
         </is>
       </c>
-      <c r="F248" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G248" t="n">
-        <v>2022</v>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
@@ -13770,8 +13774,10 @@
         </is>
       </c>
       <c r="F249" t="inlineStr"/>
-      <c r="G249" t="n">
-        <v>2017</v>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
@@ -13789,6 +13795,377 @@
       <c r="M249" t="inlineStr">
         <is>
           <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné SIV TK čerstvá Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-sivs-tc-fresh-6946/</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr"/>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 027</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F251" t="n">
+        <v>700</v>
+      </c>
+      <c r="G251" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr"/>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 294,84 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F252" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G252" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr"/>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 583,29 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F253" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G253" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr"/>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr"/>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 552,61 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F254" t="n">
+        <v>599</v>
+      </c>
+      <c r="G254" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr"/>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr"/>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 733,15 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F255" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G255" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr"/>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 221,13 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F256" t="n">
+        <v>750</v>
+      </c>
+      <c r="G256" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr"/>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr"/>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -13803,7 +14180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18720,11 +19097,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G88" t="n">
-        <v>2022</v>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -18776,8 +19157,10 @@
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" t="n">
-        <v>2017</v>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -18795,6 +19178,377 @@
       <c r="M89" t="inlineStr">
         <is>
           <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné SIV TK čerstvá Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-sivs-tc-fresh-6946/</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 027</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>700</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 294,84 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G92" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 583,29 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G93" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 552,61 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>599</v>
+      </c>
+      <c r="G94" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 733,15 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G95" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 221,13 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>750</v>
+      </c>
+      <c r="G96" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -18804,6 +19558,569 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné SIV TK čerstvá Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-sivs-tc-fresh-6946/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 027</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>700</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 294,84 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 583,29 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 552,61 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>599</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 733,15 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 221,13 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>750</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18912,19 +20229,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 294,84 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -18945,7 +20262,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -18967,24 +20284,30 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Ascent 3 90-135kg Drobné opravy TK platná (Součást kompletu) Křídlo EN A UP Ascent 3 90-135kg Drobné opra</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 733,15 CZK (1 099,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-ascent-3-90-135kg-small-repairs-tc-valid-6932/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1099</v>
+      </c>
       <c r="G3" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
@@ -18994,309 +20317,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím obalem Křídlo EN B BGD Base 2 M 75-95kg Odlehčeno S listovacím o</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-lightened-with-listing-bag-6931/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-21
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M256"/>
+  <dimension ref="A1:M262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -13825,8 +13825,10 @@
         </is>
       </c>
       <c r="F250" t="inlineStr"/>
-      <c r="G250" t="n">
-        <v>2019</v>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
@@ -13877,11 +13879,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F251" t="n">
-        <v>700</v>
-      </c>
-      <c r="G251" t="n">
-        <v>2018</v>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
@@ -13932,11 +13938,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F252" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G252" t="n">
-        <v>2020</v>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
@@ -13987,11 +13997,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F253" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G253" t="n">
-        <v>2023</v>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
@@ -14038,11 +14052,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F254" t="n">
-        <v>599</v>
-      </c>
-      <c r="G254" t="n">
-        <v>2015</v>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
@@ -14089,11 +14107,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F255" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G255" t="n">
-        <v>2020</v>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
@@ -14144,11 +14166,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F256" t="n">
-        <v>750</v>
-      </c>
-      <c r="G256" t="n">
-        <v>2023</v>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
@@ -14166,6 +14192,322 @@
       <c r="M256" t="inlineStr">
         <is>
           <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 4 M 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné oprav Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-m-90-110kg-concertinas-no-sivs-no-flying-o-6955/</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr"/>
+      <c r="G257" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr"/>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 324,98 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F258" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G258" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr"/>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 622,48 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F259" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G259" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr"/>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr"/>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 570,66 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F260" t="n">
+        <v>599</v>
+      </c>
+      <c r="G260" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr"/>
+      <c r="J260" t="inlineStr"/>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr"/>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 243,74 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>750</v>
+      </c>
+      <c r="G261" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr"/>
+      <c r="J261" t="inlineStr"/>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr"/>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 082,46 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G262" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr"/>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr"/>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -14180,7 +14522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19208,8 +19550,10 @@
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" t="n">
-        <v>2019</v>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -19260,11 +19604,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>700</v>
-      </c>
-      <c r="G91" t="n">
-        <v>2018</v>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -19315,11 +19663,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G92" t="n">
-        <v>2020</v>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -19370,11 +19722,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G93" t="n">
-        <v>2023</v>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -19421,11 +19777,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F94" t="n">
-        <v>599</v>
-      </c>
-      <c r="G94" t="n">
-        <v>2015</v>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -19472,11 +19832,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G95" t="n">
-        <v>2020</v>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -19527,11 +19891,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F96" t="n">
-        <v>750</v>
-      </c>
-      <c r="G96" t="n">
-        <v>2023</v>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -19549,6 +19917,322 @@
       <c r="M96" t="inlineStr">
         <is>
           <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 4 M 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné oprav Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-m-90-110kg-concertinas-no-sivs-no-flying-o-6955/</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 324,98 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G98" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 622,48 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G99" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 570,66 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>599</v>
+      </c>
+      <c r="G100" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 243,74 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>750</v>
+      </c>
+      <c r="G101" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 082,46 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G102" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -19563,7 +20247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19666,17 +20350,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné SIV TK čerstvá Křídlo EN B Sky Country DISCOVERY 5 M 80-100kg Žádné</t>
+          <t>Křídlo EN B Nova Mentor 4 M 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné oprav Křídlo EN B</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-country-discovery-5-m-80-100kg-no-sivs-tc-fresh-6946/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-m-90-110kg-concertinas-no-sivs-no-flying-o-6955/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -19697,7 +20381,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -19719,19 +20403,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 027</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 324,98 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -19746,13 +20430,13 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -19774,30 +20458,26 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 294,84 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 622,48 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1000</v>
+        <v>1300</v>
       </c>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
@@ -19807,7 +20487,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -19829,19 +20509,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 583,29 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 570,66 CZK (599,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1300</v>
+        <v>599</v>
       </c>
       <c r="G5" t="n">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -19858,19 +20538,19 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -19880,36 +20560,36 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 552,61 CZK (599,00</t>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 243,74 CZK (750,00 EUR) E</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>599</v>
+        <v>750</v>
       </c>
       <c r="G6" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -19931,19 +20611,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 733,15 CZK (1 099,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 082,46 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1099</v>
+        <v>2100</v>
       </c>
       <c r="G7" t="n">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -19952,70 +20632,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 221,13 CZK (750,00 EUR) E</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>750</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -20030,103 +20659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20214,6 +20747,157 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 082,46 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
@@ -20229,7 +20913,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 294,84 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 324,98 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -20262,62 +20946,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 733,15 CZK (1 099,00 EUR) EN A Veliko</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-22
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M262"/>
+  <dimension ref="A1:M265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14222,8 +14222,10 @@
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
-      <c r="G257" t="n">
-        <v>2018</v>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
@@ -14274,11 +14276,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F258" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G258" t="n">
-        <v>2020</v>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
@@ -14329,11 +14335,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F259" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G259" t="n">
-        <v>2023</v>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
@@ -14380,11 +14390,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F260" t="n">
-        <v>599</v>
-      </c>
-      <c r="G260" t="n">
-        <v>2015</v>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
@@ -14431,11 +14445,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F261" t="n">
-        <v>750</v>
-      </c>
-      <c r="G261" t="n">
-        <v>2023</v>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
@@ -14482,11 +14500,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F262" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G262" t="n">
-        <v>2026</v>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
@@ -14508,6 +14530,171 @@
       <c r="M262" t="inlineStr">
         <is>
           <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 006</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>700</v>
+      </c>
+      <c r="G263" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr"/>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr"/>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 700,03 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G264" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr"/>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr"/>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 019,17 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G265" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr"/>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -14522,7 +14709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M102"/>
+  <dimension ref="A1:M105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19947,8 +20134,10 @@
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
-      <c r="G97" t="n">
-        <v>2018</v>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -19999,11 +20188,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F98" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G98" t="n">
-        <v>2020</v>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -20054,11 +20247,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F99" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G99" t="n">
-        <v>2023</v>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -20105,11 +20302,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F100" t="n">
-        <v>599</v>
-      </c>
-      <c r="G100" t="n">
-        <v>2015</v>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -20156,11 +20357,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F101" t="n">
-        <v>750</v>
-      </c>
-      <c r="G101" t="n">
-        <v>2023</v>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -20207,11 +20412,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F102" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G102" t="n">
-        <v>2026</v>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -20233,6 +20442,171 @@
       <c r="M102" t="inlineStr">
         <is>
           <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 006</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>700</v>
+      </c>
+      <c r="G103" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 700,03 CZK (1 099,00 EUR) EN A Veliko</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1099</v>
+      </c>
+      <c r="G104" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 019,17 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G105" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -20247,7 +20621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20350,15 +20724,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 4 M 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné oprav Křídlo EN B</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 006</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-m-90-110kg-concertinas-no-sivs-no-flying-o-6955/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>700</v>
+      </c>
       <c r="G2" t="n">
         <v>2018</v>
       </c>
@@ -20375,25 +20751,25 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20403,52 +20779,52 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 324,98 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 700,03 CZK (1 099,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1000</v>
+        <v>1099</v>
       </c>
       <c r="G3" t="n">
         <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -20458,26 +20834,30 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 622,48 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 019,17 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1300</v>
+        <v>2100</v>
       </c>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
@@ -20487,164 +20867,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 570,66 CZK (599,00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>599</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 243,74 CZK (750,00 EUR) E</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>750</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 082,46 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -20762,7 +20985,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 082,46 CZK (2 100,00</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 019,17 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -20795,7 +21018,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -20898,12 +21121,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -20913,40 +21136,40 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 324,98 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 700,03 CZK (1 099,00 EUR) EN A Veliko</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1000</v>
+        <v>1099</v>
       </c>
       <c r="G2" t="n">
         <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-23
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M265"/>
+  <dimension ref="A1:M267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14559,11 +14559,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F263" t="n">
-        <v>700</v>
-      </c>
-      <c r="G263" t="n">
-        <v>2018</v>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
@@ -14614,11 +14618,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F264" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G264" t="n">
-        <v>2020</v>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
@@ -14669,11 +14677,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F265" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G265" t="n">
-        <v>2026</v>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
@@ -14695,6 +14707,114 @@
       <c r="M265" t="inlineStr">
         <is>
           <t>2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr"/>
+      <c r="G266" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr"/>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 300,66 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>999</v>
+      </c>
+      <c r="G267" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr"/>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -14709,7 +14829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M105"/>
+  <dimension ref="A1:M107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20471,11 +20591,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F103" t="n">
-        <v>700</v>
-      </c>
-      <c r="G103" t="n">
-        <v>2018</v>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -20526,11 +20650,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
         </is>
       </c>
-      <c r="F104" t="n">
-        <v>1099</v>
-      </c>
-      <c r="G104" t="n">
-        <v>2020</v>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>1099.0</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -20581,11 +20709,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F105" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G105" t="n">
-        <v>2026</v>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -20607,6 +20739,114 @@
       <c r="M105" t="inlineStr">
         <is>
           <t>2026-05-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 300,66 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>999</v>
+      </c>
+      <c r="G107" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -20621,7 +20861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20634,7 +20874,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -20724,19 +20964,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 17 006</t>
+          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -20745,19 +20983,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -20779,16 +21017,16 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 700,03 CZK (1 099,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 300,66 CZK (999,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1099</v>
+        <v>999</v>
       </c>
       <c r="G3" t="n">
         <v>2020</v>
@@ -20812,62 +21050,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 019,17 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -20970,12 +21153,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -20985,28 +21168,26 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 51 019,17 CZK (2 100,00</t>
+          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2100</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -21018,7 +21199,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -21033,7 +21214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21121,12 +21302,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21136,40 +21317,93 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 26 700,03 CZK (1 099,00 EUR) EN A Veliko</t>
+          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6899/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1099</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 300,66 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>999</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-24
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M267"/>
+  <dimension ref="A1:M270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14737,8 +14737,10 @@
         </is>
       </c>
       <c r="F266" t="inlineStr"/>
-      <c r="G266" t="n">
-        <v>2022</v>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
@@ -14789,11 +14791,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
         </is>
       </c>
-      <c r="F267" t="n">
-        <v>999</v>
-      </c>
-      <c r="G267" t="n">
-        <v>2020</v>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>999.0</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
@@ -14815,6 +14821,169 @@
       <c r="M267" t="inlineStr">
         <is>
           <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný TK platná S listovacím obalem (Součást kompletu) Křídlo EN B AXIS Pluto 3</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-tc-valid-with-listi-6970/</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr"/>
+      <c r="G268" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr"/>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 996</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>700</v>
+      </c>
+      <c r="G269" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr"/>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr"/>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 280,10 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G270" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr"/>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -14829,7 +14998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M107"/>
+  <dimension ref="A1:M110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20769,8 +20938,10 @@
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
-      <c r="G106" t="n">
-        <v>2022</v>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -20821,11 +20992,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
         </is>
       </c>
-      <c r="F107" t="n">
-        <v>999</v>
-      </c>
-      <c r="G107" t="n">
-        <v>2020</v>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>999.0</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -20847,6 +21022,169 @@
       <c r="M107" t="inlineStr">
         <is>
           <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný TK platná S listovacím obalem (Součást kompletu) Křídlo EN B AXIS Pluto 3</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-tc-valid-with-listi-6970/</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 996</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>700</v>
+      </c>
+      <c r="G109" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 280,10 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G110" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -20861,7 +21199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20874,7 +21212,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -20964,17 +21302,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
+          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný TK platná S listovacím obalem (Součást kompletu) Křídlo EN B AXIS Pluto 3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-tc-valid-with-listi-6970/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -20983,31 +21321,31 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21017,40 +21355,95 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 300,66 CZK (999,00 EUR) EN A Velikost</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 996</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>999</v>
+        <v>700</v>
       </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 280,10 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -21060,6 +21453,102 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21168,17 +21657,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 280,10 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -21187,7 +21678,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -21199,211 +21690,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoupáno Křídlo EN B BGD Epic S 60-100kg Žádné SIV Nevětveno Nekoup</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-no-sivs-no-trees-no-water-6969/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 300,66 CZK (999,00 EUR) EN A Velikost</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-6962/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>999</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-25
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M270"/>
+  <dimension ref="A1:M275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -14851,8 +14851,10 @@
         </is>
       </c>
       <c r="F268" t="inlineStr"/>
-      <c r="G268" t="n">
-        <v>2016</v>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
@@ -14903,11 +14905,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F269" t="n">
-        <v>700</v>
-      </c>
-      <c r="G269" t="n">
-        <v>2018</v>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
@@ -14958,11 +14964,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F270" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G270" t="n">
-        <v>2020</v>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H270" t="inlineStr">
         <is>
@@ -14984,6 +14994,267 @@
       <c r="M270" t="inlineStr">
         <is>
           <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota 60-85kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN B Advance Iota 60-</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-60-85kg-concertinas-no-sivs-no-flying-on-th-6982/</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr"/>
+      <c r="G271" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr"/>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr"/>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 552,61 CZK (5</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>599</v>
+      </c>
+      <c r="G272" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr"/>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M 80-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-80-105kg-concertinas-no-sivs-no-flying-on-6976/</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr"/>
+      <c r="G273" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr"/>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 564,12 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G274" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr"/>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr"/>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá Křídlo EN A UP MANA 27 80-110kg Listova</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr"/>
+      <c r="G275" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr"/>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr"/>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -14998,7 +15269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M110"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21052,8 +21323,10 @@
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
-      <c r="G108" t="n">
-        <v>2016</v>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -21104,11 +21377,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F109" t="n">
-        <v>700</v>
-      </c>
-      <c r="G109" t="n">
-        <v>2018</v>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -21159,11 +21436,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F110" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G110" t="n">
-        <v>2020</v>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -21185,6 +21466,267 @@
       <c r="M110" t="inlineStr">
         <is>
           <t>2026-05-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota 60-85kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN B Advance Iota 60-</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-60-85kg-concertinas-no-sivs-no-flying-on-th-6982/</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 552,61 CZK (5</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>599</v>
+      </c>
+      <c r="G112" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M 80-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-80-105kg-concertinas-no-sivs-no-flying-on-6976/</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 564,12 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G114" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá Křídlo EN A UP MANA 27 80-110kg Listova</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -21199,7 +21741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21302,38 +21844,34 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný TK platná S listovacím obalem (Součást kompletu) Křídlo EN B AXIS Pluto 3</t>
+          <t>Křídlo EN B Advance Iota 60-85kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN B Advance Iota 60-</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-tc-valid-with-listi-6970/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-60-85kg-concertinas-no-sivs-no-flying-on-th-6982/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -21355,19 +21893,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 996</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 552,61 CZK (5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>700</v>
+        <v>599</v>
       </c>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -21376,7 +21914,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -21388,7 +21926,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -21410,19 +21948,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 280,10 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M 80-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1000</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-80-105kg-concertinas-no-sivs-no-flying-on-6976/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -21437,13 +21973,117 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 564,12 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá Křídlo EN A UP MANA 27 80-110kg Listova</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -21554,20 +22194,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -21639,61 +22279,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 280,10 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-24</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-27
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M275"/>
+  <dimension ref="A1:M280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -15024,8 +15024,10 @@
         </is>
       </c>
       <c r="F271" t="inlineStr"/>
-      <c r="G271" t="n">
-        <v>2015</v>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
@@ -15072,11 +15074,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F272" t="n">
-        <v>599</v>
-      </c>
-      <c r="G272" t="n">
-        <v>2017</v>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
@@ -15128,8 +15134,10 @@
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
-      <c r="G273" t="n">
-        <v>2017</v>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
@@ -15180,11 +15188,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F274" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G274" t="n">
-        <v>2023</v>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
@@ -15232,8 +15244,10 @@
         </is>
       </c>
       <c r="F275" t="inlineStr"/>
-      <c r="G275" t="n">
-        <v>2020</v>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
@@ -15255,6 +15269,265 @@
       <c r="M275" t="inlineStr">
         <is>
           <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden 7 100-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B MA</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-100-130kg-concertinas-lightened-new-no-sivs-n-6993/</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr"/>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr"/>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr"/>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--6991/</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr"/>
+      <c r="G277" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr"/>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr"/>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 531,78 CZK (5</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>599</v>
+      </c>
+      <c r="G278" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr"/>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr"/>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-90-115kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr"/>
+      <c r="G279" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr"/>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr"/>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 543,78 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>599</v>
+      </c>
+      <c r="G280" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr"/>
+      <c r="J280" t="inlineStr"/>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr"/>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -15269,7 +15542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M115"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21496,8 +21769,10 @@
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
-      <c r="G111" t="n">
-        <v>2015</v>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -21544,11 +21819,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F112" t="n">
-        <v>599</v>
-      </c>
-      <c r="G112" t="n">
-        <v>2017</v>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -21600,8 +21879,10 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" t="n">
-        <v>2017</v>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -21652,11 +21933,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
         </is>
       </c>
-      <c r="F114" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G114" t="n">
-        <v>2023</v>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -21704,8 +21989,10 @@
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
-      <c r="G115" t="n">
-        <v>2020</v>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -21727,6 +22014,265 @@
       <c r="M115" t="inlineStr">
         <is>
           <t>2026-05-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden 7 100-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B MA</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-100-130kg-concertinas-lightened-new-no-sivs-n-6993/</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--6991/</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 531,78 CZK (5</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>599</v>
+      </c>
+      <c r="G118" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-90-115kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 543,78 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>599</v>
+      </c>
+      <c r="G120" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -21750,6 +22296,361 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden 7 100-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B MA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-100-130kg-concertinas-lightened-new-no-sivs-n-6993/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--6991/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 531,78 CZK (5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>599</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 28 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-90-115kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 543,78 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>599</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
@@ -21844,34 +22745,38 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Iota 60-85kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN B Advance Iota 60-</t>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-60-85kg-concertinas-no-sivs-no-flying-on-th-6982/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--6991/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -21893,19 +22798,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 552,61 CZK (5</t>
+          <t>Křídlo EN B Advance Epsilon DLS 28 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>599</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-90-115kg-no-sivs-no-flying-on-the-6848/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2017</v>
+        <v>2025</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -21914,272 +22817,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M 80-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B AXI</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-80-105kg-concertinas-no-sivs-no-flying-on-6976/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2017</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 564,12 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá Křídlo EN A UP MANA 27 80-110kg Listova</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-28
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M280"/>
+  <dimension ref="A1:M286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -15346,8 +15346,10 @@
         </is>
       </c>
       <c r="F277" t="inlineStr"/>
-      <c r="G277" t="n">
-        <v>2023</v>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
@@ -15398,11 +15400,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F278" t="n">
-        <v>599</v>
-      </c>
-      <c r="G278" t="n">
-        <v>2017</v>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
@@ -15454,8 +15460,10 @@
         </is>
       </c>
       <c r="F279" t="inlineStr"/>
-      <c r="G279" t="n">
-        <v>2025</v>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
@@ -15506,11 +15514,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F280" t="n">
-        <v>599</v>
-      </c>
-      <c r="G280" t="n">
-        <v>2015</v>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
@@ -15528,6 +15540,324 @@
       <c r="M280" t="inlineStr">
         <is>
           <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G281" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr"/>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Nelétáno na písku Nevětveno Nekoupáno TK platná S listovacím obale Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G282" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr"/>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 62</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr"/>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B AirD</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-85-105kg-concertinas-lightened-no-sivs-no-6991/</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr"/>
+      <c r="G284" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr"/>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr"/>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 210,07 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>750</v>
+      </c>
+      <c r="G285" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr"/>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr"/>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 988,20 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G286" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr"/>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -15542,7 +15872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M120"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -22091,8 +22421,10 @@
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
-      <c r="G117" t="n">
-        <v>2023</v>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -22143,11 +22475,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F118" t="n">
-        <v>599</v>
-      </c>
-      <c r="G118" t="n">
-        <v>2017</v>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -22199,8 +22535,10 @@
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
-      <c r="G119" t="n">
-        <v>2025</v>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -22251,11 +22589,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F120" t="n">
-        <v>599</v>
-      </c>
-      <c r="G120" t="n">
-        <v>2015</v>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -22273,6 +22615,324 @@
       <c r="M120" t="inlineStr">
         <is>
           <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G121" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Nelétáno na písku Nevětveno Nekoupáno TK platná S listovacím obale Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G122" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 62</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B AirD</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-85-105kg-concertinas-lightened-no-sivs-no-6991/</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 210,07 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>750</v>
+      </c>
+      <c r="G125" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 988,20 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G126" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -22287,7 +22947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -22296,7 +22956,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -22390,22 +23050,30 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Eden 7 100-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B MA</t>
+          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-100-130kg-concertinas-lightened-new-no-sivs-n-6993/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
@@ -22415,7 +23083,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -22437,17 +23105,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Nelétáno na písku Nevětveno Nekoupáno TK platná S listovacím obale Křídlo EN B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--6991/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1600</v>
+      </c>
       <c r="G3" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -22456,19 +23126,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -22490,19 +23160,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 531,78 CZK (5</t>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 62</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>599</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -22511,19 +23179,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>xs</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -22545,50 +23213,46 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 28 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+          <t>Křídlo EN B AirDesign soar 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B AirD</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-90-115kg-no-sivs-no-flying-on-the-6848/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-85-105kg-concertinas-lightened-no-sivs-no-6991/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -22598,36 +23262,91 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 543,78 CZK (599,00</t>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 210,07 CZK (750,00 EUR) E</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>599</v>
+        <v>750</v>
       </c>
       <c r="G6" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 988,20 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -22655,7 +23374,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -22745,17 +23464,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--6991/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1300</v>
+      </c>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -22764,31 +23485,31 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -22798,26 +23519,28 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 28 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advanc</t>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 988,20 CZK (2 100,00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-28-90-115kg-no-sivs-no-flying-on-the-6848/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2100</v>
+      </c>
       <c r="G3" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -22829,7 +23552,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -22844,20 +23567,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -22929,6 +23652,116 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Nelétáno na písku Nevětveno Nekoupáno TK platná S listovacím obale Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-29
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M286"/>
+  <dimension ref="A1:M290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -15569,11 +15569,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
         </is>
       </c>
-      <c r="F281" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G281" t="n">
-        <v>2022</v>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
@@ -15624,11 +15628,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
         </is>
       </c>
-      <c r="F282" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G282" t="n">
-        <v>2020</v>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
@@ -15680,8 +15688,10 @@
         </is>
       </c>
       <c r="F283" t="inlineStr"/>
-      <c r="G283" t="n">
-        <v>2021</v>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
@@ -15733,8 +15743,10 @@
         </is>
       </c>
       <c r="F284" t="inlineStr"/>
-      <c r="G284" t="n">
-        <v>2023</v>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
@@ -15781,11 +15793,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F285" t="n">
-        <v>750</v>
-      </c>
-      <c r="G285" t="n">
-        <v>2023</v>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
@@ -15832,11 +15848,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F286" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G286" t="n">
-        <v>2026</v>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H286" t="inlineStr">
         <is>
@@ -15858,6 +15878,220 @@
       <c r="M286" t="inlineStr">
         <is>
           <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Calypso L 95-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B GIN C</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-calypso-l-95-115kg-concertinas-no-sivs-no-flying-on--7006/</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr"/>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 543,78 CZK (5</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>599</v>
+      </c>
+      <c r="G288" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr"/>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 982</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>700</v>
+      </c>
+      <c r="G289" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr"/>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 531,78 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>599</v>
+      </c>
+      <c r="G290" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr"/>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr"/>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -15872,7 +16106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -22644,11 +22878,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
         </is>
       </c>
-      <c r="F121" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G121" t="n">
-        <v>2022</v>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -22699,11 +22937,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
         </is>
       </c>
-      <c r="F122" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G122" t="n">
-        <v>2020</v>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -22755,8 +22997,10 @@
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
-      <c r="G123" t="n">
-        <v>2021</v>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -22808,8 +23052,10 @@
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
-      <c r="G124" t="n">
-        <v>2023</v>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -22856,11 +23102,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F125" t="n">
-        <v>750</v>
-      </c>
-      <c r="G125" t="n">
-        <v>2023</v>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -22907,11 +23157,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
         </is>
       </c>
-      <c r="F126" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G126" t="n">
-        <v>2026</v>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -22933,6 +23187,220 @@
       <c r="M126" t="inlineStr">
         <is>
           <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Calypso L 95-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B GIN C</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-calypso-l-95-115kg-concertinas-no-sivs-no-flying-on--7006/</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 543,78 CZK (5</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>599</v>
+      </c>
+      <c r="G128" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 982</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>700</v>
+      </c>
+      <c r="G129" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 531,78 CZK (599,00</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>599</v>
+      </c>
+      <c r="G130" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -22947,7 +23415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -23050,19 +23518,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
+          <t>Křídlo EN B GIN Calypso L 95-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B GIN C</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1300</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-calypso-l-95-115kg-concertinas-no-sivs-no-flying-on--7006/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -23071,19 +23537,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -23105,19 +23571,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Nelétáno na písku Nevětveno Nekoupáno TK platná S listovacím obale Křídlo EN B</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 543,78 CZK (5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1600</v>
+        <v>599</v>
       </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -23126,19 +23592,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -23160,17 +23626,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 62</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 982</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>700</v>
+      </c>
       <c r="G4" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -23179,19 +23647,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>xs</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -23213,17 +23681,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B AirDesign soar 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B AirD</t>
+          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 531,78 CZK (599,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-85-105kg-concertinas-lightened-no-sivs-no-6991/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>599</v>
+      </c>
       <c r="G5" t="n">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -23234,119 +23704,13 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 210,07 CZK (750,00 EUR) E</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>750</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 988,20 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -23361,20 +23725,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -23443,116 +23807,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 988,20 CZK (2 100,00</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -23567,20 +23821,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -23652,116 +23906,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B BGD Epic S 60-100kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B BGD Epic S</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-epic-s-60-100kg-concertinas-no-sivs-no-tc-no-flying--7000/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Nelétáno na písku Nevětveno Nekoupáno TK platná S listovacím obale Křídlo EN B</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-flying-on-the-sand-no-tr-6999/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-30
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M290"/>
+  <dimension ref="A1:M292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -15908,8 +15908,10 @@
         </is>
       </c>
       <c r="F287" t="inlineStr"/>
-      <c r="G287" t="n">
-        <v>2021</v>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
@@ -15960,11 +15962,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F288" t="n">
-        <v>599</v>
-      </c>
-      <c r="G288" t="n">
-        <v>2017</v>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
@@ -16015,11 +16021,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F289" t="n">
-        <v>700</v>
-      </c>
-      <c r="G289" t="n">
-        <v>2018</v>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
@@ -16070,11 +16080,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F290" t="n">
-        <v>599</v>
-      </c>
-      <c r="G290" t="n">
-        <v>2015</v>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
@@ -16092,6 +16106,114 @@
       <c r="M290" t="inlineStr">
         <is>
           <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradient Orbit</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-flying-on-the-sand-no-tr-7011/</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr"/>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 270,55 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>999</v>
+      </c>
+      <c r="G292" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr"/>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr"/>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -16106,7 +16228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -23217,8 +23339,10 @@
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
-      <c r="G127" t="n">
-        <v>2021</v>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -23269,11 +23393,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>599</v>
-      </c>
-      <c r="G128" t="n">
-        <v>2017</v>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -23324,11 +23452,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F129" t="n">
-        <v>700</v>
-      </c>
-      <c r="G129" t="n">
-        <v>2018</v>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
@@ -23379,11 +23511,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
         </is>
       </c>
-      <c r="F130" t="n">
-        <v>599</v>
-      </c>
-      <c r="G130" t="n">
-        <v>2015</v>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
@@ -23401,6 +23537,114 @@
       <c r="M130" t="inlineStr">
         <is>
           <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradient Orbit</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-flying-on-the-sand-no-tr-7011/</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 270,55 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>999</v>
+      </c>
+      <c r="G132" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -23415,7 +23659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -23503,12 +23747,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -23518,50 +23762,50 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B GIN Calypso L 95-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B GIN C</t>
+          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradient Orbit</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-calypso-l-95-115kg-concertinas-no-sivs-no-flying-on--7006/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-flying-on-the-sand-no-tr-7011/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2021</v>
+        <v>2011</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -23571,146 +23815,40 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 543,78 CZK (5</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 270,55 CZK (999,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>599</v>
+        <v>999</v>
       </c>
       <c r="G3" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 982</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>700</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2018</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg Křídlo EN B Skywalk SKYWALK MOJITO / L 105-160kg 14 531,78 CZK (599,00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-skywalk-mojito-l-105-160kg-6558/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>599</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -23821,20 +23959,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -23906,6 +24044,61 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 270,55 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>999</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-05-31
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M292"/>
+  <dimension ref="A1:M301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16136,8 +16136,10 @@
         </is>
       </c>
       <c r="F291" t="inlineStr"/>
-      <c r="G291" t="n">
-        <v>2011</v>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
@@ -16188,11 +16190,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
         </is>
       </c>
-      <c r="F292" t="n">
-        <v>999</v>
-      </c>
-      <c r="G292" t="n">
-        <v>2020</v>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>999.0</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
@@ -16214,6 +16220,483 @@
       <c r="M292" t="inlineStr">
         <is>
           <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 546,60 CZK (5</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>599</v>
+      </c>
+      <c r="G293" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr"/>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr"/>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 999</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>700</v>
+      </c>
+      <c r="G294" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr"/>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr"/>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 284,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G295" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr"/>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 570,26 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G296" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr"/>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr"/>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova ION 4 S 80-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova ION 4 S 80</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-ion-4-s-80-100kg-no-sivs-no-flying-on-the-sand-no-t-7014/</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G297" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr"/>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr"/>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 260,53 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>999</v>
+      </c>
+      <c r="G298" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr"/>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 213,61 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>750</v>
+      </c>
+      <c r="G299" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr"/>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr"/>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 998,11 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G300" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr"/>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi XXS</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-XXS</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr"/>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>XXS</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr"/>
+      <c r="L301" t="inlineStr"/>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -16228,7 +16711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M132"/>
+  <dimension ref="A1:M141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -23567,8 +24050,10 @@
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
-      <c r="G131" t="n">
-        <v>2011</v>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
@@ -23619,11 +24104,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
         </is>
       </c>
-      <c r="F132" t="n">
-        <v>999</v>
-      </c>
-      <c r="G132" t="n">
-        <v>2020</v>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>999.0</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -23645,6 +24134,483 @@
       <c r="M132" t="inlineStr">
         <is>
           <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 546,60 CZK (5</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>599</v>
+      </c>
+      <c r="G133" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 999</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>700</v>
+      </c>
+      <c r="G134" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 284,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G135" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 570,26 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G136" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova ION 4 S 80-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova ION 4 S 80</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-ion-4-s-80-100kg-no-sivs-no-flying-on-the-sand-no-t-7014/</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G137" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 260,53 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>999</v>
+      </c>
+      <c r="G138" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 213,61 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>750</v>
+      </c>
+      <c r="G139" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 998,11 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G140" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi XXS</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-XXS</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>XXS</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -23659,16 +24625,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -23747,12 +24713,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -23762,26 +24728,28 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradient Orbit</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 546,60 CZK (5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-flying-on-the-sand-no-tr-7011/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>599</v>
+      </c>
       <c r="G2" t="n">
-        <v>2011</v>
+        <v>2017</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -23793,19 +24761,19 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -23815,40 +24783,407 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 270,55 CZK (999,00 EUR) EN A Velikost</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>999</v>
+        <v>700</v>
       </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 284,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 570,26 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova ION 4 S 80-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova ION 4 S 80</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-ion-4-s-80-100kg-no-sivs-no-flying-on-the-sand-no-t-7014/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 260,53 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>999</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 213,61 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>750</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 998,11 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi XXS</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-XXS</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>XXS</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -23863,103 +25198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -24047,12 +25286,269 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 570,26 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova ION 4 S 80-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova ION 4 S 80</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-ion-4-s-80-100kg-no-sivs-no-flying-on-the-sand-no-t-7014/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové Křídlo EN A Nova Nivo M 80-100kg Listovaný Nové 50 998,11 CZK (2 100,00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-nivo-m-80-100kg-concertinas-new-6618/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -24062,40 +25558,201 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 270,55 CZK (999,00 EUR) EN A Velikost</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 284,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="G2" t="n">
         <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 70-90kg Křídlo EN B UP Kibo 70-90kg 31 570,26 CZK (1 300,00 EUR) EN B Vzletová hmotnost: 70 - 90 Opo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-70-90kg-6605/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova ION 4 S 80-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova ION 4 S 80</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-ion-4-s-80-100kg-no-sivs-no-flying-on-the-sand-no-t-7014/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 24 260,53 CZK (999,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7010/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-02
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M301"/>
+  <dimension ref="A1:M305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16734,6 +16734,214 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-7022/</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr"/>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B S</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7021/</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>737</v>
+      </c>
+      <c r="G303" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr"/>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr"/>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4-85kg 67 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC Lucky 4-85kg</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-85kg-67-no-sivs-no-flying-on-the-sand-no-tre-7024/</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr"/>
+      <c r="J305" t="inlineStr"/>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr"/>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16745,20 +16953,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -16827,6 +17035,214 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-7022/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B S</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7021/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>737</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4-85kg 67 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC Lucky 4-85kg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-85kg-67-no-sivs-no-flying-on-the-sand-no-tre-7024/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -16841,20 +17257,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -16923,6 +17339,214 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-7022/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B S</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7021/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>737</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4-85kg 67 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC Lucky 4-85kg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-85kg-67-no-sivs-no-flying-on-the-sand-no-tre-7024/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -16937,20 +17561,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17019,6 +17643,110 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-7022/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -17033,20 +17761,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17118,6 +17846,57 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-03
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M305"/>
+  <dimension ref="A1:M310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16761,8 +16761,10 @@
         </is>
       </c>
       <c r="F302" t="inlineStr"/>
-      <c r="G302" t="n">
-        <v>2025</v>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
@@ -16813,11 +16815,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7021/</t>
         </is>
       </c>
-      <c r="F303" t="n">
-        <v>737</v>
-      </c>
-      <c r="G303" t="n">
-        <v>2016</v>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>737.0</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
@@ -16920,8 +16926,10 @@
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
-      <c r="G305" t="n">
-        <v>2016</v>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
@@ -16939,6 +16947,259 @@
       <c r="M305" t="inlineStr">
         <is>
           <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 18 000,00 CZK (750,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>750</v>
+      </c>
+      <c r="G306" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr"/>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr"/>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Little Cloud Spiruline EZ XL 60-120kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno (Součást kompl</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/little-cloud-spiruline-ez-xl-60-120kg-concertinas-no-siv-7029/</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr"/>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr"/>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 22 400,00 CZK (938,00 EUR) EN B Velikost: M Vzletová h</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>938</v>
+      </c>
+      <c r="G308" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr"/>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr"/>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 60</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr"/>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr"/>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>KOMPLET! MENTOR 5...</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=342&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>880</v>
+      </c>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr"/>
+      <c r="I310" t="inlineStr"/>
+      <c r="J310" t="inlineStr"/>
+      <c r="K310" t="inlineStr"/>
+      <c r="L310" t="inlineStr"/>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -16953,7 +17214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17065,8 +17326,10 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2025</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -17117,11 +17380,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7021/</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>737</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2016</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>737.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -17224,8 +17491,10 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2016</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -17243,6 +17512,259 @@
       <c r="M5" t="inlineStr">
         <is>
           <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 18 000,00 CZK (750,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>750</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Little Cloud Spiruline EZ XL 60-120kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno (Součást kompl</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/little-cloud-spiruline-ez-xl-60-120kg-concertinas-no-siv-7029/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 22 400,00 CZK (938,00 EUR) EN B Velikost: M Vzletová h</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>938</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 60</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KOMPLET! MENTOR 5...</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=342&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>880</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -17257,7 +17779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17270,7 +17792,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17360,17 +17882,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 18 000,00 CZK (750,00 EUR) EN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-7022/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>750</v>
+      </c>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -17379,19 +17903,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -17413,40 +17937,34 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B S</t>
+          <t>Křídlo EN B Little Cloud Spiruline EZ XL 60-120kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno (Součást kompl</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7021/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>737</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/little-cloud-spiruline-ez-xl-60-120kg-concertinas-no-siv-7029/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -17468,16 +17986,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 22 400,00 CZK (938,00 EUR) EN B Velikost: M Vzletová h</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>938</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
@@ -17485,31 +18007,31 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Olétané (více než 300h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -17519,34 +18041,79 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A MAC Lucky 4-85kg 67 Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC Lucky 4-85kg</t>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 60</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-85kg-67-no-sivs-no-flying-on-the-sand-no-tre-7024/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>KOMPLET! MENTOR 5...</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=342&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>880</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -17556,6 +18123,102 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17570,11 +18233,11 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -17664,17 +18327,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B BGD Base 2 M 75-95kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B BG</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 18 000,00 CZK (750,00 EUR) EN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/bgd-base-2-m-75-95kg-concertinas-new-no-sivs-no-flying-o-7022/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>750</v>
+      </c>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -17683,19 +18348,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -17717,16 +18382,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 22 400,00 CZK (938,00 EUR) EN B Velikost: M Vzletová h</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>938</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
@@ -17734,166 +18403,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Olétané (více než 300h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Trans 24 Křídlo EN B MAC Trans 24 1 500,00 CZK EN B Velikost: 24 Opotřebení: Olétané (více než 300h)</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-trans-24-7019/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Olétané (více než 300h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-04
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M310"/>
+  <dimension ref="A1:M314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -16976,11 +16976,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
         </is>
       </c>
-      <c r="F306" t="n">
-        <v>750</v>
-      </c>
-      <c r="G306" t="n">
-        <v>2020</v>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
@@ -17032,8 +17036,10 @@
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
-      <c r="G307" t="n">
-        <v>2015</v>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
@@ -17080,11 +17086,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
         </is>
       </c>
-      <c r="F308" t="n">
-        <v>938</v>
-      </c>
-      <c r="G308" t="n">
-        <v>2020</v>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>938.0</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H308" t="inlineStr">
         <is>
@@ -17136,8 +17146,10 @@
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
-      <c r="G309" t="n">
-        <v>2021</v>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H309" t="inlineStr">
         <is>
@@ -17188,8 +17200,10 @@
           <t>https://www.air-sport.cz/index.php?id_product=342&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
         </is>
       </c>
-      <c r="F310" t="n">
-        <v>880</v>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>880.0</t>
+        </is>
       </c>
       <c r="G310" t="inlineStr"/>
       <c r="H310" t="inlineStr"/>
@@ -17200,6 +17214,222 @@
       <c r="M310" t="inlineStr">
         <is>
           <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 19 000,00 CZK (790,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>790</v>
+      </c>
+      <c r="G311" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr"/>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr"/>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 4 XL 105-130kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-xl-105-130kg-concertinas-no-flying-on-the-s-7048/</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr"/>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr"/>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-24-60-80kg-concertinas-no-sivs-no-flying-7035/</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr"/>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr"/>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G314" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr"/>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr"/>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -17214,7 +17444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17541,11 +17771,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>750</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2020</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -17597,8 +17831,10 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="n">
-        <v>2015</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -17645,11 +17881,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>938</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2020</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>938.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -17701,8 +17941,10 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>2021</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -17753,8 +17995,10 @@
           <t>https://www.air-sport.cz/index.php?id_product=342&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>880</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>880.0</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -17765,6 +18009,222 @@
       <c r="M10" t="inlineStr">
         <is>
           <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 19 000,00 CZK (790,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>790</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 4 XL 105-130kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-xl-105-130kg-concertinas-no-flying-on-the-s-7048/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-24-60-80kg-concertinas-no-sivs-no-flying-7035/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -17779,7 +18239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17788,7 +18248,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -17882,7 +18342,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 18 000,00 CZK (750,00 EUR) EN</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 19 000,00 CZK (790,00 EUR) EN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -17891,7 +18351,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>750</v>
+        <v>790</v>
       </c>
       <c r="G2" t="n">
         <v>2020</v>
@@ -17915,7 +18375,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -17937,24 +18397,28 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Little Cloud Spiruline EZ XL 60-120kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno (Součást kompl</t>
+          <t>Křídlo EN B AXIS Pluto 4 XL 105-130kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/little-cloud-spiruline-ez-xl-60-120kg-concertinas-no-siv-7029/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-xl-105-130kg-concertinas-no-flying-on-the-s-7048/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2015</v>
+        <v>2025</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
@@ -17964,19 +18428,19 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -17986,52 +18450,50 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 22 400,00 CZK (938,00 EUR) EN B Velikost: M Vzletová h</t>
+          <t>Křídlo EN A Advance Alpha 6 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>938</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-24-60-80kg-concertinas-no-sivs-no-flying-7035/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -18041,26 +18503,28 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný TK platná 60</t>
+          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-tc-valid-6997/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1500</v>
+      </c>
       <c r="G5" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>xs</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -18072,48 +18536,7 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>airsport_cz</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Air-Sport CZ – Bazar</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>KOMPLET! MENTOR 5...</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.air-sport.cz/index.php?id_product=342&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>880</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -18128,20 +18551,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18210,6 +18633,61 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -18327,7 +18805,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 18 000,00 CZK (750,00 EUR) EN</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 19 000,00 CZK (790,00 EUR) EN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -18336,7 +18814,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>750</v>
+        <v>790</v>
       </c>
       <c r="G2" t="n">
         <v>2020</v>
@@ -18360,19 +18838,19 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18382,40 +18860,40 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 22 400,00 CZK (938,00 EUR) EN B Velikost: M Vzletová h</t>
+          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7028/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>938</v>
+        <v>1500</v>
       </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-05
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M314"/>
+  <dimension ref="A1:M315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17243,11 +17243,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
         </is>
       </c>
-      <c r="F311" t="n">
-        <v>790</v>
-      </c>
-      <c r="G311" t="n">
-        <v>2020</v>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>790.0</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H311" t="inlineStr">
         <is>
@@ -17299,8 +17303,10 @@
         </is>
       </c>
       <c r="F312" t="inlineStr"/>
-      <c r="G312" t="n">
-        <v>2025</v>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
@@ -17352,8 +17358,10 @@
         </is>
       </c>
       <c r="F313" t="inlineStr"/>
-      <c r="G313" t="n">
-        <v>2019</v>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H313" t="inlineStr">
         <is>
@@ -17404,11 +17412,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
         </is>
       </c>
-      <c r="F314" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G314" t="n">
-        <v>2024</v>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>1500.0</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
@@ -17430,6 +17442,51 @@
       <c r="M314" t="inlineStr">
         <is>
           <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>KOMPLET! Golden 5 22</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr"/>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr"/>
+      <c r="K315" t="inlineStr"/>
+      <c r="L315" t="inlineStr"/>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -17444,7 +17501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18038,11 +18095,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>790</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2020</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>790.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -18094,8 +18155,10 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>2025</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -18147,8 +18210,10 @@
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
-        <v>2019</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -18199,11 +18264,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G14" t="n">
-        <v>2024</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1500.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -18225,6 +18294,51 @@
       <c r="M14" t="inlineStr">
         <is>
           <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>airsport_cz</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Air-Sport CZ – Bazar</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KOMPLET! Golden 5 22</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -18239,20 +18353,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18327,12 +18441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>airsport_cz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Air-Sport CZ – Bazar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18342,201 +18456,30 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 19 000,00 CZK (790,00 EUR) EN</t>
+          <t>KOMPLET! Golden 5 22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+          <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>790</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>2360</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Pluto 4 XL 105-130kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AXIS Pluto 4</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-4-xl-105-130kg-concertinas-no-flying-on-the-s-7048/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 24 60-80kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-24-60-80kg-concertinas-no-sivs-no-flying-7035/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2019</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -18551,20 +18494,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18633,61 +18576,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
         </is>
       </c>
     </row>
@@ -18702,20 +18590,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18790,12 +18678,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>airsport_cz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Air-Sport CZ – Bazar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18805,95 +18693,30 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 19 000,00 CZK (790,00 EUR) EN</t>
+          <t>KOMPLET! Golden 5 22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+          <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>790</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>2360</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova aonic S Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Nova aonic S L</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-aonic-s-concertinas-no-sivs-no-flying-on-the-sand-n-6819/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-06
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M315"/>
+  <dimension ref="A1:M316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17471,8 +17471,10 @@
           <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
         </is>
       </c>
-      <c r="F315" t="n">
-        <v>2360</v>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>2360.0</t>
+        </is>
       </c>
       <c r="G315" t="inlineStr"/>
       <c r="H315" t="inlineStr"/>
@@ -17487,6 +17489,61 @@
       <c r="M315" t="inlineStr">
         <is>
           <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Skywalk Masala 3</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>840</v>
+      </c>
+      <c r="G316" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H316" t="inlineStr"/>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>XXS</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>55kg-85kg</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr"/>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -17501,7 +17558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17514,7 +17571,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18323,8 +18380,10 @@
           <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>2360</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2360.0</t>
+        </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -18339,6 +18398,61 @@
       <c r="M15" t="inlineStr">
         <is>
           <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Skywalk Masala 3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>840</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>XXS</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>55kg-85kg</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -18356,17 +18470,17 @@
   <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18441,45 +18555,55 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>airsport_cz</t>
+          <t>paragliding_store_at</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Air-Sport CZ – Bazar</t>
+          <t>Paragliding Store AT – Used</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KOMPLET! Golden 5 22</t>
+          <t>Skywalk Masala 3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2360</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+        <v>840</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+          <t>XXS</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>55kg-85kg</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -18590,14 +18714,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -18675,51 +18799,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>airsport_cz</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Air-Sport CZ – Bazar</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>KOMPLET! Golden 5 22</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://www.air-sport.cz/index.php?id_product=344&amp;rewrite=golden-5-22&amp;controller=product&amp;id_lang=2</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2360</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-07
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M316"/>
+  <dimension ref="A1:M319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17518,11 +17518,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F316" t="n">
-        <v>840</v>
-      </c>
-      <c r="G316" t="n">
-        <v>2020</v>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>840.0</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H316" t="inlineStr"/>
       <c r="I316" t="inlineStr">
@@ -17544,6 +17548,165 @@
       <c r="M316" t="inlineStr">
         <is>
           <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 832,05 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>899</v>
+      </c>
+      <c r="G317" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr"/>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr"/>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 4 28 78-105kg Listovaný Žádné SIV TK není Nelétáno na písku S batohem Křídlo EN A Advance Alph</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-4-28-78-105kg-concertinas-no-sivs-no-tc-no-7060/</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr"/>
+      <c r="G318" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr"/>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr"/>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 165,08 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>750</v>
+      </c>
+      <c r="G319" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr"/>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr"/>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
         </is>
       </c>
     </row>
@@ -17558,7 +17721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18427,11 +18590,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>840</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2020</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>840.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
@@ -18453,6 +18620,165 @@
       <c r="M16" t="inlineStr">
         <is>
           <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 832,05 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>899</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 4 28 78-105kg Listovaný Žádné SIV TK není Nelétáno na písku S batohem Křídlo EN A Advance Alph</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-4-28-78-105kg-concertinas-no-sivs-no-tc-no-7060/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 165,08 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>750</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
         </is>
       </c>
     </row>
@@ -18467,20 +18793,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18555,55 +18881,159 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_store_at</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Store AT – Used</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Skywalk Masala 3</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 832,05 CZK (899,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>840</v>
+        <v>899</v>
       </c>
       <c r="G2" t="n">
         <v>2020</v>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>XXS</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>55kg-85kg</t>
-        </is>
-      </c>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 4 28 78-105kg Listovaný Žádné SIV TK není Nelétáno na písku S batohem Křídlo EN A Advance Alph</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-4-28-78-105kg-concertinas-no-sivs-no-tc-no-7060/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 165,08 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>750</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-08
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M319"/>
+  <dimension ref="A1:M322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17577,11 +17577,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
-      <c r="F317" t="n">
-        <v>899</v>
-      </c>
-      <c r="G317" t="n">
-        <v>2020</v>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
@@ -17633,8 +17637,10 @@
         </is>
       </c>
       <c r="F318" t="inlineStr"/>
-      <c r="G318" t="n">
-        <v>2007</v>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
@@ -17685,11 +17691,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F319" t="n">
-        <v>750</v>
-      </c>
-      <c r="G319" t="n">
-        <v>2023</v>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
@@ -17707,6 +17717,167 @@
       <c r="M319" t="inlineStr">
         <is>
           <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná TOP Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr"/>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná 11 000,0</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-85-105kg-concertinas-tc-valid-7081/</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr"/>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr"/>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 220,11 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G322" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr"/>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr"/>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -17721,7 +17892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18649,11 +18820,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>899</v>
-      </c>
-      <c r="G17" t="n">
-        <v>2020</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -18705,8 +18880,10 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>2007</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -18757,11 +18934,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>750</v>
-      </c>
-      <c r="G19" t="n">
-        <v>2023</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -18779,6 +18960,167 @@
       <c r="M19" t="inlineStr">
         <is>
           <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná TOP Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná 11 000,0</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-85-105kg-concertinas-tc-valid-7081/</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 220,11 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -18806,7 +19148,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -18881,12 +19223,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18896,52 +19238,50 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 832,05 CZK (899,00 EUR) EN A Velikost</t>
+          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná TOP Křídlo EN B</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>899</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18951,26 +19291,26 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 4 28 78-105kg Listovaný Žádné SIV TK není Nelétáno na písku S batohem Křídlo EN A Advance Alph</t>
+          <t>Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná 11 000,0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-4-28-78-105kg-concertinas-no-sivs-no-tc-no-7060/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-85-105kg-concertinas-tc-valid-7081/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2007</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -18982,19 +19322,19 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -19004,36 +19344,40 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 165,08 CZK (750,00 EUR) E</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 220,11 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -19144,20 +19488,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -19229,6 +19573,61 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 220,11 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-09
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M322"/>
+  <dimension ref="A1:M323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17747,8 +17747,10 @@
         </is>
       </c>
       <c r="F320" t="inlineStr"/>
-      <c r="G320" t="n">
-        <v>2022</v>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
@@ -17800,8 +17802,10 @@
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
-      <c r="G321" t="n">
-        <v>2018</v>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
@@ -17852,11 +17856,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F322" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G322" t="n">
-        <v>2020</v>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H322" t="inlineStr">
         <is>
@@ -17878,6 +17886,61 @@
       <c r="M322" t="inlineStr">
         <is>
           <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 954</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>700</v>
+      </c>
+      <c r="G323" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr"/>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr"/>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -17892,7 +17955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18990,8 +19053,10 @@
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="n">
-        <v>2022</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -19043,8 +19108,10 @@
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
-        <v>2018</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -19095,11 +19162,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G22" t="n">
-        <v>2020</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -19121,6 +19192,61 @@
       <c r="M22" t="inlineStr">
         <is>
           <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 954</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>700</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -19135,7 +19261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19148,7 +19274,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -19238,17 +19364,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 4 L 90-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná TOP Křídlo EN B</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 954</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-90-115kg-no-sivs-no-flying-on-the-sand-no-6922/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>700</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -19257,127 +19385,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná Křídlo EN B AXIS Comet 3 M 85-105kg Listovaný TK platná 11 000,0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-85-105kg-concertinas-tc-valid-7081/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2018</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 220,11 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -19488,20 +19508,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -19573,61 +19593,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 220,11 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-10
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M323"/>
+  <dimension ref="A1:M332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17915,11 +17915,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F323" t="n">
-        <v>700</v>
-      </c>
-      <c r="G323" t="n">
-        <v>2018</v>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H323" t="inlineStr">
         <is>
@@ -17941,6 +17945,447 @@
       <c r="M323" t="inlineStr">
         <is>
           <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr"/>
+      <c r="G324" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr"/>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr"/>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 90-115kg Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná (Součást kompletu) Křídlo</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-90-115kg-no-sivs-no-flying-on-the-sand-no-7095/</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr"/>
+      <c r="G325" t="inlineStr"/>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr"/>
+      <c r="J325" t="inlineStr"/>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr"/>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho XL 105-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná (Součást kompletu) Kří</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-xl-105-130kg-no-sivs-no-flying-on-the-san-7094/</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr"/>
+      <c r="G326" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr"/>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr"/>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>REZERVOVÁNO: Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá REZERVOVÁNO: Křídlo EN A U</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr"/>
+      <c r="G327" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr"/>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr"/>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Gin Yeti</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>690</v>
+      </c>
+      <c r="G328" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H328" t="inlineStr"/>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>55kg-75kg</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>sehr gut --&gt; wenig geflogen--&gt;neuer Chec</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr"/>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Susi 4.23</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>2175</v>
+      </c>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr"/>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr"/>
+      <c r="K329" t="inlineStr"/>
+      <c r="L329" t="inlineStr"/>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Coral Red – Occasion</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>619</v>
+      </c>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr"/>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr"/>
+      <c r="K330" t="inlineStr"/>
+      <c r="L330" t="inlineStr"/>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Dusted Purple – Occasion</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>571</v>
+      </c>
+      <c r="G331" t="inlineStr"/>
+      <c r="H331" t="inlineStr"/>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr"/>
+      <c r="K331" t="inlineStr"/>
+      <c r="L331" t="inlineStr"/>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Advance PI 3 | Grösse 23 | Weiss – 180 Flüge</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>1667</v>
+      </c>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr"/>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr"/>
+      <c r="K332" t="inlineStr"/>
+      <c r="L332" t="inlineStr"/>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -17955,11 +18400,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -19221,11 +19666,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>700</v>
-      </c>
-      <c r="G23" t="n">
-        <v>2018</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -19247,6 +19696,447 @@
       <c r="M23" t="inlineStr">
         <is>
           <t>2026-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 90-115kg Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná (Součást kompletu) Křídlo</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-90-115kg-no-sivs-no-flying-on-the-sand-no-7095/</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho XL 105-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná (Součást kompletu) Kří</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-xl-105-130kg-no-sivs-no-flying-on-the-san-7094/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>REZERVOVÁNO: Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá REZERVOVÁNO: Křídlo EN A U</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Gin Yeti</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>690</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>55kg-75kg</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>sehr gut --&gt; wenig geflogen--&gt;neuer Chec</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Susi 4.23</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>2175</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Coral Red – Occasion</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>619</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Dusted Purple – Occasion</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>571</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Advance PI 3 | Grösse 23 | Weiss – 180 Flüge</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1667</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -19261,20 +20151,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -19349,12 +20239,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -19364,40 +20254,426 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 954</t>
+          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 90-115kg Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná (Součást kompletu) Křídlo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-90-115kg-no-sivs-no-flying-on-the-sand-no-7095/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho XL 105-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná (Součást kompletu) Kří</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-xl-105-130kg-no-sivs-no-flying-on-the-san-7094/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>REZERVOVÁNO: Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá REZERVOVÁNO: Křídlo EN A U</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Gin Yeti</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>690</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>55kg-75kg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>sehr gut --&gt; wenig geflogen--&gt;neuer Chec</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Susi 4.23</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2175</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Coral Red – Occasion</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>619</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Dusted Purple – Occasion</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>571</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Advance PI 3 | Grösse 23 | Weiss – 180 Flüge</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1667</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -19412,20 +20688,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -19494,6 +20770,149 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Coral Red – Occasion</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>619</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Advance Easiness 4 | Grösse M | Dusted Purple – Occasion</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>571</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -19508,20 +20927,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -19593,6 +21012,149 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Susi 4.23</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2175</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fly_ikarus_ch</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fly Ikarus CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Advance PI 3 | Grösse 23 | Weiss – 180 Flüge</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1667</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-11
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M332"/>
+  <dimension ref="A1:M338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -17975,8 +17975,10 @@
         </is>
       </c>
       <c r="F324" t="inlineStr"/>
-      <c r="G324" t="n">
-        <v>2022</v>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H324" t="inlineStr">
         <is>
@@ -18075,8 +18077,10 @@
         </is>
       </c>
       <c r="F326" t="inlineStr"/>
-      <c r="G326" t="n">
-        <v>2023</v>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H326" t="inlineStr">
         <is>
@@ -18128,8 +18132,10 @@
         </is>
       </c>
       <c r="F327" t="inlineStr"/>
-      <c r="G327" t="n">
-        <v>2020</v>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H327" t="inlineStr">
         <is>
@@ -18180,11 +18186,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F328" t="n">
-        <v>690</v>
-      </c>
-      <c r="G328" t="n">
-        <v>2016</v>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>690.0</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H328" t="inlineStr"/>
       <c r="I328" t="inlineStr">
@@ -18235,8 +18245,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
         </is>
       </c>
-      <c r="F329" t="n">
-        <v>2175</v>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>2175.0</t>
+        </is>
       </c>
       <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr"/>
@@ -18280,8 +18292,10 @@
           <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
         </is>
       </c>
-      <c r="F330" t="n">
-        <v>619</v>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>619.0</t>
+        </is>
       </c>
       <c r="G330" t="inlineStr"/>
       <c r="H330" t="inlineStr"/>
@@ -18325,8 +18339,10 @@
           <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
         </is>
       </c>
-      <c r="F331" t="n">
-        <v>571</v>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>571.0</t>
+        </is>
       </c>
       <c r="G331" t="inlineStr"/>
       <c r="H331" t="inlineStr"/>
@@ -18370,8 +18386,10 @@
           <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
         </is>
       </c>
-      <c r="F332" t="n">
-        <v>1667</v>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>1667.0</t>
+        </is>
       </c>
       <c r="G332" t="inlineStr"/>
       <c r="H332" t="inlineStr"/>
@@ -18386,6 +18404,332 @@
       <c r="M332" t="inlineStr">
         <is>
           <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G333" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr"/>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr"/>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný Žádné SIV Nevětveno TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Li</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-no-sivs-no-trees--6997/</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr"/>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr"/>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr"/>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr"/>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 728,62 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>899</v>
+      </c>
+      <c r="G336" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr"/>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr"/>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Nova ION 5 M</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>690</v>
+      </c>
+      <c r="G337" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H337" t="inlineStr"/>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>90kg-95kg</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>gut --&gt; keine Beschädigungen --&gt; wenig g</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr"/>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 9 26 Kommissionsverkauf</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>980</v>
+      </c>
+      <c r="G338" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H338" t="inlineStr"/>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>80kg-100kg</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr"/>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -18400,7 +18744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19726,8 +20070,10 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>2022</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -19826,8 +20172,10 @@
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="n">
-        <v>2023</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -19879,8 +20227,10 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="n">
-        <v>2020</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -19931,11 +20281,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>690</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2016</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>690.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
@@ -19986,8 +20340,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>2175</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2175.0</t>
+        </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -20031,8 +20387,10 @@
           <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>619</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>619.0</t>
+        </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -20076,8 +20434,10 @@
           <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>571</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>571.0</t>
+        </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -20121,8 +20481,10 @@
           <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>1667</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1667.0</t>
+        </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -20137,6 +20499,332 @@
       <c r="M32" t="inlineStr">
         <is>
           <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný Žádné SIV Nevětveno TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Li</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-no-sivs-no-trees--6997/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 728,62 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>899</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Nova ION 5 M</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>690</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>90kg-95kg</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>gut --&gt; keine Beschädigungen --&gt; wenig g</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 9 26 Kommissionsverkauf</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>980</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>80kg-100kg</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -20151,16 +20839,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -20239,12 +20927,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -20254,50 +20942,52 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2800</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20307,32 +20997,38 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Orbit 90-115kg Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná (Součást kompletu) Křídlo</t>
+          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný Žádné SIV Nevětveno TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Li</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-90-115kg-no-sivs-no-flying-on-the-sand-no-7095/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-no-sivs-no-trees--6997/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -20354,17 +21050,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Drift carancho XL 105-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná (Součást kompletu) Kří</t>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-xl-105-130kg-no-sivs-no-flying-on-the-san-7094/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -20373,19 +21069,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -20407,15 +21103,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>REZERVOVÁNO: Křídlo EN A UP MANA 27 80-110kg Listovaný Odlehčeno Nelétáno na písku TK čerstvá REZERVOVÁNO: Křídlo EN A U</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 728,62 CZK (899,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-mana-27-80-110kg-concertinas-lightened-no-flying-on-t-6978/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>899</v>
+      </c>
       <c r="G5" t="n">
         <v>2020</v>
       </c>
@@ -20426,19 +21124,19 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -20460,7 +21158,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Gin Yeti</t>
+          <t>Nova ION 5 M</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -20472,208 +21170,83 @@
         <v>690</v>
       </c>
       <c r="G6" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>55kg-75kg</t>
+          <t>90kg-95kg</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>sehr gut --&gt; wenig geflogen--&gt;neuer Chec</t>
+          <t>gut --&gt; keine Beschädigungen --&gt; wenig g</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hochries_de</t>
+          <t>paragliding_store_at</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+          <t>Paragliding Store AT – Used</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AIRDESIGN Susi 4.23</t>
+          <t>Advance Epsilon 9 26 Kommissionsverkauf</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2175</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
+        <v>980</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2019</v>
+      </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>80kg-100kg</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>fly_ikarus_ch</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Fly Ikarus CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Advance Easiness 4 | Grösse M | Coral Red – Occasion</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>619</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>fly_ikarus_ch</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Fly Ikarus CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Advance Easiness 4 | Grösse M | Dusted Purple – Occasion</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>571</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>fly_ikarus_ch</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Fly Ikarus CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Advance PI 3 | Grösse 23 | Weiss – 180 Flüge</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>1667</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -20688,7 +21261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20697,11 +21270,11 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -20776,12 +21349,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -20791,128 +21364,93 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2800</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fly_ikarus_ch</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fly Ikarus CH – Occasionen</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Advance Easiness 4 | Grösse M | Coral Red – Occasion</t>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-coral-red-occasion/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>619</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>fly_ikarus_ch</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fly Ikarus CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Advance Easiness 4 | Grösse M | Dusted Purple – Occasion</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://fly-ikarus.ch/produkt/advance-easiness-4-groesse-m-dusted-purple-occasion/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>571</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -20927,20 +21465,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -21015,12 +21553,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21030,128 +21568,93 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Pi 3 25 85-120kg Křídlo EN A Advance Pi 3 25 85-120kg 35 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
+          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-85-120kg-7097/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2800</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hochries_de</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AIRDESIGN Susi 4.23</t>
+          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Susi-4.23/SW10599</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>2175</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>fly_ikarus_ch</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fly Ikarus CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Advance PI 3 | Grösse 23 | Weiss – 180 Flüge</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://fly-ikarus.ch/produkt/advance-pi-3-groesse-23-weiss-180-fluege/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1667</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-12
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M338"/>
+  <dimension ref="A1:M340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18433,11 +18433,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
         </is>
       </c>
-      <c r="F333" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G333" t="n">
-        <v>2025</v>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>2800.0</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H333" t="inlineStr">
         <is>
@@ -18489,8 +18493,10 @@
         </is>
       </c>
       <c r="F334" t="inlineStr"/>
-      <c r="G334" t="n">
-        <v>2021</v>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H334" t="inlineStr">
         <is>
@@ -18542,8 +18548,10 @@
         </is>
       </c>
       <c r="F335" t="inlineStr"/>
-      <c r="G335" t="n">
-        <v>2021</v>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H335" t="inlineStr">
         <is>
@@ -18594,11 +18602,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
-      <c r="F336" t="n">
-        <v>899</v>
-      </c>
-      <c r="G336" t="n">
-        <v>2020</v>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H336" t="inlineStr">
         <is>
@@ -18649,11 +18661,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F337" t="n">
-        <v>690</v>
-      </c>
-      <c r="G337" t="n">
-        <v>2018</v>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>690.0</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H337" t="inlineStr"/>
       <c r="I337" t="inlineStr">
@@ -18704,11 +18720,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F338" t="n">
-        <v>980</v>
-      </c>
-      <c r="G338" t="n">
-        <v>2019</v>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H338" t="inlineStr"/>
       <c r="I338" t="inlineStr">
@@ -18730,6 +18750,114 @@
       <c r="M338" t="inlineStr">
         <is>
           <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G339" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr"/>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr"/>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A A</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-95kg-concertinas-no-sivs-no-flying-7120/</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr"/>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr"/>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -18744,7 +18872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20528,11 +20656,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G33" t="n">
-        <v>2025</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2800.0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -20584,8 +20716,10 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="n">
-        <v>2021</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -20637,8 +20771,10 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="n">
-        <v>2021</v>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -20689,11 +20825,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>899</v>
-      </c>
-      <c r="G36" t="n">
-        <v>2020</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -20744,11 +20884,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>690</v>
-      </c>
-      <c r="G37" t="n">
-        <v>2018</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>690.0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
@@ -20799,11 +20943,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>980</v>
-      </c>
-      <c r="G38" t="n">
-        <v>2019</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>980.0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
@@ -20825,6 +20973,114 @@
       <c r="M38" t="inlineStr">
         <is>
           <t>2026-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A A</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-95kg-concertinas-no-sivs-no-flying-7120/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -20834,428 +21090,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skywalk Chili 5 xs 70-95kg Listovaný Žádné SIV Nevětveno TK platná Křídlo EN B Skywalk Chili 5 xs 70-95kg Li</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-xs-70-95kg-concertinas-no-sivs-no-trees--6997/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>xs</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 728,62 CZK (899,00 EUR) EN A Velikost</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>899</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Nova ION 5 M</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>690</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2018</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>90kg-95kg</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>gut --&gt; keine Beschädigungen --&gt; wenig g</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Advance Epsilon 9 26 Kommissionsverkauf</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>980</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2019</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>80kg-100kg</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21349,12 +21183,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21364,23 +21198,23 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
+          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2800</v>
+        <v>1350</v>
       </c>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -21397,7 +21231,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -21419,17 +21253,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
+          <t>Křídlo EN A Advance Alpha 6 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A A</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-95kg-concertinas-no-sivs-no-flying-7120/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -21438,19 +21272,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -21459,13 +21293,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21553,12 +21387,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21568,23 +21402,23 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Niviuk Ikuma 3 26 85-105kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Niviuk Ikum</t>
+          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-ikuma-3-26-85-105kg-concertinas-no-flying-on-the--7109/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2800</v>
+        <v>1350</v>
       </c>
       <c r="G2" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -21601,60 +21435,158 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá TK platná Křídlo EN A UP Rimo S 60-90kg Drobné opravy TK čerstvá</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-rimo-s-60-90kg-small-repairs-tc-fresh-tc-valid-7110/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>Mírně létané (50-100h)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-13
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M340"/>
+  <dimension ref="A1:M344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18779,11 +18779,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
         </is>
       </c>
-      <c r="F339" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G339" t="n">
-        <v>2022</v>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>1350.0</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H339" t="inlineStr">
         <is>
@@ -18835,8 +18839,10 @@
         </is>
       </c>
       <c r="F340" t="inlineStr"/>
-      <c r="G340" t="n">
-        <v>2019</v>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H340" t="inlineStr">
         <is>
@@ -18858,6 +18864,222 @@
       <c r="M340" t="inlineStr">
         <is>
           <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Nevada 26 85-105kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Gr</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-26-85-105kg-concertinas-no-sivs-no-tc-no-7129/</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="n">
+        <v>2014</v>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr"/>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L341" t="inlineStr"/>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 918</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>700</v>
+      </c>
+      <c r="G342" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr"/>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr"/>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 169,77 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G343" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr"/>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L343" t="inlineStr"/>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena M 85-110kg Nelétáno na písku Nevětveno TK čerstvá TK platná Křídlo EN A UP Dena M 85-110kg Nelétáno</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-flying-on-the-sand-no-trees-tc-fre-7124/</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr"/>
+      <c r="G344" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr"/>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L344" t="inlineStr"/>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -18872,7 +19094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21002,11 +21224,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2022</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1350.0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -21058,8 +21284,10 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="n">
-        <v>2019</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -21081,6 +21309,222 @@
       <c r="M40" t="inlineStr">
         <is>
           <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Nevada 26 85-105kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Gr</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-26-85-105kg-concertinas-no-sivs-no-tc-no-7129/</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="n">
+        <v>2014</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 918</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>700</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 169,77 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena M 85-110kg Nelétáno na písku Nevětveno TK čerstvá TK platná Křídlo EN A UP Dena M 85-110kg Nelétáno</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-flying-on-the-sand-no-trees-tc-fre-7124/</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -21095,7 +21539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21183,12 +21627,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21198,23 +21642,21 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+          <t>Křídlo EN B Gradient Nevada 26 85-105kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Gr</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1350</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-26-85-105kg-concertinas-no-sivs-no-tc-no-7129/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -21225,25 +21667,25 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21253,38 +21695,148 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 26 70-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno S batohem Křídlo EN A A</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 918</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-95kg-concertinas-no-sivs-no-flying-7120/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>700</v>
+      </c>
       <c r="G3" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 169,77 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena M 85-110kg Nelétáno na písku Nevětveno TK čerstvá TK platná Křídlo EN A UP Dena M 85-110kg Nelétáno</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-flying-on-the-sand-no-trees-tc-fre-7124/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -21402,17 +21954,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+          <t>Křídlo EN A UP Dena M 85-110kg Nelétáno na písku Nevětveno TK čerstvá TK platná Křídlo EN A UP Dena M 85-110kg Nelétáno</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1350</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-flying-on-the-sand-no-trees-tc-fre-7124/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>2022</v>
       </c>
@@ -21423,7 +21973,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -21435,7 +21985,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -21463,7 +22013,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -21538,12 +22088,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21553,40 +22103,40 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 7 26 70 (95)-95 (110)kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 169,77 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-26-70-95-95-110kg-no-sivs-no-flying-on-t-7116/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1350</v>
+        <v>1000</v>
       </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-14
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M344"/>
+  <dimension ref="A1:M348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -18894,8 +18894,10 @@
         </is>
       </c>
       <c r="F341" t="inlineStr"/>
-      <c r="G341" t="n">
-        <v>2014</v>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
       </c>
       <c r="H341" t="inlineStr">
         <is>
@@ -18946,11 +18948,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F342" t="n">
-        <v>700</v>
-      </c>
-      <c r="G342" t="n">
-        <v>2018</v>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H342" t="inlineStr">
         <is>
@@ -19001,11 +19007,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F343" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G343" t="n">
-        <v>2020</v>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H343" t="inlineStr">
         <is>
@@ -19057,8 +19067,10 @@
         </is>
       </c>
       <c r="F344" t="inlineStr"/>
-      <c r="G344" t="n">
-        <v>2022</v>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H344" t="inlineStr">
         <is>
@@ -19080,6 +19092,214 @@
       <c r="M344" t="inlineStr">
         <is>
           <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Sigma 10 25 80-100kg Listovaný TK čerstvá TK platná Křídlo EN B Advance Sigma 10 25 80-100kg Listova</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-sigma-10-25-80-100kg-concertinas-tc-fresh-tc-val-7134/</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr"/>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr"/>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G346" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr"/>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr"/>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 477,69 CZK (5</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>599</v>
+      </c>
+      <c r="G347" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr"/>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr"/>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>ADVANCE Sigma DLS 28</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr"/>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr"/>
+      <c r="K348" t="inlineStr"/>
+      <c r="L348" t="inlineStr"/>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -19094,7 +19314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21339,8 +21559,10 @@
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="n">
-        <v>2014</v>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -21391,11 +21613,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>700</v>
-      </c>
-      <c r="G42" t="n">
-        <v>2018</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -21446,11 +21672,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G43" t="n">
-        <v>2020</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -21502,8 +21732,10 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="n">
-        <v>2022</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -21525,6 +21757,214 @@
       <c r="M44" t="inlineStr">
         <is>
           <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Sigma 10 25 80-100kg Listovaný TK čerstvá TK platná Křídlo EN B Advance Sigma 10 25 80-100kg Listova</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-sigma-10-25-80-100kg-concertinas-tc-fresh-tc-val-7134/</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 477,69 CZK (5</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>599</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ADVANCE Sigma DLS 28</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -21543,12 +21983,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -21642,17 +22082,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Nevada 26 85-105kg Listovaný Žádné SIV TK není Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Gr</t>
+          <t>Křídlo EN B Advance Sigma 10 25 80-100kg Listovaný TK čerstvá TK platná Křídlo EN B Advance Sigma 10 25 80-100kg Listova</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-26-85-105kg-concertinas-no-sivs-no-tc-no-7129/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-sigma-10-25-80-100kg-concertinas-tc-fresh-tc-val-7134/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2014</v>
+        <v>2017</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -21661,19 +22101,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -21695,19 +22135,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 918</t>
+          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>700</v>
+        <v>1100</v>
       </c>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -21716,19 +22156,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>s</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -21750,19 +22190,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 169,77 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 477,69 CZK (5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1000</v>
+        <v>599</v>
       </c>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -21771,72 +22211,64 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Dena M 85-110kg Nelétáno na písku Nevětveno TK čerstvá TK platná Křídlo EN A UP Dena M 85-110kg Nelétáno</t>
+          <t>ADVANCE Sigma DLS 28</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-flying-on-the-sand-no-trees-tc-fre-7124/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -21851,20 +22283,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -21939,12 +22371,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21954,38 +22386,85 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Dena M 85-110kg Nelétáno na písku Nevětveno TK čerstvá TK platná Křídlo EN A UP Dena M 85-110kg Nelétáno</t>
+          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-flying-on-the-sand-no-trees-tc-fre-7124/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>s</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ADVANCE Sigma DLS 28</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -22103,19 +22582,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 169,77 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -22124,7 +22603,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>s</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -22136,7 +22615,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-15
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M348"/>
+  <dimension ref="A1:M357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19122,8 +19122,10 @@
         </is>
       </c>
       <c r="F345" t="inlineStr"/>
-      <c r="G345" t="n">
-        <v>2017</v>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H345" t="inlineStr">
         <is>
@@ -19174,11 +19176,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
         </is>
       </c>
-      <c r="F346" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G346" t="n">
-        <v>2023</v>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H346" t="inlineStr">
         <is>
@@ -19229,11 +19235,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F347" t="n">
-        <v>599</v>
-      </c>
-      <c r="G347" t="n">
-        <v>2017</v>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H347" t="inlineStr">
         <is>
@@ -19284,8 +19294,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
         </is>
       </c>
-      <c r="F348" t="n">
-        <v>3450</v>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>3450.0</t>
+        </is>
       </c>
       <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr"/>
@@ -19300,6 +19312,461 @@
       <c r="M348" t="inlineStr">
         <is>
           <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr"/>
+      <c r="G349" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr"/>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L349" t="inlineStr"/>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 27 92-114kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platn Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G350" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr"/>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L350" t="inlineStr"/>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Tequila 5 85-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Tequila 5 85-</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-tequila-5-85-105kg-no-sivs-no-flying-on-the-sand-7144/</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr"/>
+      <c r="J351" t="inlineStr"/>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr"/>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115k</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-no-sivs-no-flying-on-the-sand-n-7143/</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr"/>
+      <c r="J352" t="inlineStr"/>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr"/>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 5 L 95-115kg Listovaný TK platná S listovacím obalem Křídlo EN B Ozone Rush 5 L 95-115kg Listovan</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-95-115kg-concertinas-tc-valid-with-listin-7139/</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr"/>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr"/>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Atis 2 M 75-95kg Žádné SIV TK není Nevětveno Nekoupáno Křídlo EN B SKY Paragliders Atis 2 M</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-atis-2-m-75-95kg-no-sivs-no-tc-no-trees--7135/</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr"/>
+      <c r="G354" t="n">
+        <v>2008</v>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr"/>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr"/>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr"/>
+      <c r="G355" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr"/>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L355" t="inlineStr"/>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>ADVANCE Theta ULS 29</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-ThetaULS-29</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G356" t="inlineStr"/>
+      <c r="H356" t="inlineStr"/>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr"/>
+      <c r="K356" t="inlineStr"/>
+      <c r="L356" t="inlineStr"/>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi S</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr"/>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr"/>
+      <c r="K357" t="inlineStr"/>
+      <c r="L357" t="inlineStr"/>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -19314,7 +19781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21787,8 +22254,10 @@
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
-      <c r="G45" t="n">
-        <v>2017</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -21839,11 +22308,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G46" t="n">
-        <v>2023</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1100.0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -21894,11 +22367,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>599</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2017</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -21949,8 +22426,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>3450</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>3450.0</t>
+        </is>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
@@ -21965,6 +22444,461 @@
       <c r="M48" t="inlineStr">
         <is>
           <t>2026-06-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 27 92-114kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platn Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G50" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Tequila 5 85-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Tequila 5 85-</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-tequila-5-85-105kg-no-sivs-no-flying-on-the-sand-7144/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115k</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-no-sivs-no-flying-on-the-sand-n-7143/</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 5 L 95-115kg Listovaný TK platná S listovacím obalem Křídlo EN B Ozone Rush 5 L 95-115kg Listovan</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-95-115kg-concertinas-tc-valid-with-listin-7139/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Atis 2 M 75-95kg Žádné SIV TK není Nevětveno Nekoupáno Křídlo EN B SKY Paragliders Atis 2 M</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-atis-2-m-75-95kg-no-sivs-no-tc-no-trees--7135/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="n">
+        <v>2008</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ADVANCE Theta ULS 29</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-ThetaULS-29</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi S</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -21974,6 +22908,557 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Iota DLS 27 92-114kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platn Křídlo EN B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Tequila 5 85-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Tequila 5 85-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-tequila-5-85-105kg-no-sivs-no-flying-on-the-sand-7144/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115k</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-no-sivs-no-flying-on-the-sand-n-7143/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 5 L 95-115kg Listovaný TK platná S listovacím obalem Křídlo EN B Ozone Rush 5 L 95-115kg Listovan</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-95-115kg-concertinas-tc-valid-with-listin-7139/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Atis 2 M 75-95kg Žádné SIV TK není Nevětveno Nekoupáno Křídlo EN B SKY Paragliders Atis 2 M</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-atis-2-m-75-95kg-no-sivs-no-tc-no-trees--7135/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ADVANCE Theta ULS 29</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-ThetaULS-29</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi S</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22082,17 +23567,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Sigma 10 25 80-100kg Listovaný TK čerstvá TK platná Křídlo EN B Advance Sigma 10 25 80-100kg Listova</t>
+          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-sigma-10-25-80-100kg-concertinas-tc-fresh-tc-val-7134/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -22101,19 +23586,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>SM</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -22135,19 +23620,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
+          <t>Křídlo EN B Advance Iota DLS 27 92-114kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platn Křídlo EN B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1100</v>
+        <v>2500</v>
       </c>
       <c r="G3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -22156,31 +23641,31 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -22190,40 +23675,38 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 477,69 CZK (5</t>
+          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>599</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2017</v>
+        <v>2024</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -22245,22 +23728,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ADVANCE Sigma DLS 28</t>
+          <t>AIRDESIGN Livi S</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3450</v>
+        <v>2750</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -22268,7 +23751,7 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -22277,13 +23760,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -22296,7 +23779,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -22386,19 +23869,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
+          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1100</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -22407,215 +23888,170 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>SM</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hochries_de</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ADVANCE Sigma DLS 28</t>
+          <t>Křídlo EN B Ozone Rush 5 L 95-115kg Listovaný TK platná S listovacím obalem Křídlo EN B Ozone Rush 5 L 95-115kg Listovan</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS28</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>3450</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-95-115kg-concertinas-tc-valid-with-listin-7139/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP KIBO X s 70-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B UP KIBO X s 70-90kg Žádné SI</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-s-70-90kg-no-sivs-no-flying-on-the-sand-no-tre-7133/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Jako nové (0-50h)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi S</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-16
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M357"/>
+  <dimension ref="A1:M360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19342,8 +19342,10 @@
         </is>
       </c>
       <c r="F349" t="inlineStr"/>
-      <c r="G349" t="n">
-        <v>2022</v>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H349" t="inlineStr">
         <is>
@@ -19394,11 +19396,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
         </is>
       </c>
-      <c r="F350" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G350" t="n">
-        <v>2024</v>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H350" t="inlineStr">
         <is>
@@ -19450,8 +19456,10 @@
         </is>
       </c>
       <c r="F351" t="inlineStr"/>
-      <c r="G351" t="n">
-        <v>2018</v>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H351" t="inlineStr">
         <is>
@@ -19499,8 +19507,10 @@
         </is>
       </c>
       <c r="F352" t="inlineStr"/>
-      <c r="G352" t="n">
-        <v>2022</v>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H352" t="inlineStr">
         <is>
@@ -19548,8 +19558,10 @@
         </is>
       </c>
       <c r="F353" t="inlineStr"/>
-      <c r="G353" t="n">
-        <v>2020</v>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H353" t="inlineStr">
         <is>
@@ -19601,8 +19613,10 @@
         </is>
       </c>
       <c r="F354" t="inlineStr"/>
-      <c r="G354" t="n">
-        <v>2008</v>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>2008.0</t>
+        </is>
       </c>
       <c r="H354" t="inlineStr">
         <is>
@@ -19654,8 +19668,10 @@
         </is>
       </c>
       <c r="F355" t="inlineStr"/>
-      <c r="G355" t="n">
-        <v>2024</v>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H355" t="inlineStr">
         <is>
@@ -19706,8 +19722,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-ThetaULS-29</t>
         </is>
       </c>
-      <c r="F356" t="n">
-        <v>3150</v>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>3150.0</t>
+        </is>
       </c>
       <c r="G356" t="inlineStr"/>
       <c r="H356" t="inlineStr"/>
@@ -19751,8 +19769,10 @@
           <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
         </is>
       </c>
-      <c r="F357" t="n">
-        <v>2750</v>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>2750.0</t>
+        </is>
       </c>
       <c r="G357" t="inlineStr"/>
       <c r="H357" t="inlineStr"/>
@@ -19767,6 +19787,163 @@
       <c r="M357" t="inlineStr">
         <is>
           <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Gradient</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-flying-on-the-s-7154/</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr"/>
+      <c r="G358" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr"/>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L358" t="inlineStr"/>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 95-115kg Nové Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115kg Nov</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-new-no-flying-on-the-sand-no-tr-7152/</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G359" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr"/>
+      <c r="J359" t="inlineStr"/>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L359" t="inlineStr"/>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Skyman The Rock 2 29,5 105-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno TOP Křídlo E</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skyman-the-rock-2-295-105-130kg-concertinas-lightened-ne-6792/</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr"/>
+      <c r="G360" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr"/>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L360" t="inlineStr"/>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -19781,7 +19958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -22474,8 +22651,10 @@
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="n">
-        <v>2022</v>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -22526,11 +22705,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G50" t="n">
-        <v>2024</v>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2500.0</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -22582,8 +22765,10 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="n">
-        <v>2018</v>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -22631,8 +22816,10 @@
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
-      <c r="G52" t="n">
-        <v>2022</v>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -22680,8 +22867,10 @@
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="n">
-        <v>2020</v>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -22733,8 +22922,10 @@
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="n">
-        <v>2008</v>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2008.0</t>
+        </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -22786,8 +22977,10 @@
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="n">
-        <v>2024</v>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -22838,8 +23031,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-ThetaULS-29</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>3150</v>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>3150.0</t>
+        </is>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
@@ -22883,8 +23078,10 @@
           <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>2750</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2750.0</t>
+        </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
@@ -22899,6 +23096,163 @@
       <c r="M57" t="inlineStr">
         <is>
           <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Gradient</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-flying-on-the-s-7154/</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skywalk Chili 5 95-115kg Nové Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115kg Nov</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-new-no-flying-on-the-sand-no-tr-7152/</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G59" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Skyman The Rock 2 29,5 105-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno TOP Křídlo E</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skyman-the-rock-2-295-105-130kg-concertinas-lightened-ne-6792/</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -22913,16 +23267,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -23016,17 +23370,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
+          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Gradient</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-flying-on-the-s-7154/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -23035,19 +23389,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SM</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -23069,52 +23423,48 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Iota DLS 27 92-114kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platn Křídlo EN B</t>
+          <t>Křídlo EN B Skywalk Chili 5 95-115kg Nové Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115kg Nov</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-new-no-flying-on-the-sand-no-tr-7152/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2500</v>
+        <v>2100</v>
       </c>
       <c r="G3" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -23124,24 +23474,28 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk Tequila 5 85-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Tequila 5 85-</t>
+          <t>Křídlo EN A Skyman The Rock 2 29,5 105-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno TOP Křídlo E</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-tequila-5-85-105kg-no-sivs-no-flying-on-the-sand-7144/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/skyman-the-rock-2-295-105-130kg-concertinas-lightened-ne-6792/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2018</v>
+        <v>2025</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
@@ -23151,305 +23505,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skywalk Chili 5 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115k</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-no-sivs-no-flying-on-the-sand-n-7143/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Ozone Rush 5 L 95-115kg Listovaný TK platná S listovacím obalem Křídlo EN B Ozone Rush 5 L 95-115kg Listovan</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-95-115kg-concertinas-tc-valid-with-listin-7139/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN B SKY Paragliders Atis 2 M 75-95kg Žádné SIV TK není Nevětveno Nekoupáno Křídlo EN B SKY Paragliders Atis 2 M</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-atis-2-m-75-95kg-no-sivs-no-tc-no-trees--7135/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="n">
-        <v>2008</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ADVANCE Theta ULS 29</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-ThetaULS-29</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>3150</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Livi S</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
@@ -23464,20 +23520,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -23546,212 +23602,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>SM</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Iota DLS 27 92-114kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platn Křídlo EN B</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-iota-dls-27-92-114kg-concertinas-no-sivs-no-flyi-7145/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Livi S</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -23766,20 +23616,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -23851,210 +23701,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím obalem Křídlo EN B UP Kibo 2 SM 75-95kg TK platná S listovacím o</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-sm-75-95kg-tc-valid-with-listing-bag-7146/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>SM</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Ozone Rush 5 L 95-115kg Listovaný TK platná S listovacím obalem Křídlo EN B Ozone Rush 5 L 95-115kg Listovan</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-95-115kg-concertinas-tc-valid-with-listin-7139/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Prion 5 S 75-100kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Nova Prion 5 S 75-1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-s-75-100kg-new-no-sivs-no-flying-on-the-san-7142/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Livi S</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/Airdesign-Livi-S</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2750</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-17
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M360"/>
+  <dimension ref="A1:M369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19817,8 +19817,10 @@
         </is>
       </c>
       <c r="F358" t="inlineStr"/>
-      <c r="G358" t="n">
-        <v>2018</v>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H358" t="inlineStr">
         <is>
@@ -19869,11 +19871,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-new-no-flying-on-the-sand-no-tr-7152/</t>
         </is>
       </c>
-      <c r="F359" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G359" t="n">
-        <v>2021</v>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H359" t="inlineStr">
         <is>
@@ -19921,8 +19927,10 @@
         </is>
       </c>
       <c r="F360" t="inlineStr"/>
-      <c r="G360" t="n">
-        <v>2025</v>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H360" t="inlineStr">
         <is>
@@ -19944,6 +19952,481 @@
       <c r="M360" t="inlineStr">
         <is>
           <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 465,80 CZK (5</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>599</v>
+      </c>
+      <c r="G361" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr"/>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L361" t="inlineStr"/>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 904</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>700</v>
+      </c>
+      <c r="G362" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr"/>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L362" t="inlineStr"/>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 149,92 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G363" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr"/>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L363" t="inlineStr"/>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradi</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-sivs-no-flying-on-the-sa-7169/</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr"/>
+      <c r="G364" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr"/>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L364" t="inlineStr"/>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Denali xs 69-81kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient De</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-denali-xs-69-81kg-concertinas-no-sivs-no-flying-7167/</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr"/>
+      <c r="G365" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr"/>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L365" t="inlineStr"/>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné opravy Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné oprav</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-fides-2-24-no-tc-small-repairs-7157/</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr"/>
+      <c r="G366" t="n">
+        <v>2006</v>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr"/>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L366" t="inlineStr"/>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>899</v>
+      </c>
+      <c r="G367" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr"/>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L367" t="inlineStr"/>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 112,44 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>750</v>
+      </c>
+      <c r="G368" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr"/>
+      <c r="J368" t="inlineStr"/>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L368" t="inlineStr"/>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Soar 2 L</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-2-L/SW10916</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>2875</v>
+      </c>
+      <c r="G369" t="inlineStr"/>
+      <c r="H369" t="inlineStr"/>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr"/>
+      <c r="K369" t="inlineStr"/>
+      <c r="L369" t="inlineStr"/>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
@@ -19958,7 +20441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -23126,8 +23609,10 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="n">
-        <v>2018</v>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -23178,11 +23663,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-new-no-flying-on-the-sand-no-tr-7152/</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>2100</v>
-      </c>
-      <c r="G59" t="n">
-        <v>2021</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -23230,8 +23719,10 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="n">
-        <v>2025</v>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -23253,6 +23744,481 @@
       <c r="M60" t="inlineStr">
         <is>
           <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 465,80 CZK (5</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>599</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 904</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>700</v>
+      </c>
+      <c r="G62" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 149,92 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G63" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradi</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-sivs-no-flying-on-the-sa-7169/</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Denali xs 69-81kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient De</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-denali-xs-69-81kg-concertinas-no-sivs-no-flying-7167/</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné opravy Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné oprav</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-fides-2-24-no-tc-small-repairs-7157/</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="n">
+        <v>2006</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>899</v>
+      </c>
+      <c r="G67" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 112,44 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>750</v>
+      </c>
+      <c r="G68" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Soar 2 L</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-2-L/SW10916</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>2875</v>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
@@ -23267,16 +24233,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -23370,17 +24336,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Gradient</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 465,80 CZK (5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-flying-on-the-s-7154/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>599</v>
+      </c>
       <c r="G2" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -23389,19 +24357,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
@@ -23423,48 +24391,52 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skywalk Chili 5 95-115kg Nové Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Skywalk Chili 5 95-115kg Nov</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 904</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skywalk-chili-5-95-115kg-new-no-flying-on-the-sand-no-tr-7152/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2100</v>
+        <v>700</v>
       </c>
       <c r="G3" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -23474,26 +24446,28 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Skyman The Rock 2 29,5 105-130kg Listovaný Odlehčeno Nové Žádné SIV Nelétáno na písku Nevětveno TOP Křídlo E</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 149,92 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skyman-the-rock-2-295-105-130kg-concertinas-lightened-ne-6792/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
       <c r="G4" t="n">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -23505,7 +24479,317 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-sivs-no-flying-on-the-sa-7169/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2011</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Denali xs 69-81kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient De</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-denali-xs-69-81kg-concertinas-no-sivs-no-flying-7167/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>xs</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné opravy Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné oprav</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-fides-2-24-no-tc-small-repairs-7157/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2006</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>899</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 112,44 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>750</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Soar 2 L</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-2-L/SW10916</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>2875</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
@@ -23616,20 +24900,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -23701,6 +24985,61 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 149,92 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-22
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M369"/>
+  <dimension ref="A1:M380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -19981,11 +19981,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F361" t="n">
-        <v>599</v>
-      </c>
-      <c r="G361" t="n">
-        <v>2017</v>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H361" t="inlineStr">
         <is>
@@ -20036,11 +20040,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F362" t="n">
-        <v>700</v>
-      </c>
-      <c r="G362" t="n">
-        <v>2018</v>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H362" t="inlineStr">
         <is>
@@ -20091,11 +20099,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F363" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G363" t="n">
-        <v>2020</v>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H363" t="inlineStr">
         <is>
@@ -20147,8 +20159,10 @@
         </is>
       </c>
       <c r="F364" t="inlineStr"/>
-      <c r="G364" t="n">
-        <v>2011</v>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>2011.0</t>
+        </is>
       </c>
       <c r="H364" t="inlineStr">
         <is>
@@ -20200,8 +20214,10 @@
         </is>
       </c>
       <c r="F365" t="inlineStr"/>
-      <c r="G365" t="n">
-        <v>2015</v>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H365" t="inlineStr">
         <is>
@@ -20253,8 +20269,10 @@
         </is>
       </c>
       <c r="F366" t="inlineStr"/>
-      <c r="G366" t="n">
-        <v>2006</v>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>2006.0</t>
+        </is>
       </c>
       <c r="H366" t="inlineStr">
         <is>
@@ -20305,11 +20323,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
-      <c r="F367" t="n">
-        <v>899</v>
-      </c>
-      <c r="G367" t="n">
-        <v>2020</v>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H367" t="inlineStr">
         <is>
@@ -20360,11 +20382,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F368" t="n">
-        <v>750</v>
-      </c>
-      <c r="G368" t="n">
-        <v>2023</v>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H368" t="inlineStr">
         <is>
@@ -20411,8 +20437,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-2-L/SW10916</t>
         </is>
       </c>
-      <c r="F369" t="n">
-        <v>2875</v>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>2875.0</t>
+        </is>
       </c>
       <c r="G369" t="inlineStr"/>
       <c r="H369" t="inlineStr"/>
@@ -20427,6 +20455,583 @@
       <c r="M369" t="inlineStr">
         <is>
           <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN B Gradient</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7187/</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr"/>
+      <c r="G370" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr"/>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L370" t="inlineStr"/>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žád</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-7182/</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr"/>
+      <c r="G371" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr"/>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr"/>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Buzz Z6 ML 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Oz</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z6-ml-85-105kg-concertinas-no-sivs-no-flying--7181/</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr"/>
+      <c r="G372" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr"/>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L372" t="inlineStr"/>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno TK platná (Součást kompletu) Křídl</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7172/</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>660</v>
+      </c>
+      <c r="G373" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr"/>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr"/>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-7171/</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr"/>
+      <c r="G374" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr"/>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L374" t="inlineStr"/>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B Gradient Golden 5 28 95-11</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-trees-no-water--7154/</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr"/>
+      <c r="G375" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr"/>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L375" t="inlineStr"/>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY AYA-XL 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A SKY AY</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-105-130kg-concertinas-no-sivs-no-flying-on-th-7191/</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr"/>
+      <c r="G376" t="inlineStr"/>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr"/>
+      <c r="J376" t="inlineStr"/>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr"/>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>899</v>
+      </c>
+      <c r="G377" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr"/>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr"/>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G378" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr"/>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr"/>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 29 87-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G379" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr"/>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr"/>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi M</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>3075</v>
+      </c>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr"/>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr"/>
+      <c r="K380" t="inlineStr"/>
+      <c r="L380" t="inlineStr"/>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -20441,7 +21046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -23773,11 +24378,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>599</v>
-      </c>
-      <c r="G61" t="n">
-        <v>2017</v>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2017.0</t>
+        </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -23828,11 +24437,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>700</v>
-      </c>
-      <c r="G62" t="n">
-        <v>2018</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -23883,11 +24496,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F63" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G63" t="n">
-        <v>2020</v>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -23939,8 +24556,10 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="n">
-        <v>2011</v>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2011.0</t>
+        </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -23992,8 +24611,10 @@
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="n">
-        <v>2015</v>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -24045,8 +24666,10 @@
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
-      <c r="G66" t="n">
-        <v>2006</v>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2006.0</t>
+        </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -24097,11 +24720,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>899</v>
-      </c>
-      <c r="G67" t="n">
-        <v>2020</v>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -24152,11 +24779,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>750</v>
-      </c>
-      <c r="G68" t="n">
-        <v>2023</v>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -24203,8 +24834,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-2-L/SW10916</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>2875</v>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2875.0</t>
+        </is>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
@@ -24219,6 +24852,583 @@
       <c r="M69" t="inlineStr">
         <is>
           <t>2026-06-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN B Gradient</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7187/</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žád</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-7182/</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Buzz Z6 ML 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Oz</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z6-ml-85-105kg-concertinas-no-sivs-no-flying--7181/</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno TK platná (Součást kompletu) Křídl</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7172/</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>660</v>
+      </c>
+      <c r="G73" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-7171/</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B Gradient Golden 5 28 95-11</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-trees-no-water--7154/</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY AYA-XL 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A SKY AY</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-105-130kg-concertinas-no-sivs-no-flying-on-th-7191/</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>899</v>
+      </c>
+      <c r="G77" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G78" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 29 87-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G79" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi M</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>3075</v>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24233,7 +25443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -24336,19 +25546,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 465,80 CZK (5</t>
+          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN B Gradient</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>599</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7187/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -24357,7 +25565,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -24369,7 +25577,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24391,19 +25599,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 904</t>
+          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žád</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-7182/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -24424,7 +25630,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24446,19 +25652,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 149,92 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Ozone Buzz Z6 ML 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Oz</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1000</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z6-ml-85-105kg-concertinas-no-sivs-no-flying--7181/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -24467,31 +25671,31 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -24501,50 +25705,52 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Orbit 3 28 95-115kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN A Gradi</t>
+          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno TK platná (Součást kompletu) Křídl</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-orbit-3-28-95-115kg-no-sivs-no-flying-on-the-sa-7169/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7172/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>660</v>
+      </c>
       <c r="G5" t="n">
-        <v>2011</v>
+        <v>2016</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -24554,50 +25760,50 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Denali xs 69-81kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A Gradient De</t>
+          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-denali-xs-69-81kg-concertinas-no-sivs-no-flying-7167/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-7171/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>2015</v>
+        <v>2024</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>xs</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -24607,38 +25813,38 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné opravy Křídlo EN A SKY Paragliders Fides 2 24 TK není Drobné oprav</t>
+          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B Gradient Golden 5 28 95-11</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-fides-2-24-no-tc-small-repairs-7157/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-trees-no-water--7154/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>2006</v>
+        <v>2018</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24660,40 +25866,32 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
+          <t>Křídlo EN A SKY AYA-XL 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A SKY AY</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7078/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>899</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2020</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-105-130kg-concertinas-no-sivs-no-flying-on-th-7191/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24715,81 +25913,195 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 112,44 CZK (750,00 EUR) E</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>750</v>
+        <v>899</v>
       </c>
       <c r="G9" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hochries_de</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>AIRDESIGN Soar 2 L</t>
+          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Soar-2-L/SW10916</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2875</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+        <v>1600</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 29 87-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi M</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>3075</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24804,20 +26116,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -24886,6 +26198,320 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žád</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-7182/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Buzz Z6 ML 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Oz</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z6-ml-85-105kg-concertinas-no-sivs-no-flying--7181/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-7171/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 29 87-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Livi M</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3075</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -24900,7 +26526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -24913,7 +26539,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -25003,17 +26629,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 149,92 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN B Gradient</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7187/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>2020</v>
       </c>
@@ -25024,19 +26648,74 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-23
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M380"/>
+  <dimension ref="A1:M386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -20485,8 +20485,10 @@
         </is>
       </c>
       <c r="F370" t="inlineStr"/>
-      <c r="G370" t="n">
-        <v>2020</v>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H370" t="inlineStr">
         <is>
@@ -20538,8 +20540,10 @@
         </is>
       </c>
       <c r="F371" t="inlineStr"/>
-      <c r="G371" t="n">
-        <v>2022</v>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H371" t="inlineStr">
         <is>
@@ -20591,8 +20595,10 @@
         </is>
       </c>
       <c r="F372" t="inlineStr"/>
-      <c r="G372" t="n">
-        <v>2023</v>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H372" t="inlineStr">
         <is>
@@ -20643,11 +20649,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7172/</t>
         </is>
       </c>
-      <c r="F373" t="n">
-        <v>660</v>
-      </c>
-      <c r="G373" t="n">
-        <v>2016</v>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>660.0</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H373" t="inlineStr">
         <is>
@@ -20699,8 +20709,10 @@
         </is>
       </c>
       <c r="F374" t="inlineStr"/>
-      <c r="G374" t="n">
-        <v>2024</v>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H374" t="inlineStr">
         <is>
@@ -20752,8 +20764,10 @@
         </is>
       </c>
       <c r="F375" t="inlineStr"/>
-      <c r="G375" t="n">
-        <v>2018</v>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
@@ -20851,11 +20865,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
-      <c r="F377" t="n">
-        <v>899</v>
-      </c>
-      <c r="G377" t="n">
-        <v>2020</v>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H377" t="inlineStr">
         <is>
@@ -20906,11 +20924,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
         </is>
       </c>
-      <c r="F378" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G378" t="n">
-        <v>2024</v>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H378" t="inlineStr">
         <is>
@@ -20961,11 +20983,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
         </is>
       </c>
-      <c r="F379" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G379" t="n">
-        <v>2022</v>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H379" t="inlineStr">
         <is>
@@ -21016,8 +21042,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
         </is>
       </c>
-      <c r="F380" t="n">
-        <v>3075</v>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>3075.0</t>
+        </is>
       </c>
       <c r="G380" t="inlineStr"/>
       <c r="H380" t="inlineStr"/>
@@ -21032,6 +21060,324 @@
       <c r="M380" t="inlineStr">
         <is>
           <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr"/>
+      <c r="G381" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr"/>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr"/>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Nevada 110-130kg Listovaný TK není Nevětveno Drobné opravy Křídlo EN B Gradient Nevada 110-130kg Li</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-110-130kg-concertinas-no-tc-no-trees-sma-7196/</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr"/>
+      <c r="G382" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr"/>
+      <c r="J382" t="inlineStr"/>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr"/>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 224,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G383" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr"/>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr"/>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 778,10 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>899</v>
+      </c>
+      <c r="G384" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr"/>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr"/>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 168,60 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>750</v>
+      </c>
+      <c r="G385" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr"/>
+      <c r="J385" t="inlineStr"/>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr"/>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Advance Theta 25 Kommissionsverkauf</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G386" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H386" t="inlineStr"/>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>78kg-99kg</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr"/>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -21046,7 +21392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -24882,8 +25228,10 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="n">
-        <v>2020</v>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -24935,8 +25283,10 @@
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="n">
-        <v>2022</v>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -24988,8 +25338,10 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="n">
-        <v>2023</v>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -25040,11 +25392,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7172/</t>
         </is>
       </c>
-      <c r="F73" t="n">
-        <v>660</v>
-      </c>
-      <c r="G73" t="n">
-        <v>2016</v>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>660.0</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -25096,8 +25452,10 @@
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="n">
-        <v>2024</v>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -25149,8 +25507,10 @@
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="n">
-        <v>2018</v>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -25248,11 +25608,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>899</v>
-      </c>
-      <c r="G77" t="n">
-        <v>2020</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -25303,11 +25667,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
         </is>
       </c>
-      <c r="F78" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G78" t="n">
-        <v>2024</v>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -25358,11 +25726,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G79" t="n">
-        <v>2022</v>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>1300.0</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -25413,8 +25785,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>3075</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>3075.0</t>
+        </is>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -25429,6 +25803,324 @@
       <c r="M80" t="inlineStr">
         <is>
           <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Nevada 110-130kg Listovaný TK není Nevětveno Drobné opravy Křídlo EN B Gradient Nevada 110-130kg Li</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-110-130kg-concertinas-no-tc-no-trees-sma-7196/</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 224,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G83" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 778,10 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>899</v>
+      </c>
+      <c r="G84" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 168,60 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>750</v>
+      </c>
+      <c r="G85" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Advance Theta 25 Kommissionsverkauf</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G86" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>78kg-99kg</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -25443,20 +26135,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -25546,17 +26238,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN B Gradient</t>
+          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7187/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -25565,7 +26257,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -25577,7 +26269,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -25599,38 +26291,34 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žád</t>
+          <t>Křídlo EN B Gradient Nevada 110-130kg Listovaný TK není Nevětveno Drobné opravy Křídlo EN B Gradient Nevada 110-130kg Li</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-7182/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-110-130kg-concertinas-no-tc-no-trees-sma-7196/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -25652,17 +26340,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Ozone Buzz Z6 ML 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Oz</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 224,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z6-ml-85-105kg-concertinas-no-sivs-no-flying--7181/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1000</v>
+      </c>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -25671,31 +26361,31 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -25705,52 +26395,52 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Anakis 2 L-88kg 110 Žádné SIV Nelétáno na písku Nevětveno TK platná (Součást kompletu) Křídl</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 778,10 CZK (899,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-2-l-88kg-110-no-sivs-no-flying-on-7172/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>660</v>
+        <v>899</v>
       </c>
       <c r="G5" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -25760,348 +26450,91 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 168,60 CZK (750,00 EUR) E</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-7171/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>750</v>
+      </c>
       <c r="G6" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_store_at</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Store AT – Used</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 5 28 95-115kg Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B Gradient Golden 5 28 95-11</t>
+          <t>Advance Theta 25 Kommissionsverkauf</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-28-95-115kg-no-sivs-no-trees-no-water--7154/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2690</v>
+      </c>
       <c r="G7" t="n">
-        <v>2018</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>2025</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>78kg-99kg</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SKY AYA-XL 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A SKY AY</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-aya-xl-105-130kg-concertinas-no-sivs-no-flying-on-th-7191/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 710,78 CZK (899,00 EUR) EN A Velikost</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>899</v>
-      </c>
-      <c r="G9" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Muse 5 29 87-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC M</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Livi M</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>3075</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -26111,416 +26544,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žádné SIV TK čerstvá Křídlo EN B GIN Explorer 2 M 85-105kg Listovaný Žád</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-explorer-2-m-85-105kg-concertinas-no-sivs-tc-fresh-7182/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Ozone Buzz Z6 ML 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Oz</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z6-ml-85-105kg-concertinas-no-sivs-no-flying--7181/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Illusion 28 90-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B MAC</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-90-110kg-concertinas-no-sivs-no-flying-o-7171/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Muse 5 29 87-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A MAC M</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-87-110kg-concertinas-no-sivs-no-flying-on--7170/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Livi M</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Livi-M/SW10917</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>3075</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26539,7 +26562,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -26629,17 +26652,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK platná Křídlo EN B Gradient</t>
+          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7187/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -26648,7 +26671,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -26660,50 +26683,254 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_store_at</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Store AT – Used</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A MAC Muse 5 25 70-90kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A MAC M</t>
+          <t>Advance Theta 25 Kommissionsverkauf</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-25-70-90kg-concertinas-no-sivs-no-flying-on-t-7178/</t>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1600</v>
+        <v>2690</v>
       </c>
       <c r="G3" t="n">
-        <v>2024</v>
+        <v>2025</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>78kg-99kg</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 224,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -26715,7 +26942,62 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Advance Theta 25 Kommissionsverkauf</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>78kg-99kg</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-24
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M386"/>
+  <dimension ref="A1:M393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21090,8 +21090,10 @@
         </is>
       </c>
       <c r="F381" t="inlineStr"/>
-      <c r="G381" t="n">
-        <v>2022</v>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H381" t="inlineStr">
         <is>
@@ -21143,8 +21145,10 @@
         </is>
       </c>
       <c r="F382" t="inlineStr"/>
-      <c r="G382" t="n">
-        <v>2016</v>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H382" t="inlineStr">
         <is>
@@ -21191,11 +21195,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F383" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G383" t="n">
-        <v>2020</v>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H383" t="inlineStr">
         <is>
@@ -21246,11 +21254,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
-      <c r="F384" t="n">
-        <v>899</v>
-      </c>
-      <c r="G384" t="n">
-        <v>2020</v>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H384" t="inlineStr">
         <is>
@@ -21301,11 +21313,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F385" t="n">
-        <v>750</v>
-      </c>
-      <c r="G385" t="n">
-        <v>2023</v>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H385" t="inlineStr">
         <is>
@@ -21352,11 +21368,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F386" t="n">
-        <v>2690</v>
-      </c>
-      <c r="G386" t="n">
-        <v>2025</v>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>2690.0</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H386" t="inlineStr"/>
       <c r="I386" t="inlineStr">
@@ -21378,6 +21398,381 @@
       <c r="M386" t="inlineStr">
         <is>
           <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 492,75 CZK (5</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>599</v>
+      </c>
+      <c r="G387" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr"/>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr"/>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 936</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>700</v>
+      </c>
+      <c r="G388" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr"/>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr"/>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 204,87 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G389" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr"/>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr"/>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 85-125kg Křídlo EN A Advance Alpha 6 85-125kg 22 000,00 CZK EN A Vzletová hmotnost: 85 - 125</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-85-125kg-7212/</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr"/>
+      <c r="G390" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr"/>
+      <c r="J390" t="inlineStr"/>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr"/>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 16 936,44 CZK (700,00 EUR) EN A Velikost: m Vzle</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>700</v>
+      </c>
+      <c r="G391" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr"/>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr"/>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 760,18 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>899</v>
+      </c>
+      <c r="G392" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr"/>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr"/>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 153,65 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>750</v>
+      </c>
+      <c r="G393" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr"/>
+      <c r="J393" t="inlineStr"/>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr"/>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -21392,7 +21787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -25833,8 +26228,10 @@
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
-      <c r="G81" t="n">
-        <v>2022</v>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -25886,8 +26283,10 @@
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
-      <c r="G82" t="n">
-        <v>2016</v>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -25934,11 +26333,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F83" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G83" t="n">
-        <v>2020</v>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -25989,11 +26392,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
-      <c r="F84" t="n">
-        <v>899</v>
-      </c>
-      <c r="G84" t="n">
-        <v>2020</v>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -26044,11 +26451,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F85" t="n">
-        <v>750</v>
-      </c>
-      <c r="G85" t="n">
-        <v>2023</v>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -26095,11 +26506,15 @@
           <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
         </is>
       </c>
-      <c r="F86" t="n">
-        <v>2690</v>
-      </c>
-      <c r="G86" t="n">
-        <v>2025</v>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2690.0</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
@@ -26121,6 +26536,381 @@
       <c r="M86" t="inlineStr">
         <is>
           <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 492,75 CZK (5</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>599</v>
+      </c>
+      <c r="G87" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 936</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>700</v>
+      </c>
+      <c r="G88" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 204,87 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G89" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 85-125kg Křídlo EN A Advance Alpha 6 85-125kg 22 000,00 CZK EN A Vzletová hmotnost: 85 - 125</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-85-125kg-7212/</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 16 936,44 CZK (700,00 EUR) EN A Velikost: m Vzle</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>700</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 760,18 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>899</v>
+      </c>
+      <c r="G92" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 153,65 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>750</v>
+      </c>
+      <c r="G93" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -26135,7 +26925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -26148,7 +26938,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -26238,17 +27028,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 492,75 CZK (5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>599</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -26257,7 +27049,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -26269,7 +27061,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -26291,34 +27083,40 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Nevada 110-130kg Listovaný TK není Nevětveno Drobné opravy Křídlo EN B Gradient Nevada 110-130kg Li</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 936</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-nevada-110-130kg-concertinas-no-tc-no-trees-sma-7196/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>700</v>
+      </c>
       <c r="G3" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -26340,7 +27138,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 224,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 204,87 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -26373,7 +27171,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -26395,17 +27193,15 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 778,10 CZK (899,00 EUR) EN A Velikost</t>
+          <t>Křídlo EN A Advance Alpha 6 85-125kg Křídlo EN A Advance Alpha 6 85-125kg 22 000,00 CZK EN A Vzletová hmotnost: 85 - 125</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>899</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-85-125kg-7212/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>2020</v>
       </c>
@@ -26414,21 +27210,17 @@
           <t>EN A</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -26450,91 +27242,146 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 168,60 CZK (750,00 EUR) E</t>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 16 936,44 CZK (700,00 EUR) EN A Velikost: m Vzle</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="G6" t="n">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Olétané (více než 300h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>paragliding_store_at</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paragliding Store AT – Used</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Advance Theta 25 Kommissionsverkauf</t>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 760,18 CZK (899,00 EUR) EN A Velikost</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2690</v>
+        <v>899</v>
       </c>
       <c r="G7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
+        <v>2020</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>78kg-99kg</t>
-        </is>
-      </c>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 153,65 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>750</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
@@ -26544,6 +27391,102 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26562,7 +27505,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -26652,17 +27595,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 204,87 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -26671,333 +27616,68 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_store_at</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Store AT – Used</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Advance Theta 25 Kommissionsverkauf</t>
+          <t>Křídlo EN A Advance Alpha 6 85-125kg Křídlo EN A Advance Alpha 6 85-125kg 22 000,00 CZK EN A Vzletová hmotnost: 85 - 125</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>2690</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-85-125kg-7212/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>78kg-99kg</t>
-        </is>
-      </c>
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Illusion 28 85-110kg Listovaný TK čerstvá TK platná S batohem S listovacím obalem Křídlo EN B MAC Illusi</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-28-85-110kg-concertinas-tc-fresh-tc-valid-w-7201/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 224,81 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Advance Theta 25 Kommissionsverkauf</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>2690</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>78kg-99kg</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>sehr guter Zustand  --&gt; 75h  --&gt; siehe n</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-25
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M393"/>
+  <dimension ref="A1:M397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21427,11 +21427,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F387" t="n">
-        <v>599</v>
-      </c>
-      <c r="G387" t="n">
-        <v>2017</v>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H387" t="inlineStr">
         <is>
@@ -21482,11 +21486,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F388" t="n">
-        <v>700</v>
-      </c>
-      <c r="G388" t="n">
-        <v>2018</v>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H388" t="inlineStr">
         <is>
@@ -21537,11 +21545,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F389" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G389" t="n">
-        <v>2020</v>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H389" t="inlineStr">
         <is>
@@ -21593,8 +21605,10 @@
         </is>
       </c>
       <c r="F390" t="inlineStr"/>
-      <c r="G390" t="n">
-        <v>2020</v>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H390" t="inlineStr">
         <is>
@@ -21641,11 +21655,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
         </is>
       </c>
-      <c r="F391" t="n">
-        <v>700</v>
-      </c>
-      <c r="G391" t="n">
-        <v>2015</v>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H391" t="inlineStr">
         <is>
@@ -21696,11 +21714,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
-      <c r="F392" t="n">
-        <v>899</v>
-      </c>
-      <c r="G392" t="n">
-        <v>2020</v>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H392" t="inlineStr">
         <is>
@@ -21751,11 +21773,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F393" t="n">
-        <v>750</v>
-      </c>
-      <c r="G393" t="n">
-        <v>2023</v>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H393" t="inlineStr">
         <is>
@@ -21773,6 +21799,222 @@
       <c r="M393" t="inlineStr">
         <is>
           <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 XL 95-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SK</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-xl-95-130kg-concertinas-no-sivs--7214/</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr"/>
+      <c r="G394" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr"/>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr"/>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 498,72 CZK (5</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>599</v>
+      </c>
+      <c r="G395" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr"/>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr"/>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 943</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>700</v>
+      </c>
+      <c r="G396" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr"/>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr"/>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 17 000,00 CZK EN A Velikost: m Vzletová hmotnost</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr"/>
+      <c r="G397" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr"/>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr"/>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -21787,7 +22029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M93"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -26565,11 +26807,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F87" t="n">
-        <v>599</v>
-      </c>
-      <c r="G87" t="n">
-        <v>2017</v>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -26620,11 +26866,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>700</v>
-      </c>
-      <c r="G88" t="n">
-        <v>2018</v>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -26675,11 +26925,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
         </is>
       </c>
-      <c r="F89" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G89" t="n">
-        <v>2020</v>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -26731,8 +26985,10 @@
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" t="n">
-        <v>2020</v>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -26779,11 +27035,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>700</v>
-      </c>
-      <c r="G91" t="n">
-        <v>2015</v>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -26834,11 +27094,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>899</v>
-      </c>
-      <c r="G92" t="n">
-        <v>2020</v>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>899.0</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -26889,11 +27153,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>750</v>
-      </c>
-      <c r="G93" t="n">
-        <v>2023</v>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>750.0</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -26911,6 +27179,222 @@
       <c r="M93" t="inlineStr">
         <is>
           <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 XL 95-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SK</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-xl-95-130kg-concertinas-no-sivs--7214/</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 498,72 CZK (5</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>599</v>
+      </c>
+      <c r="G95" t="n">
+        <v>2017</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 943</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>700</v>
+      </c>
+      <c r="G96" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 17 000,00 CZK EN A Velikost: m Vzletová hmotnost</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -26925,7 +27409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -27028,19 +27512,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 492,75 CZK (5</t>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 XL 95-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>599</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-xl-95-130kg-concertinas-no-sivs--7214/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -27049,19 +27531,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -27083,19 +27565,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 936</t>
+          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 498,72 CZK (5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>700</v>
+        <v>599</v>
       </c>
       <c r="G3" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -27104,7 +27586,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -27116,7 +27598,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -27138,19 +27620,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 204,87 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 943</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="G4" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -27165,13 +27647,13 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -27193,195 +27675,38 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 85-125kg Křídlo EN A Advance Alpha 6 85-125kg 22 000,00 CZK EN A Vzletová hmotnost: 85 - 125</t>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 17 000,00 CZK EN A Velikost: m Vzletová hmotnost</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-85-125kg-7212/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Olétané (více než 300h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 16 936,44 CZK (700,00 EUR) EN A Velikost: m Vzle</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>700</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Olétané (více než 300h)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 760,18 CZK (899,00 EUR) EN A Velikost</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>899</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 153,65 CZK (750,00 EUR) E</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>750</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -27492,20 +27817,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -27577,110 +27902,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 204,87 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 85-125kg Křídlo EN A Advance Alpha 6 85-125kg 22 000,00 CZK EN A Vzletová hmotnost: 85 - 125</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-85-125kg-7212/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-06-26
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M397"/>
+  <dimension ref="A1:M403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -21829,8 +21829,10 @@
         </is>
       </c>
       <c r="F394" t="inlineStr"/>
-      <c r="G394" t="n">
-        <v>2022</v>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H394" t="inlineStr">
         <is>
@@ -21881,11 +21883,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F395" t="n">
-        <v>599</v>
-      </c>
-      <c r="G395" t="n">
-        <v>2017</v>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H395" t="inlineStr">
         <is>
@@ -21936,11 +21942,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F396" t="n">
-        <v>700</v>
-      </c>
-      <c r="G396" t="n">
-        <v>2018</v>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H396" t="inlineStr">
         <is>
@@ -21992,8 +22002,10 @@
         </is>
       </c>
       <c r="F397" t="inlineStr"/>
-      <c r="G397" t="n">
-        <v>2015</v>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H397" t="inlineStr">
         <is>
@@ -22015,6 +22027,332 @@
       <c r="M397" t="inlineStr">
         <is>
           <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis M 75-95kg TK není Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-m-75-95kg-no-tc-no-flying-on-the--7215/</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>152</v>
+      </c>
+      <c r="G398" t="n">
+        <v>2009</v>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr"/>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr"/>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 17 000,00 CZK (700,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>700</v>
+      </c>
+      <c r="G399" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr"/>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr"/>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 968</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>700</v>
+      </c>
+      <c r="G400" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr"/>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr"/>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 260,07 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G401" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr"/>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr"/>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 809,80 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>899</v>
+      </c>
+      <c r="G402" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr"/>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr"/>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 195,05 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>750</v>
+      </c>
+      <c r="G403" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr"/>
+      <c r="J403" t="inlineStr"/>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr"/>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -22029,7 +22367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M97"/>
+  <dimension ref="A1:M103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -27209,8 +27547,10 @@
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
-      <c r="G94" t="n">
-        <v>2022</v>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -27261,11 +27601,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>599</v>
-      </c>
-      <c r="G95" t="n">
-        <v>2017</v>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>599.0</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -27316,11 +27660,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
         </is>
       </c>
-      <c r="F96" t="n">
-        <v>700</v>
-      </c>
-      <c r="G96" t="n">
-        <v>2018</v>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>700.0</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -27372,8 +27720,10 @@
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
-      <c r="G97" t="n">
-        <v>2015</v>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -27395,6 +27745,332 @@
       <c r="M97" t="inlineStr">
         <is>
           <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Anakis M 75-95kg TK není Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-m-75-95kg-no-tc-no-flying-on-the--7215/</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>152</v>
+      </c>
+      <c r="G98" t="n">
+        <v>2009</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 17 000,00 CZK (700,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>700</v>
+      </c>
+      <c r="G99" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 968</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-5-m-90-110kg-concertinas-no-trees-6860/</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>700</v>
+      </c>
+      <c r="G100" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 260,07 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G101" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 809,80 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>899</v>
+      </c>
+      <c r="G102" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 195,05 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>750</v>
+      </c>
+      <c r="G103" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -27409,7 +28085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -27422,7 +28098,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -27512,17 +28188,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 XL 95-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SK</t>
+          <t>Křídlo EN B SKY Paragliders Anakis M 75-95kg TK není Nelétáno na písku Nevětveno Nekoupáno Drobné opravy Křídlo EN B SKY</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-xl-95-130kg-concertinas-no-sivs--7214/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-anakis-m-75-95kg-no-tc-no-flying-on-the--7215/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>152</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2009</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -27531,19 +28209,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -27565,19 +28243,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá Křídlo EN B Advance epsilon 8 23 55-85kg TK čerstvá 14 498,72 CZK (5</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 17 000,00 CZK (700,00 EUR) EN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-8-23-55-85kg-tc-fresh-6981/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>599</v>
+        <v>700</v>
       </c>
       <c r="G3" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -27586,19 +28264,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -27620,7 +28298,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 943</t>
+          <t>Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno Křídlo EN B Nova Mentor 5 M 90-110kg Listovaný Nevětveno 16 968</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -27653,19 +28331,19 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -27675,38 +28353,146 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Křídlo EN A GIN Bolero 5 m 85-105kg 17 000,00 CZK EN A Velikost: m Vzletová hmotnost</t>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 260,07 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-7211/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1000</v>
+      </c>
       <c r="G5" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Olétané (více než 300h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Advance Alpha 6 28 85-125kg Křídlo EN A Advance Alpha 6 28 85-125kg 21 809,80 CZK (899,00 EUR) EN A Velikost</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-28-85-125kg-7179/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>899</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný Křídlo EN A Niviuk Koyot 5 90-115kg Listovaný 18 195,05 CZK (750,00 EUR) E</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/niviuk-koyot-5-90-115kg-concertinas-6886/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>750</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -27817,20 +28603,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -27902,6 +28688,116 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná TOP Křídlo EN B 777 Rook 3 S 70-85kg TK platná 17 000,00 CZK (700,00 EUR) EN</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7032/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>700</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Křídlo EN B AXIS Comet 3 M 24 260,07 CZK (1 000,00 EUR) EN B Velikost: M Opotřebení: Jako nov</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-6785/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+  